<commit_message>
Updates to GitHub workflows
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{129E3F12-0442-4857-B401-69AABB57E7A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F86AC4-0747-45C1-8F70-9FAD7149DCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$K$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$K$100</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="176">
   <si>
     <t>Item</t>
   </si>
@@ -523,9 +522,6 @@
     <t>Body Text alignment not implemented in frontend</t>
   </si>
   <si>
-    <t>Provide ability to set column names and use them as header</t>
-  </si>
-  <si>
     <t>Maintenance: Log or delete post blocks without matching table</t>
   </si>
   <si>
@@ -548,6 +544,30 @@
   </si>
   <si>
     <t>Allow a TAB on the bottom right cell to insert a new row</t>
+  </si>
+  <si>
+    <t>Add Date/Time column data type</t>
+  </si>
+  <si>
+    <t>Allow for column names to be changed/updated</t>
+  </si>
+  <si>
+    <t>Changing a date format causes error when editing existing value of different format</t>
+  </si>
+  <si>
+    <t>Arrow navigation doesn't always work on arrow key nav from edit mode</t>
+  </si>
+  <si>
+    <t>Allow date/time to be edited by input as well as button</t>
+  </si>
+  <si>
+    <t>Create navigation layer separate from editing</t>
+  </si>
+  <si>
+    <t>Provide use column names as header</t>
+  </si>
+  <si>
+    <t>Created Cell component</t>
   </si>
 </sst>
 </file>
@@ -657,10 +677,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2771,7 +2787,7 @@
         <v>87</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>17</v>
@@ -2790,15 +2806,15 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>82</v>
+        <v>131</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>56</v>
@@ -2807,65 +2823,57 @@
         <v>6</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="G66" s="5">
         <v>1.2</v>
       </c>
-      <c r="I66" s="4">
-        <v>99</v>
-      </c>
       <c r="J66" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="K66" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>31</v>
+        <v>133</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G67" s="5">
         <v>1.2</v>
       </c>
-      <c r="I67" s="4">
-        <v>99</v>
-      </c>
+      <c r="I67" s="5"/>
       <c r="J67" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>37</v>
+        <v>168</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F68" s="4" t="s">
         <v>11</v>
@@ -2873,138 +2881,129 @@
       <c r="G68" s="5">
         <v>1.2</v>
       </c>
-      <c r="I68" s="4">
-        <v>99</v>
-      </c>
+      <c r="I68" s="5"/>
       <c r="J68" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
-        <v>43</v>
+        <v>94</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>39</v>
+        <v>169</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G69" s="5">
         <v>1.2</v>
       </c>
-      <c r="I69" s="4">
-        <v>99</v>
-      </c>
+      <c r="I69" s="5"/>
       <c r="J69" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>29</v>
+        <v>173</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F70" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G70" s="5">
         <v>1.2</v>
       </c>
-      <c r="I70" s="4">
-        <v>99</v>
-      </c>
+      <c r="I70" s="5"/>
       <c r="J70" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="K70" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>41</v>
+        <v>170</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>7</v>
       </c>
       <c r="G71" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="I71" s="4">
-        <v>99</v>
+        <v>1.3</v>
+      </c>
+      <c r="I71" s="5">
+        <v>1</v>
       </c>
       <c r="J71" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>80</v>
+        <v>171</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>18</v>
+        <v>40</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G72" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="I72" s="4">
-        <v>99</v>
+        <v>1.3</v>
+      </c>
+      <c r="I72" s="5">
+        <v>2</v>
       </c>
       <c r="J72" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>56</v>
@@ -3013,71 +3012,71 @@
         <v>6</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G73" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="I73" s="4">
-        <v>99</v>
+        <v>1.3</v>
+      </c>
+      <c r="I73" s="5">
+        <v>3</v>
       </c>
       <c r="J73" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>139</v>
+        <v>17</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G74" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="I74" s="4">
-        <v>99</v>
+        <v>1.3</v>
+      </c>
+      <c r="I74" s="5">
+        <v>4</v>
       </c>
       <c r="J74" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G75" s="5">
-        <v>1.2</v>
-      </c>
-      <c r="I75" s="4">
-        <v>99</v>
+        <v>1.3</v>
+      </c>
+      <c r="I75" s="5">
+        <v>5</v>
       </c>
       <c r="J75" s="4" t="s">
         <v>27</v>
@@ -3085,16 +3084,16 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>151</v>
+        <v>82</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>152</v>
+        <v>56</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>6</v>
@@ -3103,7 +3102,7 @@
         <v>11</v>
       </c>
       <c r="G76" s="5">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="I76" s="4">
         <v>99</v>
@@ -3112,30 +3111,30 @@
         <v>27</v>
       </c>
       <c r="K76" s="4" t="s">
-        <v>158</v>
+        <v>93</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>155</v>
+        <v>30</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G77" s="5">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="I77" s="4">
         <v>99</v>
@@ -3146,25 +3145,25 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>161</v>
+        <v>37</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>133</v>
+        <v>31</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G78" s="5">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="I78" s="4">
         <v>99</v>
@@ -3175,183 +3174,216 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>137</v>
+        <v>39</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>133</v>
+        <v>31</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G79" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="I79" s="5">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G79" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I79" s="4">
+        <v>99</v>
       </c>
       <c r="J79" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>138</v>
+        <v>29</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>133</v>
+        <v>21</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G80" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="I80" s="5">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G80" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I80" s="4">
+        <v>99</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="K80" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>167</v>
+        <v>41</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G81" s="5" t="s">
-        <v>166</v>
+        <v>11</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G81" s="5">
+        <v>1.3</v>
       </c>
       <c r="I81" s="4">
-        <v>3</v>
+        <v>99</v>
       </c>
       <c r="J81" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>168</v>
+        <v>80</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="E82" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F82" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G82" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="I82" s="5">
-        <v>4</v>
+      <c r="G82" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I82" s="4">
+        <v>99</v>
       </c>
       <c r="J82" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>17</v>
+        <v>139</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G83" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="I83" s="5"/>
+        <v>6</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G83" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I83" s="4">
+        <v>99</v>
+      </c>
       <c r="J83" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>17</v>
+        <v>88</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G84" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="I84" s="5"/>
+        <v>6</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G84" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I84" s="4">
+        <v>99</v>
+      </c>
       <c r="J84" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G85" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="I85" s="5"/>
+        <v>6</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G85" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I85" s="4">
+        <v>99</v>
+      </c>
       <c r="J85" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="K85" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>17</v>
@@ -3360,22 +3392,27 @@
         <v>133</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G86" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="I86" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G86" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="I86" s="4">
+        <v>99</v>
+      </c>
       <c r="J86" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>17</v>
@@ -3387,100 +3424,101 @@
         <v>25</v>
       </c>
       <c r="G87" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="H87" s="5" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="I87" s="5"/>
       <c r="J87" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G88" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="I88" s="5"/>
+        <v>165</v>
+      </c>
       <c r="J88" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G89" s="5" t="s">
-        <v>134</v>
+        <v>165</v>
       </c>
       <c r="I89" s="5"/>
       <c r="J89" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="E90" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="F90" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="G90" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="I90" s="5"/>
+      <c r="I90" s="4">
+        <v>99</v>
+      </c>
       <c r="J90" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>156</v>
+        <v>87</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="E91" s="4" t="s">
         <v>25</v>
@@ -3493,18 +3531,15 @@
         <v>134</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="D92" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="E92" s="4" t="s">
         <v>25</v>
@@ -3517,48 +3552,45 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G93" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="H93" s="5">
-        <v>98</v>
       </c>
       <c r="I93" s="5"/>
       <c r="J93" s="4" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G94" s="5" t="s">
         <v>134</v>
@@ -3568,70 +3600,207 @@
         <v>134</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G95" s="5"/>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A95" s="4">
+        <v>77</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H95" s="5" t="s">
+        <v>149</v>
+      </c>
       <c r="I95" s="5"/>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G96" s="5"/>
+      <c r="J95" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>79</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="I96" s="5"/>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G97" s="5"/>
+      <c r="J96" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>80</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G97" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="I97" s="5"/>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G98" s="5"/>
+      <c r="J97" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>84</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="I98" s="5"/>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G99" s="5"/>
+      <c r="J98" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A99" s="4">
+        <v>86</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G99" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="I99" s="5"/>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G100" s="5"/>
+      <c r="J99" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A100" s="4">
+        <v>89</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H100" s="5">
+        <v>98</v>
+      </c>
       <c r="I100" s="5"/>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J100" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="K100" s="4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G101" s="5"/>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G102" s="5"/>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G103" s="5"/>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G104" s="5"/>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G105" s="5"/>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G106" s="5"/>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G107" s="5"/>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G108" s="5"/>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G109" s="5"/>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="9">
         <f>MAX(A1:A109)</f>
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B110" s="9" t="s">
         <v>97</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:K94" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:K100" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="1.2"/>
+        <filter val="1.3"/>
+        <filter val="Roadmap"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="8">
       <filters>
+        <filter val="In Process"/>
         <filter val="Open"/>
         <filter val="Roadmap"/>
       </filters>
@@ -3640,10 +3809,10 @@
       <sortCondition ref="I1:I77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K94">
-    <sortCondition ref="G2:G94"/>
-    <sortCondition ref="I2:I94"/>
-    <sortCondition ref="A2:A94"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K100">
+    <sortCondition ref="G2:G100"/>
+    <sortCondition ref="I2:I100"/>
+    <sortCondition ref="A2:A100"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix date/time render bug
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F86AC4-0747-45C1-8F70-9FAD7149DCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4058CB-9634-4555-A090-92AC6F6E0D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$K$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$K$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="179">
   <si>
     <t>Item</t>
   </si>
@@ -568,6 +568,15 @@
   </si>
   <si>
     <t>Created Cell component</t>
+  </si>
+  <si>
+    <t>Empty date/time populates on front end as 1/1/1970</t>
+  </si>
+  <si>
+    <t>Urgent</t>
+  </si>
+  <si>
+    <t>1.2.1</t>
   </si>
 </sst>
 </file>
@@ -2806,7 +2815,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>68</v>
       </c>
@@ -2832,7 +2841,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>78</v>
       </c>
@@ -2859,7 +2868,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>93</v>
       </c>
@@ -2886,7 +2895,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>94</v>
       </c>
@@ -2913,7 +2922,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>98</v>
       </c>
@@ -3480,28 +3489,28 @@
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>24</v>
+        <v>177</v>
       </c>
       <c r="G90" s="5" t="s">
-        <v>134</v>
+        <v>178</v>
       </c>
       <c r="I90" s="4">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="J90" s="4" t="s">
         <v>27</v>
@@ -3509,10 +3518,10 @@
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>87</v>
+        <v>155</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>17</v>
@@ -3523,23 +3532,31 @@
       <c r="E91" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="F91" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="G91" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="I91" s="5"/>
+      <c r="I91" s="4">
+        <v>99</v>
+      </c>
       <c r="J91" s="4" t="s">
-        <v>134</v>
+        <v>27</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>135</v>
+        <v>87</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>17</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="E92" s="4" t="s">
         <v>25</v>
@@ -3552,18 +3569,15 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="D93" s="4" t="s">
-        <v>133</v>
       </c>
       <c r="E93" s="4" t="s">
         <v>25</v>
@@ -3576,12 +3590,12 @@
         <v>134</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>17</v>
@@ -3602,10 +3616,10 @@
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>17</v>
@@ -3618,9 +3632,6 @@
       </c>
       <c r="G95" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="H95" s="5" t="s">
-        <v>149</v>
       </c>
       <c r="I95" s="5"/>
       <c r="J95" s="4" t="s">
@@ -3629,10 +3640,10 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>17</v>
@@ -3645,6 +3656,9 @@
       </c>
       <c r="G96" s="5" t="s">
         <v>134</v>
+      </c>
+      <c r="H96" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="I96" s="5"/>
       <c r="J96" s="4" t="s">
@@ -3653,10 +3667,10 @@
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>17</v>
@@ -3677,10 +3691,10 @@
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>17</v>
@@ -3701,16 +3715,16 @@
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>25</v>
@@ -3725,36 +3739,57 @@
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G100" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="H100" s="5">
-        <v>98</v>
-      </c>
       <c r="I100" s="5"/>
       <c r="J100" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
+        <v>89</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G101" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H101" s="5">
+        <v>98</v>
+      </c>
+      <c r="I101" s="5"/>
+      <c r="J101" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="K100" s="4" t="s">
+      <c r="K101" s="4" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G101" s="5"/>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G102" s="5"/>
@@ -3783,25 +3818,19 @@
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="9">
         <f>MAX(A1:A109)</f>
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B110" s="9" t="s">
         <v>97</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:K100" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:K101" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="5">
       <filters>
         <filter val="1.2"/>
+        <filter val="1.2.1"/>
         <filter val="1.3"/>
-        <filter val="Roadmap"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="8">
-      <filters>
-        <filter val="In Process"/>
-        <filter val="Open"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>
@@ -3809,10 +3838,10 @@
       <sortCondition ref="I1:I77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K100">
-    <sortCondition ref="G2:G100"/>
-    <sortCondition ref="I2:I100"/>
-    <sortCondition ref="A2:A100"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K101">
+    <sortCondition ref="G2:G101"/>
+    <sortCondition ref="I2:I101"/>
+    <sortCondition ref="A2:A101"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Allow new row to be inserted either above or below the current row
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A48DD4-EA1D-40D5-831D-2A72612CD13C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0437A3A1-A392-4DE8-9452-DE67E3E1B2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$126</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="245">
   <si>
     <t>Item</t>
   </si>
@@ -702,9 +702,6 @@
     <t>1.2.2</t>
   </si>
   <si>
-    <t>Move is done.  Set menu guardrails so we don't move it out of bounds</t>
-  </si>
-  <si>
     <t>Support undo/redo</t>
   </si>
   <si>
@@ -778,6 +775,9 @@
   </si>
   <si>
     <t>Create Separate Cell Component</t>
+  </si>
+  <si>
+    <t>Fix grid lines so that double border lines don't appear</t>
   </si>
 </sst>
 </file>
@@ -3303,7 +3303,7 @@
         <v>89</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C66" s="15" t="s">
         <v>194</v>
@@ -3617,27 +3617,24 @@
         <v>1</v>
       </c>
       <c r="K76" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="L76" s="4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>227</v>
+        <v>165</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>6</v>
@@ -3648,28 +3645,28 @@
       <c r="H77" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="J77" s="4">
-        <v>2</v>
+      <c r="J77" s="5">
+        <v>1</v>
       </c>
       <c r="K77" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>228</v>
+        <v>166</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>6</v>
@@ -3680,19 +3677,19 @@
       <c r="H78" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="J78" s="4">
-        <v>3</v>
+      <c r="J78" s="5">
+        <v>2</v>
       </c>
       <c r="K78" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="C79" s="15" t="s">
         <v>195</v>
@@ -3713,24 +3710,24 @@
         <v>218</v>
       </c>
       <c r="J79" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K79" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>56</v>
@@ -3739,33 +3736,33 @@
         <v>6</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H80" s="13" t="s">
         <v>218</v>
       </c>
       <c r="J80" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K80" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="F81" s="4" t="s">
         <v>6</v>
@@ -3776,80 +3773,83 @@
       <c r="H81" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="J81" s="5">
-        <v>2</v>
+      <c r="J81" s="4">
+        <v>3</v>
       </c>
       <c r="K81" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>167</v>
+        <v>240</v>
       </c>
       <c r="C82" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="F82" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H82" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="J82" s="5">
-        <v>3</v>
+      <c r="J82" s="4">
+        <v>4</v>
       </c>
       <c r="K82" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>220</v>
+        <v>244</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="F83" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G83" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H83" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J83" s="5">
-        <v>10</v>
+      <c r="J83" s="4">
+        <v>5</v>
       </c>
       <c r="K83" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>195</v>
@@ -3858,12 +3858,9 @@
         <v>17</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>132</v>
+        <v>56</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G84" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H84" s="13" t="s">
@@ -3876,12 +3873,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>142</v>
+        <v>217</v>
       </c>
       <c r="C85" s="15" t="s">
         <v>195</v>
@@ -3895,12 +3892,12 @@
       <c r="F85" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="G85" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H85" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="I85" s="5" t="s">
-        <v>145</v>
-      </c>
       <c r="J85" s="5">
         <v>10</v>
       </c>
@@ -3908,12 +3905,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>174</v>
+        <v>142</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>195</v>
@@ -3922,27 +3919,30 @@
         <v>17</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>56</v>
+        <v>132</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H86" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J86" s="4">
+      <c r="I86" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="J86" s="5">
         <v>10</v>
       </c>
       <c r="K86" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>222</v>
+        <v>174</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>195</v>
@@ -3951,10 +3951,10 @@
         <v>17</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H87" s="13" t="s">
         <v>133</v>
@@ -3966,21 +3966,24 @@
         <v>133</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C88" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>56</v>
+        <v>87</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="H88" s="13" t="s">
         <v>133</v>
@@ -3992,15 +3995,15 @@
         <v>133</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>17</v>
@@ -4008,9 +4011,6 @@
       <c r="E89" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F89" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="H89" s="13" t="s">
         <v>133</v>
       </c>
@@ -4021,12 +4021,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>195</v>
@@ -4050,12 +4050,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>195</v>
@@ -4066,19 +4066,22 @@
       <c r="E91" s="4" t="s">
         <v>56</v>
       </c>
+      <c r="F91" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="H91" s="13" t="s">
         <v>133</v>
       </c>
       <c r="J91" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K91" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>65</v>
+        <v>116</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>233</v>
@@ -4092,31 +4095,25 @@
       <c r="E92" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F92" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="H92" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="I92" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="J92" s="5">
-        <v>20</v>
+      <c r="J92" s="4">
+        <v>15</v>
       </c>
       <c r="K92" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>17</v>
@@ -4130,6 +4127,9 @@
       <c r="H93" s="13" t="s">
         <v>133</v>
       </c>
+      <c r="I93" s="5" t="s">
+        <v>237</v>
+      </c>
       <c r="J93" s="5">
         <v>20</v>
       </c>
@@ -4137,76 +4137,73 @@
         <v>133</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>173</v>
+        <v>216</v>
       </c>
       <c r="C94" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E94" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H94" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J94" s="4">
+      <c r="J94" s="5">
         <v>20</v>
       </c>
       <c r="K94" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="C95" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E95" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H95" s="13" t="s">
         <v>133</v>
       </c>
       <c r="J95" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K95" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="C96" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>17</v>
@@ -4215,7 +4212,10 @@
         <v>56</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H96" s="13" t="s">
         <v>133</v>
@@ -4227,26 +4227,23 @@
         <v>133</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>229</v>
+        <v>175</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G97" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H97" s="13" t="s">
@@ -4259,23 +4256,26 @@
         <v>133</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C98" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>87</v>
       </c>
       <c r="F98" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G98" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H98" s="13" t="s">
@@ -4288,12 +4288,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C99" s="15" t="s">
         <v>195</v>
@@ -4317,9 +4317,9 @@
         <v>133</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>231</v>
@@ -4346,12 +4346,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>143</v>
+        <v>230</v>
       </c>
       <c r="C101" s="15" t="s">
         <v>195</v>
@@ -4360,27 +4360,27 @@
         <v>17</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>132</v>
+        <v>87</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H101" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J101" s="5">
-        <v>40</v>
+      <c r="J101" s="4">
+        <v>30</v>
       </c>
       <c r="K101" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>235</v>
+        <v>143</v>
       </c>
       <c r="C102" s="15" t="s">
         <v>195</v>
@@ -4389,36 +4389,33 @@
         <v>17</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>56</v>
+        <v>132</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H102" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="I102" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="J102" s="4">
+      <c r="J102" s="5">
         <v>40</v>
       </c>
       <c r="K102" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C103" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="E103" s="4" t="s">
         <v>56</v>
@@ -4426,12 +4423,12 @@
       <c r="F103" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G103" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H103" s="13" t="s">
         <v>133</v>
       </c>
+      <c r="I103" s="5" t="s">
+        <v>237</v>
+      </c>
       <c r="J103" s="4">
         <v>40</v>
       </c>
@@ -4439,12 +4436,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C104" s="15" t="s">
         <v>194</v>
@@ -4471,41 +4468,44 @@
         <v>133</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>131</v>
+        <v>242</v>
       </c>
       <c r="C105" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>132</v>
+        <v>56</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
+      </c>
+      <c r="G105" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H105" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J105" s="5">
-        <v>50</v>
+      <c r="J105" s="4">
+        <v>40</v>
       </c>
       <c r="K105" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="C106" s="15" t="s">
         <v>195</v>
@@ -4529,12 +4529,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>221</v>
+        <v>144</v>
       </c>
       <c r="C107" s="15" t="s">
         <v>195</v>
@@ -4543,27 +4543,27 @@
         <v>17</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>56</v>
+        <v>132</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H107" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J107" s="4">
+      <c r="J107" s="5">
         <v>50</v>
       </c>
       <c r="K107" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C108" s="15" t="s">
         <v>195</v>
@@ -4575,7 +4575,7 @@
         <v>56</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H108" s="13" t="s">
         <v>133</v>
@@ -4587,24 +4587,24 @@
         <v>133</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E109" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H109" s="13" t="s">
         <v>133</v>
@@ -4616,12 +4616,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C110" s="15" t="s">
         <v>194</v>
@@ -4645,50 +4645,50 @@
         <v>133</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E111" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H111" s="13" t="s">
         <v>133</v>
       </c>
       <c r="J111" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K111" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>134</v>
+        <v>223</v>
       </c>
       <c r="C112" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D112" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>132</v>
+        <v>56</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>25</v>
@@ -4696,19 +4696,19 @@
       <c r="H112" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J112" s="5">
-        <v>80</v>
+      <c r="J112" s="4">
+        <v>60</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>194</v>
@@ -4732,12 +4732,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>225</v>
+        <v>152</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>194</v>
@@ -4745,72 +4745,66 @@
       <c r="D114" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="E114" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="H114" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="J114" s="4">
+      <c r="J114" s="5">
         <v>80</v>
       </c>
       <c r="K114" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>82</v>
+        <v>224</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E115" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F115" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G115" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H115" s="13" t="s">
         <v>133</v>
       </c>
       <c r="J115" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="L115" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="F116" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G116" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H116" s="13" t="s">
         <v>133</v>
@@ -4821,13 +4815,16 @@
       <c r="K116" s="4" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L116" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C117" s="15" t="s">
         <v>194</v>
@@ -4842,7 +4839,7 @@
         <v>6</v>
       </c>
       <c r="G117" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H117" s="13" t="s">
         <v>133</v>
@@ -4854,18 +4851,18 @@
         <v>133</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E118" s="4" t="s">
         <v>31</v>
@@ -4874,7 +4871,7 @@
         <v>6</v>
       </c>
       <c r="G118" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H118" s="13" t="s">
         <v>133</v>
@@ -4886,21 +4883,21 @@
         <v>133</v>
       </c>
     </row>
-    <row r="119" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="C119" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F119" s="4" t="s">
         <v>6</v>
@@ -4917,16 +4914,13 @@
       <c r="K119" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="L119" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>194</v>
@@ -4935,13 +4929,13 @@
         <v>18</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G120" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H120" s="13" t="s">
         <v>133</v>
@@ -4952,13 +4946,16 @@
       <c r="K120" s="4" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L120" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>194</v>
@@ -4966,11 +4963,14 @@
       <c r="D121" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="E121" s="4" t="s">
+        <v>31</v>
+      </c>
       <c r="F121" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G121" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H121" s="13" t="s">
         <v>133</v>
@@ -4982,24 +4982,21 @@
         <v>133</v>
       </c>
     </row>
-    <row r="122" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E122" s="4" t="s">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G122" s="4" t="s">
         <v>24</v>
@@ -5014,12 +5011,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="123" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>194</v>
@@ -5046,27 +5043,27 @@
         <v>133</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>40</v>
+        <v>87</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>148</v>
+        <v>56</v>
       </c>
       <c r="F124" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H124" s="13" t="s">
         <v>133</v>
@@ -5077,28 +5074,25 @@
       <c r="K124" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="L124" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>194</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G125" s="4" t="s">
         <v>11</v>
@@ -5112,9 +5106,41 @@
       <c r="K125" s="4" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H126" s="13"/>
+      <c r="L125" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="4">
+        <v>88</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C126" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E126" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G126" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H126" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="J126" s="4">
+        <v>99</v>
+      </c>
+      <c r="K126" s="4" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H127" s="13"/>
@@ -5131,7 +5157,7 @@
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="9">
         <f>MAX(A1:A130)</f>
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B131" s="9" t="s">
         <v>96</v>
@@ -7825,22 +7851,21 @@
       <c r="H1026" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L125" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L126" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
         <filter val="1.2.1"/>
         <filter val="1.2.2"/>
-        <filter val="Roadmap"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L77">
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L125">
-    <sortCondition ref="H2:H125"/>
-    <sortCondition ref="J2:J125"/>
-    <sortCondition ref="A2:A125"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L126">
+    <sortCondition ref="H2:H126"/>
+    <sortCondition ref="J2:J126"/>
+    <sortCondition ref="A2:A126"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Allow date/time am/pm to be updated from typing a or p
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E08237C-E014-4FD6-B1DA-53313AC66A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B926123-7FF0-4B32-A406-8BA2E1CB2A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="248">
   <si>
     <t>Item</t>
   </si>
@@ -122,9 +122,6 @@
   </si>
   <si>
     <t>Done</t>
-  </si>
-  <si>
-    <t>Open</t>
   </si>
   <si>
     <t>Create optional grid border</t>
@@ -784,6 +781,12 @@
   </si>
   <si>
     <t>Allow Tab key to optionally create a new row from the bottom right cell</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Time format don't match what is entered on the screen.  Date and date/time appear okay</t>
   </si>
 </sst>
 </file>
@@ -1298,13 +1301,13 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -1319,10 +1322,10 @@
         <v>3</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>23</v>
@@ -1331,7 +1334,7 @@
         <v>16</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N1" s="7"/>
       <c r="O1" s="8"/>
@@ -1341,16 +1344,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>6</v>
@@ -1359,7 +1362,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>26</v>
@@ -1370,16 +1373,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>6</v>
@@ -1388,13 +1391,13 @@
         <v>7</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
@@ -1402,16 +1405,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
         <v>6</v>
@@ -1420,7 +1423,7 @@
         <v>7</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I4"/>
       <c r="J4"/>
@@ -1434,16 +1437,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D5" t="s">
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -1452,7 +1455,7 @@
         <v>7</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I5"/>
       <c r="J5"/>
@@ -1466,16 +1469,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
@@ -1484,7 +1487,7 @@
         <v>7</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I6"/>
       <c r="J6"/>
@@ -1498,16 +1501,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1516,7 +1519,7 @@
         <v>7</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1530,16 +1533,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D8" t="s">
         <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1548,7 +1551,7 @@
         <v>7</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I8"/>
       <c r="J8"/>
@@ -1562,16 +1565,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D9" t="s">
         <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1580,7 +1583,7 @@
         <v>7</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1594,16 +1597,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1612,7 +1615,7 @@
         <v>7</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I10"/>
       <c r="J10"/>
@@ -1626,16 +1629,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1644,7 +1647,7 @@
         <v>7</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I11"/>
       <c r="J11"/>
@@ -1658,16 +1661,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D12" t="s">
         <v>18</v>
       </c>
       <c r="E12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1676,7 +1679,7 @@
         <v>7</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I12"/>
       <c r="J12"/>
@@ -1690,16 +1693,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D13" t="s">
         <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1708,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I13"/>
       <c r="J13"/>
@@ -1722,10 +1725,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D14" t="s">
         <v>18</v>
@@ -1740,7 +1743,7 @@
         <v>7</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I14"/>
       <c r="J14"/>
@@ -1757,7 +1760,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -1772,7 +1775,7 @@
         <v>7</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I15"/>
       <c r="J15"/>
@@ -1786,10 +1789,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
@@ -1804,7 +1807,7 @@
         <v>7</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I16"/>
       <c r="J16"/>
@@ -1818,16 +1821,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D17" t="s">
         <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F17" t="s">
         <v>6</v>
@@ -1836,7 +1839,7 @@
         <v>11</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17"/>
@@ -1850,10 +1853,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D18" t="s">
         <v>18</v>
@@ -1868,7 +1871,7 @@
         <v>11</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18"/>
@@ -1882,10 +1885,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D19" t="s">
         <v>18</v>
@@ -1900,7 +1903,7 @@
         <v>11</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19"/>
@@ -1914,10 +1917,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D20" t="s">
         <v>18</v>
@@ -1932,7 +1935,7 @@
         <v>11</v>
       </c>
       <c r="H20" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20"/>
@@ -1946,10 +1949,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D21" t="s">
         <v>17</v>
@@ -1964,7 +1967,7 @@
         <v>7</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I21"/>
       <c r="J21"/>
@@ -1978,10 +1981,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D22" t="s">
         <v>18</v>
@@ -1996,7 +1999,7 @@
         <v>7</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I22"/>
       <c r="J22"/>
@@ -2013,7 +2016,7 @@
         <v>12</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
@@ -2028,7 +2031,7 @@
         <v>7</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I23"/>
       <c r="J23"/>
@@ -2042,10 +2045,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D24" t="s">
         <v>17</v>
@@ -2060,7 +2063,7 @@
         <v>7</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I24"/>
       <c r="J24"/>
@@ -2077,7 +2080,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D25" t="s">
         <v>18</v>
@@ -2092,7 +2095,7 @@
         <v>7</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I25"/>
       <c r="J25"/>
@@ -2109,7 +2112,7 @@
         <v>14</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D26" t="s">
         <v>18</v>
@@ -2124,7 +2127,7 @@
         <v>7</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I26"/>
       <c r="J26"/>
@@ -2138,16 +2141,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>6</v>
@@ -2156,7 +2159,7 @@
         <v>7</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K27" s="4" t="s">
         <v>26</v>
@@ -2170,7 +2173,7 @@
         <v>15</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D28" t="s">
         <v>18</v>
@@ -2185,7 +2188,7 @@
         <v>7</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I28"/>
       <c r="J28"/>
@@ -2202,7 +2205,7 @@
         <v>8</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D29" t="s">
         <v>18</v>
@@ -2217,7 +2220,7 @@
         <v>7</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I29"/>
       <c r="J29"/>
@@ -2231,16 +2234,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>6</v>
@@ -2249,7 +2252,7 @@
         <v>11</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>26</v>
@@ -2260,10 +2263,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D31" t="s">
         <v>18</v>
@@ -2278,7 +2281,7 @@
         <v>7</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I31"/>
       <c r="J31"/>
@@ -2292,16 +2295,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>25</v>
@@ -2310,7 +2313,7 @@
         <v>7</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K32" s="4" t="s">
         <v>26</v>
@@ -2321,16 +2324,16 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>6</v>
@@ -2339,13 +2342,13 @@
         <v>7</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K33" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L33" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -2353,16 +2356,16 @@
         <v>34</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>25</v>
@@ -2371,7 +2374,7 @@
         <v>7</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K34" s="4" t="s">
         <v>26</v>
@@ -2382,16 +2385,16 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
       </c>
       <c r="E35" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F35" t="s">
         <v>25</v>
@@ -2400,7 +2403,7 @@
         <v>24</v>
       </c>
       <c r="H35" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I35"/>
       <c r="J35"/>
@@ -2414,16 +2417,16 @@
         <v>38</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>11</v>
@@ -2432,7 +2435,7 @@
         <v>7</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>26</v>
@@ -2443,16 +2446,16 @@
         <v>40</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>11</v>
@@ -2461,7 +2464,7 @@
         <v>7</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>26</v>
@@ -2475,7 +2478,7 @@
         <v>19</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
@@ -2488,7 +2491,7 @@
         <v>11</v>
       </c>
       <c r="H38" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I38"/>
       <c r="J38"/>
@@ -2502,16 +2505,16 @@
         <v>42</v>
       </c>
       <c r="B39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
       </c>
       <c r="E39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F39" t="s">
         <v>6</v>
@@ -2520,7 +2523,7 @@
         <v>11</v>
       </c>
       <c r="H39" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I39"/>
       <c r="J39"/>
@@ -2534,16 +2537,16 @@
         <v>44</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>11</v>
@@ -2552,13 +2555,13 @@
         <v>7</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L40" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -2566,16 +2569,16 @@
         <v>45</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>6</v>
@@ -2584,7 +2587,7 @@
         <v>7</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K41" s="4" t="s">
         <v>26</v>
@@ -2595,16 +2598,16 @@
         <v>46</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>6</v>
@@ -2613,7 +2616,7 @@
         <v>7</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K42" s="4" t="s">
         <v>26</v>
@@ -2624,16 +2627,16 @@
         <v>47</v>
       </c>
       <c r="B43" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="D43" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C43" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="E43" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>6</v>
@@ -2642,13 +2645,13 @@
         <v>7</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K43" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L43" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -2656,16 +2659,16 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
       </c>
       <c r="E44" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F44" t="s">
         <v>6</v>
@@ -2674,7 +2677,7 @@
         <v>7</v>
       </c>
       <c r="H44" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I44" s="1"/>
       <c r="J44"/>
@@ -2688,16 +2691,16 @@
         <v>49</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>11</v>
@@ -2706,7 +2709,7 @@
         <v>11</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K45" s="4" t="s">
         <v>26</v>
@@ -2717,16 +2720,16 @@
         <v>50</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>6</v>
@@ -2735,7 +2738,7 @@
         <v>11</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K46" s="4" t="s">
         <v>26</v>
@@ -2746,16 +2749,16 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D47" t="s">
         <v>17</v>
       </c>
       <c r="E47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F47" t="s">
         <v>6</v>
@@ -2764,7 +2767,7 @@
         <v>7</v>
       </c>
       <c r="H47" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I47" s="1"/>
       <c r="J47"/>
@@ -2778,16 +2781,16 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D48" t="s">
         <v>17</v>
       </c>
       <c r="E48" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F48" t="s">
         <v>6</v>
@@ -2796,7 +2799,7 @@
         <v>7</v>
       </c>
       <c r="H48" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I48" s="1"/>
       <c r="J48"/>
@@ -2810,16 +2813,16 @@
         <v>58</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>11</v>
@@ -2828,7 +2831,7 @@
         <v>7</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K49" s="4" t="s">
         <v>26</v>
@@ -2839,16 +2842,16 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D50" t="s">
         <v>18</v>
       </c>
       <c r="E50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F50" t="s">
         <v>6</v>
@@ -2857,7 +2860,7 @@
         <v>7</v>
       </c>
       <c r="H50" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I50" s="1"/>
       <c r="J50"/>
@@ -2874,7 +2877,7 @@
         <v>22</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>17</v>
@@ -2889,7 +2892,7 @@
         <v>7</v>
       </c>
       <c r="H51" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K51" s="4" t="s">
         <v>26</v>
@@ -2900,16 +2903,16 @@
         <v>62</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>6</v>
@@ -2918,7 +2921,7 @@
         <v>7</v>
       </c>
       <c r="H52" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K52" s="4" t="s">
         <v>26</v>
@@ -2929,16 +2932,16 @@
         <v>63</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>25</v>
@@ -2947,7 +2950,7 @@
         <v>7</v>
       </c>
       <c r="H53" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K53" s="4" t="s">
         <v>26</v>
@@ -2959,16 +2962,16 @@
         <v>66</v>
       </c>
       <c r="B54" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F54" t="s">
         <v>6</v>
@@ -2977,7 +2980,7 @@
         <v>7</v>
       </c>
       <c r="H54" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54"/>
@@ -2991,16 +2994,16 @@
         <v>67</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>6</v>
@@ -3009,7 +3012,7 @@
         <v>7</v>
       </c>
       <c r="H55" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K55" s="4" t="s">
         <v>26</v>
@@ -3020,16 +3023,16 @@
         <v>69</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>6</v>
@@ -3038,7 +3041,7 @@
         <v>7</v>
       </c>
       <c r="H56" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K56" s="4" t="s">
         <v>26</v>
@@ -3049,16 +3052,16 @@
         <v>76</v>
       </c>
       <c r="B57" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E57" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="C57" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>138</v>
       </c>
       <c r="F57" s="4" t="s">
         <v>6</v>
@@ -3067,7 +3070,7 @@
         <v>7</v>
       </c>
       <c r="H57" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K57" s="4" t="s">
         <v>26</v>
@@ -3078,16 +3081,16 @@
         <v>76</v>
       </c>
       <c r="B58" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="D58" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C58" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>140</v>
-      </c>
       <c r="E58" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F58" s="4" t="s">
         <v>6</v>
@@ -3096,7 +3099,7 @@
         <v>7</v>
       </c>
       <c r="H58" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K58" s="4" t="s">
         <v>26</v>
@@ -3107,16 +3110,16 @@
         <v>82</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>6</v>
@@ -3125,7 +3128,7 @@
         <v>11</v>
       </c>
       <c r="H59" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J59" s="5"/>
       <c r="K59" s="4" t="s">
@@ -3137,16 +3140,16 @@
         <v>83</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>6</v>
@@ -3155,14 +3158,14 @@
         <v>11</v>
       </c>
       <c r="H60" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J60" s="5"/>
       <c r="K60" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L60" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -3170,16 +3173,16 @@
         <v>85</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>6</v>
@@ -3188,7 +3191,7 @@
         <v>7</v>
       </c>
       <c r="H61" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J61" s="5"/>
       <c r="K61" s="4" t="s">
@@ -3200,10 +3203,10 @@
         <v>32</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>18</v>
@@ -3218,7 +3221,7 @@
         <v>24</v>
       </c>
       <c r="H62" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K62" s="4" t="s">
         <v>26</v>
@@ -3229,10 +3232,10 @@
         <v>54</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>18</v>
@@ -3244,7 +3247,7 @@
         <v>24</v>
       </c>
       <c r="H63" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K63" s="4" t="s">
         <v>26</v>
@@ -3255,10 +3258,10 @@
         <v>61</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>17</v>
@@ -3270,7 +3273,7 @@
         <v>7</v>
       </c>
       <c r="H64" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J64" s="5"/>
       <c r="K64" s="4" t="s">
@@ -3282,22 +3285,22 @@
         <v>87</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H65" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J65" s="5"/>
       <c r="K65" s="4" t="s">
@@ -3309,22 +3312,22 @@
         <v>89</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F66" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H66" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J66" s="5">
         <v>20</v>
@@ -3338,22 +3341,22 @@
         <v>74</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H67" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J67" s="5"/>
       <c r="K67" s="4" t="s">
@@ -3365,22 +3368,22 @@
         <v>91</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F68" s="4" t="s">
         <v>24</v>
       </c>
       <c r="H68" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K68" s="4" t="s">
         <v>26</v>
@@ -3391,22 +3394,22 @@
         <v>92</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>24</v>
       </c>
       <c r="H69" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J69" s="5"/>
       <c r="K69" s="4" t="s">
@@ -3418,16 +3421,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>6</v>
@@ -3436,7 +3439,7 @@
         <v>24</v>
       </c>
       <c r="H70" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K70" s="4" t="s">
         <v>26</v>
@@ -3447,16 +3450,16 @@
         <v>78</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>25</v>
@@ -3465,7 +3468,7 @@
         <v>7</v>
       </c>
       <c r="H71" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J71" s="5"/>
       <c r="K71" s="4" t="s">
@@ -3477,16 +3480,16 @@
         <v>93</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>24</v>
@@ -3495,7 +3498,7 @@
         <v>11</v>
       </c>
       <c r="H72" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J72" s="5"/>
       <c r="K72" s="4" t="s">
@@ -3507,16 +3510,16 @@
         <v>94</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C73" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F73" s="4" t="s">
         <v>24</v>
@@ -3525,7 +3528,7 @@
         <v>11</v>
       </c>
       <c r="H73" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J73" s="5"/>
       <c r="K73" s="4" t="s">
@@ -3537,22 +3540,22 @@
         <v>98</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H74" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J74" s="5"/>
       <c r="K74" s="4" t="s">
@@ -3564,31 +3567,31 @@
         <v>99</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C75" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F75" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G75" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="H75" s="13" t="s">
         <v>170</v>
-      </c>
-      <c r="H75" s="13" t="s">
-        <v>171</v>
       </c>
       <c r="K75" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L75" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3596,16 +3599,16 @@
         <v>96</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F76" s="4" t="s">
         <v>6</v>
@@ -3614,30 +3617,30 @@
         <v>7</v>
       </c>
       <c r="H76" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J76" s="5">
         <v>1</v>
       </c>
       <c r="K76" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>97</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>6</v>
@@ -3646,11 +3649,16 @@
         <v>11</v>
       </c>
       <c r="H77" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="J77" s="5"/>
+        <v>217</v>
+      </c>
+      <c r="J77" s="5">
+        <v>2</v>
+      </c>
       <c r="K77" s="4" t="s">
-        <v>26</v>
+        <v>156</v>
+      </c>
+      <c r="L77" s="4" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
@@ -3658,16 +3666,16 @@
         <v>90</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>11</v>
@@ -3676,7 +3684,7 @@
         <v>7</v>
       </c>
       <c r="H78" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J78" s="5"/>
       <c r="K78" s="4" t="s">
@@ -3688,16 +3696,16 @@
         <v>95</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F79" s="4" t="s">
         <v>6</v>
@@ -3706,7 +3714,7 @@
         <v>7</v>
       </c>
       <c r="H79" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J79" s="5"/>
       <c r="K79" s="4" t="s">
@@ -3718,16 +3726,16 @@
         <v>109</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F80" s="4" t="s">
         <v>6</v>
@@ -3736,7 +3744,7 @@
         <v>7</v>
       </c>
       <c r="H80" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K80" s="4" t="s">
         <v>26</v>
@@ -3747,16 +3755,16 @@
         <v>110</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F81" s="4" t="s">
         <v>6</v>
@@ -3765,7 +3773,7 @@
         <v>7</v>
       </c>
       <c r="H81" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K81" s="4" t="s">
         <v>26</v>
@@ -3776,16 +3784,16 @@
         <v>111</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C82" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F82" s="4" t="s">
         <v>6</v>
@@ -3794,7 +3802,7 @@
         <v>7</v>
       </c>
       <c r="H82" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K82" s="4" t="s">
         <v>26</v>
@@ -3805,16 +3813,16 @@
         <v>125</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F83" s="4" t="s">
         <v>6</v>
@@ -3823,7 +3831,7 @@
         <v>7</v>
       </c>
       <c r="H83" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K83" s="4" t="s">
         <v>26</v>
@@ -3834,16 +3842,16 @@
         <v>124</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F84" s="4" t="s">
         <v>6</v>
@@ -3852,13 +3860,13 @@
         <v>7</v>
       </c>
       <c r="H84" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J84" s="4">
         <v>5</v>
       </c>
       <c r="K84" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="85" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -3866,28 +3874,28 @@
         <v>56</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H85" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J85" s="5">
         <v>10</v>
       </c>
       <c r="K85" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -3895,16 +3903,16 @@
         <v>73</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C86" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F86" s="4" t="s">
         <v>25</v>
@@ -3913,13 +3921,13 @@
         <v>7</v>
       </c>
       <c r="H86" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J86" s="5">
         <v>10</v>
       </c>
       <c r="K86" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -3927,31 +3935,31 @@
         <v>77</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F87" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H87" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I87" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J87" s="5">
         <v>10</v>
       </c>
       <c r="K87" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -3959,28 +3967,28 @@
         <v>101</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C88" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F88" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H88" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J88" s="4">
         <v>10</v>
       </c>
       <c r="K88" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -3988,28 +3996,28 @@
         <v>104</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F89" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H89" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J89" s="4">
         <v>10</v>
       </c>
       <c r="K89" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4017,25 +4025,25 @@
         <v>105</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H90" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J90" s="4">
         <v>10</v>
       </c>
       <c r="K90" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4043,28 +4051,28 @@
         <v>118</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F91" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H91" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J91" s="4">
         <v>10</v>
       </c>
       <c r="K91" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="92" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4072,28 +4080,28 @@
         <v>119</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C92" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F92" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H92" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J92" s="4">
         <v>10</v>
       </c>
       <c r="K92" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4101,25 +4109,25 @@
         <v>116</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H93" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J93" s="4">
         <v>15</v>
       </c>
       <c r="K93" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4127,31 +4135,31 @@
         <v>65</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C94" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H94" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J94" s="5">
         <v>20</v>
       </c>
       <c r="K94" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="95" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4159,28 +4167,28 @@
         <v>86</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C95" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H95" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J95" s="5">
         <v>20</v>
       </c>
       <c r="K95" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4188,28 +4196,28 @@
         <v>100</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C96" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F96" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H96" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J96" s="4">
         <v>20</v>
       </c>
       <c r="K96" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4217,16 +4225,16 @@
         <v>83</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F97" s="4" t="s">
         <v>25</v>
@@ -4235,13 +4243,13 @@
         <v>24</v>
       </c>
       <c r="H97" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J97" s="4">
         <v>30</v>
       </c>
       <c r="K97" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4249,28 +4257,28 @@
         <v>102</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C98" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F98" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H98" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J98" s="4">
         <v>30</v>
       </c>
       <c r="K98" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4278,16 +4286,16 @@
         <v>112</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C99" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F99" s="4" t="s">
         <v>6</v>
@@ -4296,13 +4304,13 @@
         <v>7</v>
       </c>
       <c r="H99" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J99" s="4">
         <v>30</v>
       </c>
       <c r="K99" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4310,28 +4318,28 @@
         <v>113</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C100" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F100" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H100" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J100" s="4">
         <v>30</v>
       </c>
       <c r="K100" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
@@ -4339,28 +4347,28 @@
         <v>114</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C101" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F101" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H101" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J101" s="4">
         <v>30</v>
       </c>
       <c r="K101" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4368,28 +4376,28 @@
         <v>115</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F102" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H102" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J102" s="4">
         <v>30</v>
       </c>
       <c r="K102" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4397,28 +4405,28 @@
         <v>79</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C103" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D103" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F103" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H103" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J103" s="5">
         <v>40</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4426,31 +4434,31 @@
         <v>117</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C104" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D104" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F104" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H104" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I104" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J104" s="4">
         <v>40</v>
       </c>
       <c r="K104" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4458,16 +4466,16 @@
         <v>122</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C105" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F105" s="4" t="s">
         <v>7</v>
@@ -4476,13 +4484,13 @@
         <v>11</v>
       </c>
       <c r="H105" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J105" s="4">
         <v>40</v>
       </c>
       <c r="K105" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4490,16 +4498,16 @@
         <v>123</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C106" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F106" s="4" t="s">
         <v>7</v>
@@ -4508,13 +4516,13 @@
         <v>11</v>
       </c>
       <c r="H106" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J106" s="4">
         <v>40</v>
       </c>
       <c r="K106" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
@@ -4522,16 +4530,16 @@
         <v>26</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C107" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>11</v>
@@ -4540,13 +4548,13 @@
         <v>11</v>
       </c>
       <c r="H107" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J107" s="4">
         <v>50</v>
       </c>
       <c r="K107" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
@@ -4554,28 +4562,28 @@
         <v>72</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F108" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H108" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J108" s="5">
         <v>50</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4583,28 +4591,28 @@
         <v>80</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F109" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H109" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J109" s="5">
         <v>50</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4612,28 +4620,28 @@
         <v>103</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D110" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F110" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H110" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J110" s="4">
         <v>50</v>
       </c>
       <c r="K110" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4641,28 +4649,28 @@
         <v>108</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D111" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F111" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H111" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J111" s="4">
         <v>50</v>
       </c>
       <c r="K111" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -4670,28 +4678,28 @@
         <v>120</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C112" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D112" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H112" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J112" s="4">
         <v>50</v>
       </c>
       <c r="K112" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4699,28 +4707,28 @@
         <v>121</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C113" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D113" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F113" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H113" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J113" s="4">
         <v>50</v>
       </c>
       <c r="K113" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4728,28 +4736,28 @@
         <v>106</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C114" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D114" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F114" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H114" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J114" s="4">
         <v>60</v>
       </c>
       <c r="K114" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4757,28 +4765,28 @@
         <v>75</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C115" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D115" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H115" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J115" s="5">
         <v>80</v>
       </c>
       <c r="K115" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4786,28 +4794,28 @@
         <v>84</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C116" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F116" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H116" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J116" s="5">
         <v>80</v>
       </c>
       <c r="K116" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4815,22 +4823,22 @@
         <v>107</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>17</v>
       </c>
       <c r="H117" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J117" s="4">
         <v>80</v>
       </c>
       <c r="K117" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4838,16 +4846,16 @@
         <v>35</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F118" s="4" t="s">
         <v>6</v>
@@ -4856,16 +4864,16 @@
         <v>11</v>
       </c>
       <c r="H118" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J118" s="4">
         <v>99</v>
       </c>
       <c r="K118" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L118" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4873,16 +4881,16 @@
         <v>36</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F119" s="4" t="s">
         <v>6</v>
@@ -4891,13 +4899,13 @@
         <v>24</v>
       </c>
       <c r="H119" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J119" s="4">
         <v>99</v>
       </c>
       <c r="K119" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4905,16 +4913,16 @@
         <v>39</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F120" s="4" t="s">
         <v>6</v>
@@ -4923,13 +4931,13 @@
         <v>11</v>
       </c>
       <c r="H120" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J120" s="4">
         <v>99</v>
       </c>
       <c r="K120" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -4937,16 +4945,16 @@
         <v>43</v>
       </c>
       <c r="B121" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C121" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="D121" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C121" s="15" t="s">
-        <v>194</v>
-      </c>
-      <c r="D121" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="E121" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>6</v>
@@ -4955,13 +4963,13 @@
         <v>24</v>
       </c>
       <c r="H121" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J121" s="4">
         <v>99</v>
       </c>
       <c r="K121" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="122" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
@@ -4969,10 +4977,10 @@
         <v>52</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C122" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D122" s="4" t="s">
         <v>18</v>
@@ -4987,16 +4995,16 @@
         <v>24</v>
       </c>
       <c r="H122" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J122" s="4">
         <v>99</v>
       </c>
       <c r="K122" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L122" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -5004,16 +5012,16 @@
         <v>53</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C123" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F123" s="4" t="s">
         <v>11</v>
@@ -5022,13 +5030,13 @@
         <v>7</v>
       </c>
       <c r="H123" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J123" s="4">
         <v>99</v>
       </c>
       <c r="K123" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -5036,10 +5044,10 @@
         <v>55</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C124" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D124" s="4" t="s">
         <v>18</v>
@@ -5051,13 +5059,13 @@
         <v>24</v>
       </c>
       <c r="H124" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J124" s="4">
         <v>99</v>
       </c>
       <c r="K124" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="125" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
@@ -5065,16 +5073,16 @@
         <v>70</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>6</v>
@@ -5083,13 +5091,13 @@
         <v>24</v>
       </c>
       <c r="H125" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J125" s="4">
         <v>99</v>
       </c>
       <c r="K125" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="126" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
@@ -5097,16 +5105,16 @@
         <v>71</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
         <v>6</v>
@@ -5115,13 +5123,13 @@
         <v>24</v>
       </c>
       <c r="H126" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J126" s="4">
         <v>99</v>
       </c>
       <c r="K126" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -5129,16 +5137,16 @@
         <v>81</v>
       </c>
       <c r="B127" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C127" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E127" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="C127" s="15" t="s">
-        <v>194</v>
-      </c>
-      <c r="D127" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E127" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>6</v>
@@ -5147,16 +5155,16 @@
         <v>11</v>
       </c>
       <c r="H127" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J127" s="4">
         <v>99</v>
       </c>
       <c r="K127" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L127" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -5164,16 +5172,16 @@
         <v>88</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>11</v>
@@ -5182,13 +5190,13 @@
         <v>11</v>
       </c>
       <c r="H128" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J128" s="4">
         <v>99</v>
       </c>
       <c r="K128" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.25">
@@ -5233,7 +5241,7 @@
         <v>125</v>
       </c>
       <c r="B141" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C141" s="16"/>
       <c r="H141" s="13"/>
@@ -7971,56 +7979,56 @@
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D1" s="19"/>
       <c r="E1" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J1" s="19"/>
       <c r="K1" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="L1" s="20" t="s">
         <v>183</v>
-      </c>
-      <c r="L1" s="20" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:44" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21"/>
       <c r="B2" s="21"/>
       <c r="C2" s="22" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E2" s="23"/>
       <c r="F2" s="23"/>
       <c r="G2" s="23"/>
       <c r="H2" s="23"/>
       <c r="I2" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="J2" s="22" t="s">
         <v>190</v>
-      </c>
-      <c r="J2" s="22" t="s">
-        <v>191</v>
       </c>
       <c r="K2" s="23"/>
       <c r="L2" s="23"/>
@@ -8039,34 +8047,34 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K3" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
@@ -8103,40 +8111,40 @@
     </row>
     <row r="4" spans="1:44" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K4" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="L4" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>188</v>
       </c>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
@@ -8173,7 +8181,7 @@
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>7</v>
@@ -8182,7 +8190,7 @@
       <c r="D5" s="13"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -8225,7 +8233,7 @@
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
@@ -8234,7 +8242,7 @@
       <c r="D6" s="13"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -8277,7 +8285,7 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>7</v>
@@ -8286,7 +8294,7 @@
       <c r="D7" s="13"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -8329,7 +8337,7 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>24</v>
@@ -8338,7 +8346,7 @@
       <c r="D8" s="13"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -8381,7 +8389,7 @@
     </row>
     <row r="9" spans="1:44" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>24</v>
@@ -8390,7 +8398,7 @@
       <c r="D9" s="13"/>
       <c r="E9" s="14"/>
       <c r="F9" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -8433,7 +8441,7 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>11</v>
@@ -8442,7 +8450,7 @@
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -8485,7 +8493,7 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>11</v>
@@ -8494,7 +8502,7 @@
       <c r="D11" s="13"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -8537,7 +8545,7 @@
     </row>
     <row r="12" spans="1:44" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>11</v>
@@ -8546,7 +8554,7 @@
       <c r="D12" s="13"/>
       <c r="E12" s="14"/>
       <c r="F12" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -8589,7 +8597,7 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>11</v>
@@ -8598,7 +8606,7 @@
       <c r="D13" s="13"/>
       <c r="E13" s="14"/>
       <c r="F13" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -12718,148 +12726,148 @@
   <sheetData>
     <row r="9" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
         <v>98</v>
       </c>
-      <c r="C9" t="s">
-        <v>99</v>
-      </c>
       <c r="D9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="T16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" t="s">
         <v>98</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>100</v>
       </c>
-      <c r="E19" t="s">
-        <v>101</v>
-      </c>
       <c r="G19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="G21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" t="s">
         <v>98</v>
       </c>
-      <c r="C24" t="s">
-        <v>99</v>
-      </c>
       <c r="D24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E24" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="G25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" t="s">
         <v>98</v>
       </c>
-      <c r="C29" t="s">
-        <v>99</v>
-      </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E29" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="G30" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G34" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E36" t="s">
+        <v>107</v>
+      </c>
+      <c r="G36" t="s">
         <v>108</v>
-      </c>
-      <c r="G36" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="37" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G37" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G38" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G39" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" spans="5:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G40" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="41" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="42" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G42" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="5:7" x14ac:dyDescent="0.25">
       <c r="G43" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial commit to add number column type and css class maintenance system
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64EAD9AA-0D77-4D54-B638-B93A102A052D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C48947E-9A46-4158-8194-2DE2B9D52F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
     <sheet name="Data Types" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="date-time Data Shape" sheetId="5" r:id="rId3"/>
+    <sheet name="Number Data Shape" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$138</definedName>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="299">
   <si>
     <t>Item</t>
   </si>
@@ -850,6 +852,96 @@
   </si>
   <si>
     <t>1.2.4</t>
+  </si>
+  <si>
+    <t>dataType</t>
+  </si>
+  <si>
+    <t>attributes.columnDataType {</t>
+  </si>
+  <si>
+    <t>type,</t>
+  </si>
+  <si>
+    <t>dataType.type</t>
+  </si>
+  <si>
+    <t>settings {</t>
+  </si>
+  <si>
+    <t>format,</t>
+  </si>
+  <si>
+    <t>formatOptions {</t>
+  </si>
+  <si>
+    <t>decimalPlaces</t>
+  </si>
+  <si>
+    <t>thousandSeparator</t>
+  </si>
+  <si>
+    <t>decimalPlaces,</t>
+  </si>
+  <si>
+    <t>showCurrencySymbol,</t>
+  </si>
+  <si>
+    <t>thousandSeparator,</t>
+  </si>
+  <si>
+    <t>}</t>
+  </si>
+  <si>
+    <t>Object Shape</t>
+  </si>
+  <si>
+    <t>dataTypeFormat</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>State Variable</t>
+  </si>
+  <si>
+    <t>date-time</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>Default Value</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>defaultToToday,</t>
+  </si>
+  <si>
+    <t>dateDefaultToToday</t>
+  </si>
+  <si>
+    <t>Valid</t>
+  </si>
+  <si>
+    <t>Any integer</t>
+  </si>
+  <si>
+    <t>true | false</t>
+  </si>
+  <si>
+    <t>number | integer | currency</t>
   </si>
 </sst>
 </file>
@@ -960,7 +1052,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1016,6 +1108,9 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1031,6 +1126,8 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3485,7 +3582,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>68</v>
       </c>
@@ -3514,7 +3611,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>78</v>
       </c>
@@ -3544,7 +3641,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>93</v>
       </c>
@@ -3574,7 +3671,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>94</v>
       </c>
@@ -3604,7 +3701,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>98</v>
       </c>
@@ -3631,7 +3728,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>99</v>
       </c>
@@ -3663,7 +3760,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>90</v>
       </c>
@@ -3693,7 +3790,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>95</v>
       </c>
@@ -3723,7 +3820,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>96</v>
       </c>
@@ -3753,7 +3850,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>97</v>
       </c>
@@ -3786,7 +3883,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>109</v>
       </c>
@@ -3815,7 +3912,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>110</v>
       </c>
@@ -3844,7 +3941,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>111</v>
       </c>
@@ -3873,7 +3970,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>125</v>
       </c>
@@ -8305,6 +8402,9 @@
   <autoFilter ref="B1:L138" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
+        <filter val="1.2.0"/>
+        <filter val="1.2.1"/>
+        <filter val="1.2.2"/>
         <filter val="1.2.3"/>
         <filter val="1.2.4"/>
         <filter val="Roadmap"/>
@@ -8343,43 +8443,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="19"/>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="24" t="s">
         <v>194</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="21" t="s">
+      <c r="E1" s="24"/>
+      <c r="F1" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="J1" s="23" t="s">
+      <c r="J1" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="K1" s="23"/>
-      <c r="L1" s="21" t="s">
+      <c r="K1" s="24"/>
+      <c r="L1" s="22" t="s">
         <v>180</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="22" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:45" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
       <c r="C2" s="20" t="s">
         <v>16</v>
       </c>
@@ -8389,18 +8489,18 @@
       <c r="E2" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
       <c r="J2" s="18" t="s">
         <v>187</v>
       </c>
       <c r="K2" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -13222,6 +13322,239 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C07A045-EDB0-4506-A2E7-225FA060F54C}">
+  <dimension ref="B2:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
+    <col min="2" max="5" width="3.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="21" t="s">
+        <v>285</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G4" t="s">
+        <v>272</v>
+      </c>
+      <c r="H4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>274</v>
+      </c>
+      <c r="G6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>293</v>
+      </c>
+      <c r="G7" t="s">
+        <v>294</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>281</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F4CAB31-52FD-431F-AA77-05BD26AC0272}">
+  <dimension ref="B2:I13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
+    <col min="2" max="5" width="3.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" customWidth="1"/>
+    <col min="9" max="9" width="68.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="21" t="s">
+        <v>285</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G4" t="s">
+        <v>272</v>
+      </c>
+      <c r="H4" t="s">
+        <v>289</v>
+      </c>
+      <c r="I4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>274</v>
+      </c>
+      <c r="G6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H6" t="s">
+        <v>289</v>
+      </c>
+      <c r="I6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>278</v>
+      </c>
+      <c r="G8" t="s">
+        <v>276</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>290</v>
+      </c>
+      <c r="I8" s="28" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>279</v>
+      </c>
+      <c r="G9" t="s">
+        <v>284</v>
+      </c>
+      <c r="H9" s="28" t="s">
+        <v>291</v>
+      </c>
+      <c r="I9" s="28" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>280</v>
+      </c>
+      <c r="G10" t="s">
+        <v>277</v>
+      </c>
+      <c r="H10" s="28" t="s">
+        <v>292</v>
+      </c>
+      <c r="I10" s="28" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>281</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
   <dimension ref="B9:T43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add support for keyboard insert/delete rows and columns
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714634A0-50FA-45A1-9653-453C305AD504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{384A0E14-06CB-4B5A-A9E5-DE43B4A5F7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -973,15 +973,14 @@
 - currency</t>
   </si>
   <si>
+    <t>Create CSS class controller</t>
+  </si>
+  <si>
+    <t>1.2.5</t>
+  </si>
+  <si>
     <t>- Add support for multi-currency
-- Add decimal alignment
-- Percent entry shows fractional number</t>
-  </si>
-  <si>
-    <t>Create CSS class controller</t>
-  </si>
-  <si>
-    <t>1.2.5</t>
+- Add decimal alignment</t>
   </si>
 </sst>
 </file>
@@ -3625,7 +3624,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>68</v>
       </c>
@@ -3654,7 +3653,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>78</v>
       </c>
@@ -3684,7 +3683,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>93</v>
       </c>
@@ -3714,7 +3713,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>94</v>
       </c>
@@ -3744,7 +3743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>98</v>
       </c>
@@ -3771,7 +3770,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>99</v>
       </c>
@@ -3803,7 +3802,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>90</v>
       </c>
@@ -3833,7 +3832,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>95</v>
       </c>
@@ -3863,7 +3862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>96</v>
       </c>
@@ -3893,7 +3892,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>97</v>
       </c>
@@ -3926,7 +3925,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>109</v>
       </c>
@@ -3955,7 +3954,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>110</v>
       </c>
@@ -3984,7 +3983,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>111</v>
       </c>
@@ -4013,7 +4012,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>125</v>
       </c>
@@ -4042,7 +4041,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>128</v>
       </c>
@@ -4071,7 +4070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>135</v>
       </c>
@@ -4102,25 +4101,22 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>307</v>
+        <v>260</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G86" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H86" s="13" t="s">
         <v>265</v>
@@ -4131,22 +4127,25 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>260</v>
+        <v>306</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H87" s="13" t="s">
         <v>265</v>
@@ -4178,10 +4177,10 @@
         <v>7</v>
       </c>
       <c r="H88" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J88" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K88" s="4" t="s">
         <v>256</v>
@@ -4210,10 +4209,10 @@
         <v>7</v>
       </c>
       <c r="H89" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J89" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K89" s="4" t="s">
         <v>256</v>
@@ -4242,10 +4241,10 @@
         <v>168</v>
       </c>
       <c r="H90" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J90" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K90" s="4" t="s">
         <v>256</v>
@@ -4256,10 +4255,10 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>56</v>
+        <v>134</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>214</v>
+        <v>262</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>190</v>
@@ -4271,24 +4270,27 @@
         <v>55</v>
       </c>
       <c r="F91" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G91" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H91" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J91" s="5">
-        <v>10</v>
+        <v>307</v>
+      </c>
+      <c r="J91" s="4">
+        <v>4</v>
       </c>
       <c r="K91" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>190</v>
@@ -4297,12 +4299,9 @@
         <v>17</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G92" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H92" s="13" t="s">
@@ -4317,10 +4316,10 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
       <c r="C93" s="15" t="s">
         <v>190</v>
@@ -4334,12 +4333,12 @@
       <c r="F93" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="G93" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H93" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I93" s="5">
-        <v>80</v>
-      </c>
       <c r="J93" s="5">
         <v>10</v>
       </c>
@@ -4347,12 +4346,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>258</v>
+        <v>141</v>
       </c>
       <c r="C94" s="15" t="s">
         <v>190</v>
@@ -4361,33 +4360,30 @@
         <v>17</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H94" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I94" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="J94" s="4">
+      <c r="I94" s="5">
+        <v>80</v>
+      </c>
+      <c r="J94" s="5">
         <v>10</v>
       </c>
       <c r="K94" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L94" s="4" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>216</v>
+        <v>258</v>
       </c>
       <c r="C95" s="15" t="s">
         <v>190</v>
@@ -4396,36 +4392,45 @@
         <v>17</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H95" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I95" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J95" s="4">
         <v>10</v>
       </c>
       <c r="K95" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L95" s="4" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C96" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="H96" s="13" t="s">
         <v>132</v>
@@ -4439,13 +4444,13 @@
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>17</v>
@@ -4453,9 +4458,6 @@
       <c r="E97" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F97" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="H97" s="13" t="s">
         <v>132</v>
       </c>
@@ -4468,16 +4470,16 @@
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="C98" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>55</v>
@@ -4485,9 +4487,6 @@
       <c r="F98" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G98" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H98" s="13" t="s">
         <v>132</v>
       </c>
@@ -4500,10 +4499,10 @@
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C99" s="15" t="s">
         <v>190</v>
@@ -4515,7 +4514,7 @@
         <v>55</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G99" s="4" t="s">
         <v>7</v>
@@ -4529,16 +4528,13 @@
       <c r="K99" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L99" s="4" t="s">
-        <v>248</v>
-      </c>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C100" s="15" t="s">
         <v>190</v>
@@ -4564,25 +4560,28 @@
       <c r="K100" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L100" s="4" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="C101" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E101" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>7</v>
@@ -8498,11 +8497,8 @@
   <autoFilter ref="B1:L139" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
-        <filter val="1.2.0"/>
-        <filter val="1.2.1"/>
-        <filter val="1.2.2"/>
-        <filter val="1.2.3"/>
         <filter val="1.2.4"/>
+        <filter val="1.2.5"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>
@@ -8529,7 +8525,7 @@
     <col min="2" max="2" width="10.7109375" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="14.140625" style="12" customWidth="1"/>
     <col min="4" max="5" width="9.5703125" style="12" customWidth="1"/>
-    <col min="6" max="6" width="35.140625" style="12" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="35.140625" style="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
@@ -8758,14 +8754,14 @@
         <v>7</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>155</v>
+        <v>261</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>265</v>
       </c>
       <c r="E5" s="13"/>
       <c r="F5" s="29" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>203</v>

</xml_diff>

<commit_message>
Start clearnup for Aria support
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{384A0E14-06CB-4B5A-A9E5-DE43B4A5F7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E071E3-7028-4FBE-ADD3-FB44E7F87007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="313">
   <si>
     <t>Item</t>
   </si>
@@ -981,6 +981,18 @@
   <si>
     <t>- Add support for multi-currency
 - Add decimal alignment</t>
+  </si>
+  <si>
+    <t>Support Aria semantics for screen readers</t>
+  </si>
+  <si>
+    <t>Enhancement</t>
+  </si>
+  <si>
+    <t>Cleanup</t>
+  </si>
+  <si>
+    <t>On Render, text color is same as banded row color</t>
   </si>
 </sst>
 </file>
@@ -2841,10 +2853,10 @@
         <v>178</v>
       </c>
       <c r="D43" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>6</v>
@@ -3208,10 +3220,10 @@
         <v>178</v>
       </c>
       <c r="D55" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E55" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>6</v>
@@ -3237,10 +3249,10 @@
         <v>178</v>
       </c>
       <c r="D56" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E56" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>6</v>
@@ -3635,10 +3647,10 @@
         <v>189</v>
       </c>
       <c r="D70" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E70" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>6</v>
@@ -4278,11 +4290,8 @@
       <c r="H91" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="J91" s="4">
-        <v>4</v>
-      </c>
       <c r="K91" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
@@ -4598,25 +4607,31 @@
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>228</v>
+        <v>309</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>17</v>
+        <v>310</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H102" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J102" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K102" s="4" t="s">
         <v>132</v>
@@ -4624,10 +4639,10 @@
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C103" s="15" t="s">
         <v>190</v>
@@ -4638,9 +4653,6 @@
       <c r="E103" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F103" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="H103" s="13" t="s">
         <v>132</v>
       </c>
@@ -4653,10 +4665,10 @@
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C104" s="15" t="s">
         <v>190</v>
@@ -4668,16 +4680,13 @@
         <v>55</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H104" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I104" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J104" s="5">
-        <v>20</v>
+      <c r="J104" s="4">
+        <v>15</v>
       </c>
       <c r="K104" s="4" t="s">
         <v>132</v>
@@ -4685,13 +4694,13 @@
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="C105" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D105" s="4" t="s">
         <v>17</v>
@@ -4705,6 +4714,9 @@
       <c r="H105" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I105" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J105" s="5">
         <v>20</v>
       </c>
@@ -4714,27 +4726,27 @@
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="C106" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E106" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H106" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J106" s="4">
+      <c r="J106" s="5">
         <v>20</v>
       </c>
       <c r="K106" s="4" t="s">
@@ -4743,13 +4755,13 @@
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C107" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>18</v>
@@ -4758,10 +4770,7 @@
         <v>55</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G107" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H107" s="13" t="s">
         <v>132</v>
@@ -4772,28 +4781,25 @@
       <c r="K107" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L107" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>83</v>
+        <v>127</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>149</v>
+        <v>244</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E108" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G108" s="4" t="s">
         <v>24</v>
@@ -4802,21 +4808,24 @@
         <v>132</v>
       </c>
       <c r="J108" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K108" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L108" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>17</v>
@@ -4825,7 +4834,10 @@
         <v>55</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G109" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H109" s="13" t="s">
         <v>132</v>
@@ -4839,24 +4851,21 @@
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G110" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H110" s="13" t="s">
@@ -4871,21 +4880,24 @@
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E111" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F111" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G111" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
@@ -4898,12 +4910,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="112" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C112" s="15" t="s">
         <v>190</v>
@@ -4927,12 +4939,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>190</v>
@@ -4958,10 +4970,10 @@
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>190</v>
@@ -4970,16 +4982,16 @@
         <v>17</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H114" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J114" s="5">
-        <v>40</v>
+      <c r="J114" s="4">
+        <v>30</v>
       </c>
       <c r="K114" s="4" t="s">
         <v>132</v>
@@ -4987,10 +4999,10 @@
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>190</v>
@@ -4999,18 +5011,15 @@
         <v>17</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H115" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I115" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J115" s="4">
+      <c r="J115" s="5">
         <v>40</v>
       </c>
       <c r="K115" s="4" t="s">
@@ -5019,16 +5028,16 @@
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C116" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="E116" s="4" t="s">
         <v>55</v>
@@ -5036,12 +5045,12 @@
       <c r="F116" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G116" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H116" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I116" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J116" s="4">
         <v>40</v>
       </c>
@@ -5051,19 +5060,19 @@
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C117" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E117" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E117" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>7</v>
@@ -5081,12 +5090,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="118" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>189</v>
@@ -5095,10 +5104,10 @@
         <v>17</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G118" s="4" t="s">
         <v>11</v>
@@ -5107,7 +5116,7 @@
         <v>132</v>
       </c>
       <c r="J118" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K118" s="4" t="s">
         <v>132</v>
@@ -5115,39 +5124,42 @@
     </row>
     <row r="119" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G119" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H119" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J119" s="5">
+      <c r="J119" s="4">
         <v>50</v>
       </c>
       <c r="K119" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>190</v>
@@ -5173,10 +5185,10 @@
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>190</v>
@@ -5185,15 +5197,15 @@
         <v>17</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H121" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J121" s="4">
+      <c r="J121" s="5">
         <v>50</v>
       </c>
       <c r="K121" s="4" t="s">
@@ -5202,10 +5214,10 @@
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>190</v>
@@ -5217,7 +5229,7 @@
         <v>55</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H122" s="13" t="s">
         <v>132</v>
@@ -5231,22 +5243,22 @@
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>233</v>
+        <v>220</v>
       </c>
       <c r="C123" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E123" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H123" s="13" t="s">
         <v>132</v>
@@ -5260,10 +5272,10 @@
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>189</v>
@@ -5289,28 +5301,28 @@
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E125" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H125" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J125" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K125" s="4" t="s">
         <v>132</v>
@@ -5318,19 +5330,19 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
         <v>25</v>
@@ -5338,8 +5350,8 @@
       <c r="H126" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J126" s="5">
-        <v>80</v>
+      <c r="J126" s="4">
+        <v>60</v>
       </c>
       <c r="K126" s="4" t="s">
         <v>132</v>
@@ -5347,10 +5359,10 @@
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="C127" s="15" t="s">
         <v>189</v>
@@ -5376,10 +5388,10 @@
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="C128" s="15" t="s">
         <v>189</v>
@@ -5388,12 +5400,15 @@
         <v>17</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H128" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J128" s="4">
+      <c r="J128" s="5">
         <v>80</v>
       </c>
       <c r="K128" s="4" t="s">
@@ -5402,60 +5417,51 @@
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>81</v>
+        <v>219</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E129" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F129" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G129" s="4" t="s">
-        <v>11</v>
+        <v>146</v>
       </c>
       <c r="H129" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J129" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K129" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L129" s="4" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="F130" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G130" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H130" s="13" t="s">
         <v>132</v>
@@ -5466,13 +5472,16 @@
       <c r="K130" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L130" s="4" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>189</v>
@@ -5487,7 +5496,7 @@
         <v>6</v>
       </c>
       <c r="G131" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
@@ -5501,16 +5510,16 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C132" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E132" s="4" t="s">
         <v>30</v>
@@ -5519,7 +5528,7 @@
         <v>6</v>
       </c>
       <c r="G132" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
@@ -5531,21 +5540,21 @@
         <v>132</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C133" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F133" s="4" t="s">
         <v>6</v>
@@ -5562,16 +5571,13 @@
       <c r="K133" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L133" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>189</v>
@@ -5580,13 +5586,13 @@
         <v>18</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G134" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H134" s="13" t="s">
         <v>132</v>
@@ -5597,13 +5603,16 @@
       <c r="K134" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L134" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C135" s="15" t="s">
         <v>189</v>
@@ -5612,13 +5621,13 @@
         <v>18</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G135" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
@@ -5630,24 +5639,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="136" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C136" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>55</v>
+        <v>251</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G136" s="4" t="s">
         <v>24</v>
@@ -5664,19 +5673,19 @@
     </row>
     <row r="137" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C137" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D137" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E137" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E137" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>6</v>
@@ -5694,27 +5703,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="C138" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>39</v>
+        <v>310</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>146</v>
+        <v>86</v>
       </c>
       <c r="F138" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G138" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H138" s="13" t="s">
         <v>132</v>
@@ -5725,28 +5734,25 @@
       <c r="K138" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L138" s="4" t="s">
-        <v>152</v>
-      </c>
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G139" s="4" t="s">
         <v>11</v>
@@ -5760,12 +5766,73 @@
       <c r="K139" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L139" s="4" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H140" s="13"/>
+      <c r="A140" s="4">
+        <v>88</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C140" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D140" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E140" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G140" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H140" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J140" s="4">
+        <v>99</v>
+      </c>
+      <c r="K140" s="4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H141" s="13"/>
+      <c r="A141" s="4">
+        <v>138</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C141" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D141" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E141" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F141" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G141" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H141" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J141" s="4">
+        <v>5</v>
+      </c>
+      <c r="K141" s="4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H142" s="13"/>
@@ -5800,7 +5867,7 @@
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <f>MAX(A1:A151)</f>
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B152" s="9" t="s">
         <v>95</v>
@@ -8494,7 +8561,7 @@
       <c r="H1047" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L139" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L140" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
         <filter val="1.2.4"/>
@@ -8506,10 +8573,10 @@
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L139">
-    <sortCondition ref="H2:H139"/>
-    <sortCondition ref="J2:J139"/>
-    <sortCondition ref="A2:A139"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L140">
+    <sortCondition ref="H2:H140"/>
+    <sortCondition ref="J2:J140"/>
+    <sortCondition ref="A2:A140"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add Aria support on main block on editor/js side
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E071E3-7028-4FBE-ADD3-FB44E7F87007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CDBF02-D1C9-42AB-998B-A005C82DF647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$141</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1501,7 +1501,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:O1047"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1559,7 +1558,7 @@
       <c r="N1" s="7"/>
       <c r="O1" s="8"/>
     </row>
-    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1588,7 +1587,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1620,7 +1619,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1652,7 +1651,7 @@
       </c>
       <c r="L4"/>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1684,7 +1683,7 @@
       </c>
       <c r="L5"/>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1716,7 +1715,7 @@
       </c>
       <c r="L6"/>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1748,7 +1747,7 @@
       </c>
       <c r="L7"/>
     </row>
-    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1780,7 +1779,7 @@
       </c>
       <c r="L8"/>
     </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1812,7 +1811,7 @@
       </c>
       <c r="L9"/>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1844,7 +1843,7 @@
       </c>
       <c r="L10"/>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1876,7 +1875,7 @@
       </c>
       <c r="L11"/>
     </row>
-    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1908,7 +1907,7 @@
       </c>
       <c r="L12"/>
     </row>
-    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1940,7 +1939,7 @@
       </c>
       <c r="L13"/>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1972,7 +1971,7 @@
       </c>
       <c r="L14"/>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2004,7 +2003,7 @@
       </c>
       <c r="L15"/>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2036,7 +2035,7 @@
       </c>
       <c r="L16"/>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2068,7 +2067,7 @@
       </c>
       <c r="L17"/>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2100,7 +2099,7 @@
       </c>
       <c r="L18"/>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2132,7 +2131,7 @@
       </c>
       <c r="L19"/>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2164,7 +2163,7 @@
       </c>
       <c r="L20"/>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2196,7 +2195,7 @@
       </c>
       <c r="L21"/>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2228,7 +2227,7 @@
       </c>
       <c r="L22"/>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2260,7 +2259,7 @@
       </c>
       <c r="L23"/>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2292,7 +2291,7 @@
       </c>
       <c r="L24"/>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2324,7 +2323,7 @@
       </c>
       <c r="L25"/>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2356,7 +2355,7 @@
       </c>
       <c r="L26"/>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2385,7 +2384,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2417,7 +2416,7 @@
       </c>
       <c r="L28"/>
     </row>
-    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2449,7 +2448,7 @@
       </c>
       <c r="L29"/>
     </row>
-    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -2478,7 +2477,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2510,7 +2509,7 @@
       </c>
       <c r="L31"/>
     </row>
-    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -2539,7 +2538,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>33</v>
       </c>
@@ -2571,7 +2570,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>34</v>
       </c>
@@ -2600,7 +2599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>37</v>
       </c>
@@ -2632,7 +2631,7 @@
       </c>
       <c r="L35"/>
     </row>
-    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>38</v>
       </c>
@@ -2661,7 +2660,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>40</v>
       </c>
@@ -2690,7 +2689,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>41</v>
       </c>
@@ -2720,7 +2719,7 @@
       </c>
       <c r="L38"/>
     </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>42</v>
       </c>
@@ -2752,7 +2751,7 @@
       </c>
       <c r="L39"/>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>44</v>
       </c>
@@ -2784,7 +2783,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>45</v>
       </c>
@@ -2813,7 +2812,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>46</v>
       </c>
@@ -2842,7 +2841,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" ht="120" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>47</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>48</v>
       </c>
@@ -2906,7 +2905,7 @@
       </c>
       <c r="L44"/>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>49</v>
       </c>
@@ -2935,7 +2934,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>50</v>
       </c>
@@ -2964,7 +2963,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>51</v>
       </c>
@@ -2996,7 +2995,7 @@
       </c>
       <c r="L47"/>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>57</v>
       </c>
@@ -3028,7 +3027,7 @@
       </c>
       <c r="L48"/>
     </row>
-    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>58</v>
       </c>
@@ -3057,7 +3056,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>59</v>
       </c>
@@ -3089,7 +3088,7 @@
       </c>
       <c r="L50"/>
     </row>
-    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>60</v>
       </c>
@@ -3118,7 +3117,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>62</v>
       </c>
@@ -3147,7 +3146,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>63</v>
       </c>
@@ -3177,7 +3176,7 @@
       </c>
       <c r="L53" s="6"/>
     </row>
-    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>66</v>
       </c>
@@ -3209,7 +3208,7 @@
       </c>
       <c r="L54"/>
     </row>
-    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>67</v>
       </c>
@@ -3238,7 +3237,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>69</v>
       </c>
@@ -3267,7 +3266,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>76</v>
       </c>
@@ -3296,7 +3295,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>76</v>
       </c>
@@ -3325,7 +3324,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>82</v>
       </c>
@@ -3355,7 +3354,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>83</v>
       </c>
@@ -3388,7 +3387,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>85</v>
       </c>
@@ -3418,7 +3417,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>32</v>
       </c>
@@ -3447,7 +3446,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>54</v>
       </c>
@@ -3473,7 +3472,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>61</v>
       </c>
@@ -3500,7 +3499,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>87</v>
       </c>
@@ -3527,7 +3526,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>89</v>
       </c>
@@ -3556,7 +3555,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>74</v>
       </c>
@@ -3583,7 +3582,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>91</v>
       </c>
@@ -3609,7 +3608,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>92</v>
       </c>
@@ -3636,7 +3635,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>68</v>
       </c>
@@ -3665,7 +3664,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>78</v>
       </c>
@@ -3695,7 +3694,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>93</v>
       </c>
@@ -3725,7 +3724,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>94</v>
       </c>
@@ -3755,7 +3754,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>98</v>
       </c>
@@ -3782,7 +3781,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>99</v>
       </c>
@@ -3814,7 +3813,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>90</v>
       </c>
@@ -3844,7 +3843,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>95</v>
       </c>
@@ -3874,7 +3873,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>96</v>
       </c>
@@ -3904,7 +3903,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>97</v>
       </c>
@@ -3937,7 +3936,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>109</v>
       </c>
@@ -3966,7 +3965,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>110</v>
       </c>
@@ -3995,7 +3994,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>111</v>
       </c>
@@ -4024,7 +4023,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>125</v>
       </c>
@@ -4053,7 +4052,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>128</v>
       </c>
@@ -4082,7 +4081,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>135</v>
       </c>
@@ -4267,22 +4266,22 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>262</v>
+        <v>309</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>17</v>
+        <v>310</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>7</v>
@@ -4290,16 +4289,19 @@
       <c r="H91" s="13" t="s">
         <v>307</v>
       </c>
+      <c r="J91" s="4">
+        <v>4</v>
+      </c>
       <c r="K91" s="4" t="s">
-        <v>26</v>
+        <v>256</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>56</v>
+        <v>134</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>214</v>
+        <v>262</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>190</v>
@@ -4311,36 +4313,36 @@
         <v>55</v>
       </c>
       <c r="F92" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G92" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H92" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J92" s="5">
-        <v>10</v>
+        <v>307</v>
       </c>
       <c r="K92" s="4" t="s">
-        <v>132</v>
+        <v>26</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>73</v>
+        <v>138</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>212</v>
+        <v>312</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>7</v>
@@ -4348,8 +4350,8 @@
       <c r="H93" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J93" s="5">
-        <v>10</v>
+      <c r="J93" s="4">
+        <v>5</v>
       </c>
       <c r="K93" s="4" t="s">
         <v>132</v>
@@ -4357,10 +4359,10 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>141</v>
+        <v>214</v>
       </c>
       <c r="C94" s="15" t="s">
         <v>190</v>
@@ -4369,17 +4371,14 @@
         <v>17</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H94" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I94" s="5">
-        <v>80</v>
-      </c>
       <c r="J94" s="5">
         <v>10</v>
       </c>
@@ -4387,12 +4386,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="95" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>258</v>
+        <v>212</v>
       </c>
       <c r="C95" s="15" t="s">
         <v>190</v>
@@ -4401,33 +4400,30 @@
         <v>17</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F95" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G95" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H95" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I95" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="J95" s="4">
+      <c r="J95" s="5">
         <v>10</v>
       </c>
       <c r="K95" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L95" s="4" t="s">
-        <v>259</v>
-      </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>216</v>
+        <v>141</v>
       </c>
       <c r="C96" s="15" t="s">
         <v>190</v>
@@ -4436,30 +4432,33 @@
         <v>17</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H96" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J96" s="4">
+      <c r="I96" s="5">
+        <v>80</v>
+      </c>
+      <c r="J96" s="5">
         <v>10</v>
       </c>
       <c r="K96" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>217</v>
+        <v>258</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>17</v>
@@ -4467,22 +4466,31 @@
       <c r="E97" s="4" t="s">
         <v>55</v>
       </c>
+      <c r="F97" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H97" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I97" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J97" s="4">
         <v>10</v>
       </c>
       <c r="K97" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L97" s="4" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="C98" s="15" t="s">
         <v>190</v>
@@ -4491,7 +4499,7 @@
         <v>17</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F98" s="4" t="s">
         <v>6</v>
@@ -4508,26 +4516,20 @@
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>243</v>
+        <v>217</v>
       </c>
       <c r="C99" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F99" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G99" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H99" s="13" t="s">
         <v>132</v>
       </c>
@@ -4540,25 +4542,22 @@
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>247</v>
+        <v>230</v>
       </c>
       <c r="C100" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E100" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G100" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H100" s="13" t="s">
         <v>132</v>
@@ -4569,16 +4568,13 @@
       <c r="K100" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L100" s="4" t="s">
-        <v>248</v>
-      </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C101" s="15" t="s">
         <v>190</v>
@@ -4590,7 +4586,7 @@
         <v>55</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>7</v>
@@ -4607,19 +4603,19 @@
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>309</v>
+        <v>247</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>310</v>
+        <v>18</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F102" s="4" t="s">
         <v>11</v>
@@ -4636,28 +4632,37 @@
       <c r="K102" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L102" s="4" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>228</v>
+        <v>249</v>
       </c>
       <c r="C103" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E103" s="4" t="s">
         <v>55</v>
       </c>
+      <c r="F103" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G103" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H103" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J103" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K103" s="4" t="s">
         <v>132</v>
@@ -4665,10 +4670,10 @@
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C104" s="15" t="s">
         <v>190</v>
@@ -4679,9 +4684,6 @@
       <c r="E104" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F104" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="H104" s="13" t="s">
         <v>132</v>
       </c>
@@ -4694,10 +4696,10 @@
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C105" s="15" t="s">
         <v>190</v>
@@ -4709,16 +4711,13 @@
         <v>55</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H105" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I105" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J105" s="5">
-        <v>20</v>
+      <c r="J105" s="4">
+        <v>15</v>
       </c>
       <c r="K105" s="4" t="s">
         <v>132</v>
@@ -4726,13 +4725,13 @@
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="C106" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>17</v>
@@ -4746,6 +4745,9 @@
       <c r="H106" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I106" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J106" s="5">
         <v>20</v>
       </c>
@@ -4755,27 +4757,27 @@
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="C107" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E107" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H107" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J107" s="4">
+      <c r="J107" s="5">
         <v>20</v>
       </c>
       <c r="K107" s="4" t="s">
@@ -4784,13 +4786,13 @@
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>18</v>
@@ -4799,10 +4801,7 @@
         <v>55</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G108" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H108" s="13" t="s">
         <v>132</v>
@@ -4813,28 +4812,25 @@
       <c r="K108" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L108" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>83</v>
+        <v>127</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>149</v>
+        <v>244</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E109" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G109" s="4" t="s">
         <v>24</v>
@@ -4843,21 +4839,24 @@
         <v>132</v>
       </c>
       <c r="J109" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K109" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L109" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D110" s="4" t="s">
         <v>17</v>
@@ -4866,7 +4865,10 @@
         <v>55</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G110" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H110" s="13" t="s">
         <v>132</v>
@@ -4880,24 +4882,21 @@
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G111" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
@@ -4912,21 +4911,24 @@
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C112" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E112" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F112" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G112" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H112" s="13" t="s">
@@ -4939,12 +4941,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="113" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>190</v>
@@ -4968,12 +4970,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>190</v>
@@ -4999,10 +5001,10 @@
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>190</v>
@@ -5011,16 +5013,16 @@
         <v>17</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H115" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J115" s="5">
-        <v>40</v>
+      <c r="J115" s="4">
+        <v>30</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>132</v>
@@ -5028,10 +5030,10 @@
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>190</v>
@@ -5040,18 +5042,15 @@
         <v>17</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H116" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I116" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J116" s="4">
+      <c r="J116" s="5">
         <v>40</v>
       </c>
       <c r="K116" s="4" t="s">
@@ -5060,29 +5059,29 @@
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G117" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H117" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I117" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J117" s="4">
         <v>40</v>
       </c>
@@ -5092,10 +5091,10 @@
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>189</v>
@@ -5122,12 +5121,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="119" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C119" s="15" t="s">
         <v>189</v>
@@ -5136,10 +5135,10 @@
         <v>17</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G119" s="4" t="s">
         <v>11</v>
@@ -5148,7 +5147,7 @@
         <v>132</v>
       </c>
       <c r="J119" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K119" s="4" t="s">
         <v>132</v>
@@ -5156,39 +5155,42 @@
     </row>
     <row r="120" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G120" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H120" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J120" s="5">
+      <c r="J120" s="4">
         <v>50</v>
       </c>
       <c r="K120" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>190</v>
@@ -5214,10 +5216,10 @@
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>190</v>
@@ -5226,15 +5228,15 @@
         <v>17</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H122" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J122" s="4">
+      <c r="J122" s="5">
         <v>50</v>
       </c>
       <c r="K122" s="4" t="s">
@@ -5243,10 +5245,10 @@
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>190</v>
@@ -5258,7 +5260,7 @@
         <v>55</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H123" s="13" t="s">
         <v>132</v>
@@ -5272,22 +5274,22 @@
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>233</v>
+        <v>220</v>
       </c>
       <c r="C124" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E124" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H124" s="13" t="s">
         <v>132</v>
@@ -5301,10 +5303,10 @@
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>189</v>
@@ -5330,28 +5332,28 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E126" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H126" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J126" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K126" s="4" t="s">
         <v>132</v>
@@ -5359,19 +5361,19 @@
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>25</v>
@@ -5379,8 +5381,8 @@
       <c r="H127" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J127" s="5">
-        <v>80</v>
+      <c r="J127" s="4">
+        <v>60</v>
       </c>
       <c r="K127" s="4" t="s">
         <v>132</v>
@@ -5388,10 +5390,10 @@
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="C128" s="15" t="s">
         <v>189</v>
@@ -5417,10 +5419,10 @@
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>189</v>
@@ -5429,12 +5431,15 @@
         <v>17</v>
       </c>
       <c r="E129" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F129" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H129" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J129" s="4">
+      <c r="J129" s="5">
         <v>80</v>
       </c>
       <c r="K129" s="4" t="s">
@@ -5443,60 +5448,51 @@
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>81</v>
+        <v>219</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F130" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G130" s="4" t="s">
-        <v>11</v>
+        <v>146</v>
       </c>
       <c r="H130" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J130" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K130" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L130" s="4" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="F131" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G131" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
@@ -5507,13 +5503,16 @@
       <c r="K131" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L131" s="4" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C132" s="15" t="s">
         <v>189</v>
@@ -5528,7 +5527,7 @@
         <v>6</v>
       </c>
       <c r="G132" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
@@ -5542,16 +5541,16 @@
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C133" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>30</v>
@@ -5560,7 +5559,7 @@
         <v>6</v>
       </c>
       <c r="G133" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
@@ -5572,21 +5571,21 @@
         <v>132</v>
       </c>
     </row>
-    <row r="134" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F134" s="4" t="s">
         <v>6</v>
@@ -5603,16 +5602,13 @@
       <c r="K134" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L134" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C135" s="15" t="s">
         <v>189</v>
@@ -5621,13 +5617,13 @@
         <v>18</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G135" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
@@ -5638,13 +5634,16 @@
       <c r="K135" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L135" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C136" s="15" t="s">
         <v>189</v>
@@ -5653,13 +5652,13 @@
         <v>18</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G136" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H136" s="13" t="s">
         <v>132</v>
@@ -5671,24 +5670,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="137" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C137" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D137" s="4" t="s">
-        <v>310</v>
+        <v>18</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>86</v>
+        <v>251</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G137" s="4" t="s">
         <v>24</v>
@@ -5705,10 +5704,10 @@
     </row>
     <row r="138" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C138" s="15" t="s">
         <v>189</v>
@@ -5735,27 +5734,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>39</v>
+        <v>310</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>146</v>
+        <v>86</v>
       </c>
       <c r="F139" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G139" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H139" s="13" t="s">
         <v>132</v>
@@ -5766,28 +5765,25 @@
       <c r="K139" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L139" s="4" t="s">
-        <v>152</v>
-      </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="C140" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G140" s="4" t="s">
         <v>11</v>
@@ -5801,34 +5797,37 @@
       <c r="K140" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L140" s="4" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>312</v>
+        <v>154</v>
       </c>
       <c r="C141" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D141" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E141" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G141" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H141" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J141" s="4">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="K141" s="4" t="s">
         <v>132</v>
@@ -8561,22 +8560,15 @@
       <c r="H1047" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L140" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="1.2.4"/>
-        <filter val="1.2.5"/>
-        <filter val="Roadmap"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="B1:L141" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L77">
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L140">
-    <sortCondition ref="H2:H140"/>
-    <sortCondition ref="J2:J140"/>
-    <sortCondition ref="A2:A140"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L141">
+    <sortCondition ref="H2:H141"/>
+    <sortCondition ref="J2:J141"/>
+    <sortCondition ref="A2:A141"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add support for accessibility narration
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CDBF02-D1C9-42AB-998B-A005C82DF647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8357564D-0375-4889-BFE1-4EE00AD258AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="316">
   <si>
     <t>Item</t>
   </si>
@@ -993,6 +993,15 @@
   </si>
   <si>
     <t>On Render, text color is same as banded row color</t>
+  </si>
+  <si>
+    <t>Accessibility</t>
+  </si>
+  <si>
+    <t>Add explicit header-to-cell association if needed</t>
+  </si>
+  <si>
+    <t>Likely front-end only.  Triggered by table complexity including sorting, filtering, etc.</t>
   </si>
 </sst>
 </file>
@@ -4278,7 +4287,7 @@
         <v>310</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>86</v>
+        <v>313</v>
       </c>
       <c r="F91" s="4" t="s">
         <v>11</v>
@@ -4289,11 +4298,8 @@
       <c r="H91" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="J91" s="4">
-        <v>4</v>
-      </c>
       <c r="K91" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
@@ -5050,6 +5056,9 @@
       <c r="H116" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I116" s="5">
+        <v>139</v>
+      </c>
       <c r="J116" s="5">
         <v>40</v>
       </c>
@@ -5833,8 +5842,40 @@
         <v>132</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H142" s="13"/>
+    <row r="142" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A142" s="4">
+        <v>139</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C142" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E142" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G142" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H142" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J142" s="4">
+        <v>99</v>
+      </c>
+      <c r="K142" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L142" s="4" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H143" s="13"/>
@@ -5866,7 +5907,7 @@
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <f>MAX(A1:A151)</f>
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B152" s="9" t="s">
         <v>95</v>

</xml_diff>

<commit_message>
Initial REST API for filtered, multi-table GET and attaching loaded tables
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08336E4E-1AFD-4E31-8D00-5C8ACB8E2185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{24E36E80-132B-4373-A848-F41FC3AA7986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$148</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1334" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="330">
   <si>
     <t>Item</t>
   </si>
@@ -817,9 +817,6 @@
   </si>
   <si>
     <t>Open</t>
-  </si>
-  <si>
-    <t>In prod, Table header was to be displayed by wasn't rendered. Refreshed post in edit and "display header" was cleared.  Re-applied the display and it worked.  Perhaps there is an issue on initial save?</t>
   </si>
   <si>
     <t>Add support for basic numberic content type</t>
@@ -1032,10 +1029,22 @@
     <t>Provide Copy/Paste support between cells</t>
   </si>
   <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>Still need to create serializer for formatted text output</t>
+    <t>1.3.2</t>
+  </si>
+  <si>
+    <t>In prod, Table header was to be displayed but wasn't rendered. Refreshed post in edit and "display header" was cleared.  Re-applied the display and it worked.  Perhaps there is an issue on initial save?</t>
+  </si>
+  <si>
+    <t>Enable endpoint to get multiple tables</t>
+  </si>
+  <si>
+    <t>Create a summary table store</t>
+  </si>
+  <si>
+    <t>Implement permissions outstanding</t>
+  </si>
+  <si>
+    <t>Update the UI to be more user friendly</t>
   </si>
 </sst>
 </file>
@@ -2896,7 +2905,7 @@
         <v>178</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>86</v>
@@ -3263,7 +3272,7 @@
         <v>178</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>86</v>
@@ -3292,7 +3301,7 @@
         <v>178</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>86</v>
@@ -3690,7 +3699,7 @@
         <v>189</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>86</v>
@@ -4101,7 +4110,7 @@
         <v>128</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>190</v>
@@ -4127,25 +4136,25 @@
     </row>
     <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="H85" s="13" t="s">
         <v>255</v>
@@ -4156,25 +4165,28 @@
     </row>
     <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C86" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E86" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="G86" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="H86" s="13" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="K86" s="4" t="s">
         <v>26</v>
@@ -4182,28 +4194,25 @@
     </row>
     <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G87" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H87" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="K87" s="4" t="s">
         <v>26</v>
@@ -4211,28 +4220,28 @@
     </row>
     <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>260</v>
+        <v>303</v>
       </c>
       <c r="C88" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H88" s="13" t="s">
-        <v>305</v>
+        <v>262</v>
       </c>
       <c r="K88" s="4" t="s">
         <v>26</v>
@@ -4240,141 +4249,138 @@
     </row>
     <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>307</v>
+        <v>259</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>308</v>
+        <v>17</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>311</v>
+        <v>55</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K89" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>39</v>
+        <v>307</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>86</v>
+        <v>310</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H90" s="13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K90" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>316</v>
+        <v>39</v>
       </c>
       <c r="E91" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F91" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G91" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G91" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="H91" s="13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K91" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L91" s="4" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>81</v>
+        <v>314</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>72</v>
+        <v>315</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>11</v>
+        <v>168</v>
       </c>
       <c r="H92" s="13" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="K92" s="4" t="s">
         <v>26</v>
       </c>
       <c r="L92" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="C93" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="F93" s="4" t="s">
         <v>6</v>
@@ -4383,24 +4389,27 @@
         <v>11</v>
       </c>
       <c r="H93" s="13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K93" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L93" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C94" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E94" s="4" t="s">
         <v>30</v>
@@ -4409,21 +4418,21 @@
         <v>6</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H94" s="13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K94" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>145</v>
+        <v>38</v>
       </c>
       <c r="C95" s="15" t="s">
         <v>189</v>
@@ -4432,112 +4441,100 @@
         <v>39</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>146</v>
+        <v>30</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G95" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H95" s="13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K95" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L95" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
-        <v>120</v>
+        <v>81</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>233</v>
+        <v>145</v>
       </c>
       <c r="C96" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>55</v>
+        <v>146</v>
       </c>
       <c r="F96" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G96" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="H96" s="13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K96" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L96" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>324</v>
+        <v>233</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E97" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H97" s="13" t="s">
-        <v>319</v>
-      </c>
-      <c r="I97" s="5">
-        <v>126</v>
-      </c>
-      <c r="J97" s="4">
-        <v>1</v>
+        <v>317</v>
       </c>
       <c r="K97" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="L97" s="4" t="s">
-        <v>326</v>
+        <v>26</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
-        <v>131</v>
+        <v>101</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>249</v>
+        <v>323</v>
       </c>
       <c r="C98" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G98" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H98" s="13" t="s">
-        <v>319</v>
-      </c>
-      <c r="J98" s="4">
-        <v>2</v>
+        <v>318</v>
       </c>
       <c r="K98" s="4" t="s">
         <v>26</v>
@@ -4566,10 +4563,7 @@
         <v>7</v>
       </c>
       <c r="H99" s="13" t="s">
-        <v>319</v>
-      </c>
-      <c r="J99" s="4">
-        <v>3</v>
+        <v>318</v>
       </c>
       <c r="K99" s="4" t="s">
         <v>26</v>
@@ -4577,10 +4571,10 @@
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C100" s="15" t="s">
         <v>190</v>
@@ -4598,24 +4592,18 @@
         <v>7</v>
       </c>
       <c r="H100" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="K100" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
         <v>132</v>
       </c>
-      <c r="J100" s="4">
-        <v>50</v>
-      </c>
-      <c r="K100" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="L100" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A101" s="4">
-        <v>124</v>
-      </c>
       <c r="B101" s="4" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="C101" s="15" t="s">
         <v>189</v>
@@ -4624,33 +4612,39 @@
         <v>39</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>86</v>
+        <v>254</v>
       </c>
       <c r="F101" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G101" s="4" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="H101" s="13" t="s">
-        <v>319</v>
+        <v>324</v>
+      </c>
+      <c r="J101" s="4">
+        <v>1</v>
       </c>
       <c r="K101" s="4" t="s">
         <v>256</v>
       </c>
+      <c r="L101" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E102" s="4" t="s">
         <v>86</v>
@@ -4662,68 +4656,71 @@
         <v>7</v>
       </c>
       <c r="H102" s="13" t="s">
-        <v>255</v>
+        <v>324</v>
+      </c>
+      <c r="J102" s="4">
+        <v>2</v>
       </c>
       <c r="K102" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="103" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>253</v>
+        <v>326</v>
       </c>
       <c r="C103" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>254</v>
+        <v>30</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G103" s="4" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="H103" s="13" t="s">
-        <v>319</v>
+        <v>324</v>
+      </c>
+      <c r="J103" s="4">
+        <v>3</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>256</v>
+        <v>155</v>
       </c>
       <c r="L103" s="4" t="s">
-        <v>257</v>
+        <v>328</v>
       </c>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>138</v>
+        <v>65</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>310</v>
+        <v>227</v>
       </c>
       <c r="C104" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G104" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H104" s="13" t="s">
-        <v>319</v>
+        <v>324</v>
+      </c>
+      <c r="J104" s="5">
+        <v>4</v>
       </c>
       <c r="K104" s="4" t="s">
         <v>256</v>
@@ -4731,10 +4728,10 @@
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="C105" s="15" t="s">
         <v>190</v>
@@ -4746,24 +4743,24 @@
         <v>55</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H105" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J105" s="5">
-        <v>10</v>
+        <v>324</v>
+      </c>
+      <c r="J105" s="4">
+        <v>5</v>
       </c>
       <c r="K105" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>73</v>
+        <v>116</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="C106" s="15" t="s">
         <v>190</v>
@@ -4772,30 +4769,24 @@
         <v>17</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F106" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G106" s="4" t="s">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="H106" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J106" s="5">
-        <v>10</v>
+        <v>324</v>
+      </c>
+      <c r="J106" s="4">
+        <v>6</v>
       </c>
       <c r="K106" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>77</v>
+        <v>119</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>141</v>
+        <v>231</v>
       </c>
       <c r="C107" s="15" t="s">
         <v>190</v>
@@ -4804,36 +4795,36 @@
         <v>17</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H107" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I107" s="5">
-        <v>80</v>
-      </c>
-      <c r="J107" s="5">
-        <v>10</v>
+        <v>324</v>
+      </c>
+      <c r="J107" s="4">
+        <v>7</v>
       </c>
       <c r="K107" s="4" t="s">
-        <v>132</v>
+        <v>155</v>
+      </c>
+      <c r="L107" s="4" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>104</v>
+        <v>138</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>216</v>
+        <v>309</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E108" s="4" t="s">
         <v>86</v>
@@ -4841,48 +4832,45 @@
       <c r="F108" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G108" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H108" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J108" s="4">
-        <v>10</v>
+        <v>324</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>132</v>
+        <v>26</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>217</v>
+        <v>327</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H109" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J109" s="4">
-        <v>10</v>
+        <v>324</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>132</v>
+        <v>26</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="C110" s="15" t="s">
         <v>190</v>
@@ -4894,12 +4882,12 @@
         <v>55</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H110" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J110" s="4">
+      <c r="J110" s="5">
         <v>10</v>
       </c>
       <c r="K110" s="4" t="s">
@@ -4908,10 +4896,10 @@
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>116</v>
+        <v>73</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="C111" s="15" t="s">
         <v>190</v>
@@ -4920,13 +4908,19 @@
         <v>17</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G111" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J111" s="4">
-        <v>15</v>
+      <c r="J111" s="5">
+        <v>10</v>
       </c>
       <c r="K111" s="4" t="s">
         <v>132</v>
@@ -4934,10 +4928,10 @@
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="C112" s="15" t="s">
         <v>190</v>
@@ -4946,16 +4940,19 @@
         <v>17</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H112" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J112" s="4">
-        <v>15</v>
+      <c r="I112" s="5">
+        <v>80</v>
+      </c>
+      <c r="J112" s="5">
+        <v>10</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>132</v>
@@ -4963,10 +4960,10 @@
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>65</v>
+        <v>104</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>190</v>
@@ -4975,19 +4972,16 @@
         <v>17</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H113" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I113" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J113" s="5">
-        <v>20</v>
+      <c r="J113" s="4">
+        <v>10</v>
       </c>
       <c r="K113" s="4" t="s">
         <v>132</v>
@@ -4995,10 +4989,10 @@
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>189</v>
@@ -5009,14 +5003,11 @@
       <c r="E114" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F114" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="H114" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J114" s="5">
-        <v>20</v>
+      <c r="J114" s="4">
+        <v>10</v>
       </c>
       <c r="K114" s="4" t="s">
         <v>132</v>
@@ -5024,27 +5015,27 @@
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E115" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H115" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J115" s="4">
+      <c r="J115" s="5">
         <v>20</v>
       </c>
       <c r="K115" s="4" t="s">
@@ -5053,13 +5044,13 @@
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C116" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>18</v>
@@ -5068,10 +5059,7 @@
         <v>55</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G116" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H116" s="13" t="s">
         <v>132</v>
@@ -5082,28 +5070,25 @@
       <c r="K116" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L116" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>83</v>
+        <v>127</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>149</v>
+        <v>244</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E117" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G117" s="4" t="s">
         <v>24</v>
@@ -5112,21 +5097,24 @@
         <v>132</v>
       </c>
       <c r="J117" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K117" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L117" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>17</v>
@@ -5135,7 +5123,10 @@
         <v>55</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G118" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H118" s="13" t="s">
         <v>132</v>
@@ -5149,24 +5140,21 @@
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G119" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H119" s="13" t="s">
@@ -5181,21 +5169,24 @@
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E120" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F120" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G120" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H120" s="13" t="s">
@@ -5208,12 +5199,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="121" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>190</v>
@@ -5237,12 +5228,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>190</v>
@@ -5268,10 +5259,10 @@
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>190</v>
@@ -5280,19 +5271,16 @@
         <v>17</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H123" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I123" s="5">
-        <v>139</v>
-      </c>
-      <c r="J123" s="5">
-        <v>40</v>
+      <c r="J123" s="4">
+        <v>30</v>
       </c>
       <c r="K123" s="4" t="s">
         <v>132</v>
@@ -5300,10 +5288,10 @@
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>190</v>
@@ -5312,18 +5300,18 @@
         <v>17</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H124" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I124" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J124" s="4">
+      <c r="I124" s="5">
+        <v>139</v>
+      </c>
+      <c r="J124" s="5">
         <v>40</v>
       </c>
       <c r="K124" s="4" t="s">
@@ -5332,29 +5320,29 @@
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G125" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H125" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I125" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J125" s="4">
         <v>40</v>
       </c>
@@ -5364,10 +5352,10 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C126" s="15" t="s">
         <v>189</v>
@@ -5394,12 +5382,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="127" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C127" s="15" t="s">
         <v>189</v>
@@ -5408,10 +5396,10 @@
         <v>17</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G127" s="4" t="s">
         <v>11</v>
@@ -5420,7 +5408,7 @@
         <v>132</v>
       </c>
       <c r="J127" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K127" s="4" t="s">
         <v>132</v>
@@ -5428,39 +5416,42 @@
     </row>
     <row r="128" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G128" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H128" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J128" s="5">
+      <c r="J128" s="4">
         <v>50</v>
       </c>
       <c r="K128" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>190</v>
@@ -5486,10 +5477,10 @@
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>190</v>
@@ -5498,15 +5489,15 @@
         <v>17</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H130" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J130" s="4">
+      <c r="J130" s="5">
         <v>50</v>
       </c>
       <c r="K130" s="4" t="s">
@@ -5515,10 +5506,10 @@
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>190</v>
@@ -5530,7 +5521,7 @@
         <v>55</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
@@ -5544,22 +5535,22 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="C132" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E132" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
@@ -5571,31 +5562,28 @@
         <v>132</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>323</v>
+        <v>234</v>
       </c>
       <c r="C133" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I133" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="J133" s="4">
         <v>50</v>
       </c>
@@ -5605,57 +5593,66 @@
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E134" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G134" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H134" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J134" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K134" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L134" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>133</v>
+        <v>322</v>
       </c>
       <c r="C135" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J135" s="5">
-        <v>80</v>
+      <c r="I135" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="J135" s="4">
+        <v>50</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>132</v>
@@ -5663,19 +5660,19 @@
     </row>
     <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>150</v>
+        <v>218</v>
       </c>
       <c r="C136" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D136" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F136" s="4" t="s">
         <v>25</v>
@@ -5683,8 +5680,8 @@
       <c r="H136" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J136" s="5">
-        <v>80</v>
+      <c r="J136" s="4">
+        <v>60</v>
       </c>
       <c r="K136" s="4" t="s">
         <v>132</v>
@@ -5692,10 +5689,10 @@
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>219</v>
+        <v>133</v>
       </c>
       <c r="C137" s="15" t="s">
         <v>189</v>
@@ -5704,12 +5701,15 @@
         <v>17</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H137" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J137" s="4">
+      <c r="J137" s="5">
         <v>80</v>
       </c>
       <c r="K137" s="4" t="s">
@@ -5718,77 +5718,65 @@
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>29</v>
+        <v>150</v>
       </c>
       <c r="C138" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>30</v>
+        <v>131</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G138" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H138" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J138" s="4">
-        <v>99</v>
+      <c r="J138" s="5">
+        <v>80</v>
       </c>
       <c r="K138" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="139" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>28</v>
+        <v>219</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F139" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G139" s="4" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="H139" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J139" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K139" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L139" s="4" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C140" s="15" t="s">
         <v>189</v>
@@ -5800,10 +5788,10 @@
         <v>30</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G140" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H140" s="13" t="s">
         <v>132</v>
@@ -5815,12 +5803,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C141" s="15" t="s">
         <v>189</v>
@@ -5829,10 +5817,10 @@
         <v>18</v>
       </c>
       <c r="E141" s="4" t="s">
-        <v>251</v>
+        <v>21</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G141" s="4" t="s">
         <v>24</v>
@@ -5846,28 +5834,31 @@
       <c r="K141" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="142" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L141" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>125</v>
+        <v>40</v>
       </c>
       <c r="C142" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>308</v>
+        <v>18</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G142" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
@@ -5879,24 +5870,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="143" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
       <c r="C143" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>308</v>
+        <v>18</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>86</v>
+        <v>251</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>24</v>
@@ -5911,27 +5902,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>154</v>
+        <v>125</v>
       </c>
       <c r="C144" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G144" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H144" s="13" t="s">
         <v>132</v>
@@ -5945,22 +5936,22 @@
     </row>
     <row r="145" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
-        <v>139</v>
+        <v>71</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>312</v>
+        <v>128</v>
       </c>
       <c r="C145" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D145" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>311</v>
+        <v>86</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G145" s="4" t="s">
         <v>24</v>
@@ -5974,28 +5965,25 @@
       <c r="K145" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L145" s="4" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="146" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
-        <v>142</v>
+        <v>88</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>320</v>
+        <v>154</v>
       </c>
       <c r="C146" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>321</v>
+        <v>131</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G146" s="4" t="s">
         <v>11</v>
@@ -6009,15 +5997,76 @@
       <c r="K146" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L146" s="4" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H147" s="13"/>
-    </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H148" s="13"/>
+    </row>
+    <row r="147" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A147" s="4">
+        <v>139</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C147" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D147" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E147" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G147" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H147" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J147" s="4">
+        <v>99</v>
+      </c>
+      <c r="K147" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L147" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A148" s="4">
+        <v>142</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C148" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D148" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E148" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G148" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H148" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J148" s="4">
+        <v>99</v>
+      </c>
+      <c r="K148" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L148" s="4" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H149" s="13"/>
@@ -6031,7 +6080,7 @@
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <f>MAX(A1:A151)</f>
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B152" s="9" t="s">
         <v>95</v>
@@ -8725,11 +8774,11 @@
       <c r="H1047" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L146" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L148" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
-        <filter val="1.3.0"/>
         <filter val="1.3.1"/>
+        <filter val="1.3.2"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>
@@ -8737,10 +8786,10 @@
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L146">
-    <sortCondition ref="H2:H146"/>
-    <sortCondition ref="J2:J146"/>
-    <sortCondition ref="A2:A146"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L148">
+    <sortCondition ref="H2:H148"/>
+    <sortCondition ref="J2:J148"/>
+    <sortCondition ref="A2:A148"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8912,7 +8961,7 @@
         <v>7</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>194</v>
@@ -8930,7 +8979,7 @@
         <v>176</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>190</v>
@@ -8985,23 +9034,23 @@
         <v>7</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E5" s="13"/>
       <c r="F5" s="23" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>203</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>190</v>
@@ -9013,7 +9062,7 @@
         <v>183</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
@@ -13675,112 +13724,112 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
       <c r="E2" s="29"/>
       <c r="F2" s="29"/>
       <c r="G2" s="21" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G4" t="s">
         <v>266</v>
       </c>
-      <c r="G4" t="s">
-        <v>267</v>
-      </c>
       <c r="H4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
+        <v>287</v>
+      </c>
+      <c r="G7" t="s">
         <v>288</v>
       </c>
-      <c r="G7" t="s">
-        <v>289</v>
-      </c>
       <c r="H7" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
+        <v>295</v>
+      </c>
+      <c r="G9" t="s">
         <v>296</v>
       </c>
-      <c r="G9" t="s">
-        <v>297</v>
-      </c>
       <c r="H9" s="22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J9" s="22"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I10" s="22"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I11" s="22"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I12" s="22"/>
     </row>
@@ -13810,165 +13859,165 @@
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
       <c r="E2" s="29"/>
       <c r="F2" s="29"/>
       <c r="G2" s="21" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G4" t="s">
         <v>266</v>
       </c>
-      <c r="G4" t="s">
-        <v>267</v>
-      </c>
       <c r="H4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
+        <v>292</v>
+      </c>
+      <c r="G11" t="s">
         <v>293</v>
       </c>
-      <c r="G11" t="s">
-        <v>294</v>
-      </c>
       <c r="H11" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
+        <v>295</v>
+      </c>
+      <c r="G13" t="s">
         <v>296</v>
       </c>
-      <c r="G13" t="s">
-        <v>297</v>
-      </c>
       <c r="H13" s="22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update documentation for new features
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{24E36E80-132B-4373-A848-F41FC3AA7986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21DD0F4E-2ED2-4B29-8C74-B70425C628CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1346" uniqueCount="329">
   <si>
     <t>Item</t>
   </si>
@@ -1029,9 +1029,6 @@
     <t>Provide Copy/Paste support between cells</t>
   </si>
   <si>
-    <t>1.3.2</t>
-  </si>
-  <si>
     <t>In prod, Table header was to be displayed but wasn't rendered. Refreshed post in edit and "display header" was cleared.  Re-applied the display and it worked.  Perhaps there is an issue on initial save?</t>
   </si>
   <si>
@@ -1041,10 +1038,10 @@
     <t>Create a summary table store</t>
   </si>
   <si>
-    <t>Implement permissions outstanding</t>
-  </si>
-  <si>
-    <t>Update the UI to be more user friendly</t>
+    <t>1.4.0</t>
+  </si>
+  <si>
+    <t>1.4.1</t>
   </si>
 </sst>
 </file>
@@ -4598,271 +4595,260 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
-        <v>132</v>
+        <v>65</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>253</v>
+        <v>227</v>
       </c>
       <c r="C101" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>254</v>
+        <v>55</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G101" s="4" t="s">
-        <v>168</v>
+        <v>25</v>
       </c>
       <c r="H101" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="J101" s="4">
-        <v>1</v>
-      </c>
+        <v>327</v>
+      </c>
+      <c r="J101" s="5"/>
       <c r="K101" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L101" s="4" t="s">
-        <v>325</v>
+        <v>26</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F102" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G102" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H102" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="J102" s="4">
-        <v>2</v>
+        <v>327</v>
       </c>
       <c r="K102" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>326</v>
+        <v>309</v>
       </c>
       <c r="C103" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="F103" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G103" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H103" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="J103" s="4">
-        <v>3</v>
+        <v>327</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="L103" s="4" t="s">
-        <v>328</v>
+        <v>26</v>
       </c>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>65</v>
+        <v>144</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>227</v>
+        <v>325</v>
       </c>
       <c r="C104" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H104" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="J104" s="5">
-        <v>4</v>
+        <v>327</v>
       </c>
       <c r="K104" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>118</v>
+        <v>145</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>230</v>
+        <v>326</v>
       </c>
       <c r="C105" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F105" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H105" s="13" t="s">
+        <v>327</v>
+      </c>
+      <c r="K105" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A106" s="4">
+        <v>132</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C106" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="F106" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H105" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="J105" s="4">
-        <v>5</v>
-      </c>
-      <c r="K105" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A106" s="4">
-        <v>116</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C106" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="D106" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E106" s="4" t="s">
-        <v>55</v>
+      <c r="G106" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="H106" s="13" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="J106" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K106" s="4" t="s">
         <v>256</v>
       </c>
+      <c r="L106" s="4" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="C107" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G107" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H107" s="13" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="J107" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K107" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="L107" s="4" t="s">
-        <v>329</v>
+        <v>256</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>309</v>
+        <v>230</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F108" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G108" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H108" s="13" t="s">
-        <v>324</v>
+        <v>328</v>
+      </c>
+      <c r="J108" s="4">
+        <v>3</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>26</v>
+        <v>256</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>145</v>
+        <v>116</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>327</v>
+        <v>228</v>
       </c>
       <c r="C109" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="H109" s="13" t="s">
-        <v>324</v>
+        <v>328</v>
+      </c>
+      <c r="J109" s="4">
+        <v>4</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>26</v>
+        <v>256</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
@@ -8778,7 +8764,8 @@
     <filterColumn colId="6">
       <filters>
         <filter val="1.3.1"/>
-        <filter val="1.3.2"/>
+        <filter val="1.4.0"/>
+        <filter val="1.4.1"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>

</xml_diff>

<commit_message>
Fix bugs saving new post and changing status in maintenance .
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21DD0F4E-2ED2-4B29-8C74-B70425C628CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE08882-DF59-4B9C-9CCD-2DDB1021949B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$149</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1346" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="333">
   <si>
     <t>Item</t>
   </si>
@@ -1042,6 +1042,18 @@
   </si>
   <si>
     <t>1.4.1</t>
+  </si>
+  <si>
+    <t>Support delete of table for unattached tables</t>
+  </si>
+  <si>
+    <t>In process</t>
+  </si>
+  <si>
+    <t>Create new table leaves it in New status and the Save button is gray</t>
+  </si>
+  <si>
+    <t>1.4.2</t>
   </si>
 </sst>
 </file>
@@ -1551,7 +1563,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:O1047"/>
+  <dimension ref="A1:O1059"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.42578125" style="4" customWidth="1"/>
@@ -4511,7 +4523,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
         <v>101</v>
       </c>
@@ -4537,7 +4549,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
         <v>126</v>
       </c>
@@ -4566,7 +4578,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>131</v>
       </c>
@@ -4795,10 +4807,10 @@
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>230</v>
+        <v>329</v>
       </c>
       <c r="C108" s="15" t="s">
         <v>190</v>
@@ -4819,15 +4831,15 @@
         <v>3</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C109" s="15" t="s">
         <v>190</v>
@@ -4848,15 +4860,15 @@
         <v>4</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>256</v>
+        <v>330</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>56</v>
+        <v>116</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="C110" s="15" t="s">
         <v>190</v>
@@ -4868,24 +4880,24 @@
         <v>55</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H110" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J110" s="5">
-        <v>10</v>
+        <v>328</v>
+      </c>
+      <c r="J110" s="4">
+        <v>5</v>
       </c>
       <c r="K110" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C111" s="15" t="s">
         <v>190</v>
@@ -4894,12 +4906,9 @@
         <v>17</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G111" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
@@ -4914,10 +4923,10 @@
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
       <c r="C112" s="15" t="s">
         <v>190</v>
@@ -4931,12 +4940,12 @@
       <c r="F112" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="G112" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H112" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I112" s="5">
-        <v>80</v>
-      </c>
       <c r="J112" s="5">
         <v>10</v>
       </c>
@@ -4946,10 +4955,10 @@
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>216</v>
+        <v>141</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>190</v>
@@ -4958,15 +4967,18 @@
         <v>17</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H113" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J113" s="4">
+      <c r="I113" s="5">
+        <v>80</v>
+      </c>
+      <c r="J113" s="5">
         <v>10</v>
       </c>
       <c r="K113" s="4" t="s">
@@ -4975,19 +4987,22 @@
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C114" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D114" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="H114" s="13" t="s">
         <v>132</v>
@@ -5001,10 +5016,10 @@
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>189</v>
@@ -5015,14 +5030,11 @@
       <c r="E115" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F115" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="H115" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J115" s="5">
-        <v>20</v>
+      <c r="J115" s="4">
+        <v>10</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>132</v>
@@ -5030,27 +5042,27 @@
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E116" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H116" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J116" s="4">
+      <c r="J116" s="5">
         <v>20</v>
       </c>
       <c r="K116" s="4" t="s">
@@ -5059,13 +5071,13 @@
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>18</v>
@@ -5074,10 +5086,7 @@
         <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G117" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H117" s="13" t="s">
         <v>132</v>
@@ -5088,28 +5097,25 @@
       <c r="K117" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L117" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>83</v>
+        <v>127</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>149</v>
+        <v>244</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E118" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G118" s="4" t="s">
         <v>24</v>
@@ -5118,21 +5124,24 @@
         <v>132</v>
       </c>
       <c r="J118" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K118" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L118" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>17</v>
@@ -5141,7 +5150,10 @@
         <v>55</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G119" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H119" s="13" t="s">
         <v>132</v>
@@ -5155,24 +5167,21 @@
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G120" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H120" s="13" t="s">
@@ -5187,21 +5196,24 @@
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C121" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E121" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F121" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G121" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H121" s="13" t="s">
@@ -5214,12 +5226,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="122" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>190</v>
@@ -5243,12 +5255,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>190</v>
@@ -5274,10 +5286,10 @@
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>190</v>
@@ -5286,19 +5298,16 @@
         <v>17</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H124" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I124" s="5">
-        <v>139</v>
-      </c>
-      <c r="J124" s="5">
-        <v>40</v>
+      <c r="J124" s="4">
+        <v>30</v>
       </c>
       <c r="K124" s="4" t="s">
         <v>132</v>
@@ -5306,10 +5315,10 @@
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>190</v>
@@ -5318,18 +5327,18 @@
         <v>17</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H125" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I125" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J125" s="4">
+      <c r="I125" s="5">
+        <v>139</v>
+      </c>
+      <c r="J125" s="5">
         <v>40</v>
       </c>
       <c r="K125" s="4" t="s">
@@ -5338,29 +5347,29 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G126" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H126" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I126" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J126" s="4">
         <v>40</v>
       </c>
@@ -5370,10 +5379,10 @@
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C127" s="15" t="s">
         <v>189</v>
@@ -5400,12 +5409,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C128" s="15" t="s">
         <v>189</v>
@@ -5414,10 +5423,10 @@
         <v>17</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G128" s="4" t="s">
         <v>11</v>
@@ -5426,7 +5435,7 @@
         <v>132</v>
       </c>
       <c r="J128" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K128" s="4" t="s">
         <v>132</v>
@@ -5434,39 +5443,42 @@
     </row>
     <row r="129" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C129" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E129" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G129" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H129" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J129" s="5">
+      <c r="J129" s="4">
         <v>50</v>
       </c>
       <c r="K129" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>190</v>
@@ -5492,10 +5504,10 @@
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>190</v>
@@ -5504,15 +5516,15 @@
         <v>17</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J131" s="4">
+      <c r="J131" s="5">
         <v>50</v>
       </c>
       <c r="K131" s="4" t="s">
@@ -5521,10 +5533,10 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C132" s="15" t="s">
         <v>190</v>
@@ -5536,7 +5548,7 @@
         <v>55</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
@@ -5550,22 +5562,22 @@
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="C133" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
@@ -5579,13 +5591,13 @@
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="C134" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D134" s="4" t="s">
         <v>18</v>
@@ -5594,10 +5606,7 @@
         <v>55</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G134" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H134" s="13" t="s">
         <v>132</v>
@@ -5608,48 +5617,48 @@
       <c r="K134" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L134" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="135" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>322</v>
+        <v>247</v>
       </c>
       <c r="C135" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E135" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F135" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G135" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I135" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="J135" s="4">
         <v>50</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L135" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>218</v>
+        <v>322</v>
       </c>
       <c r="C136" s="15" t="s">
         <v>190</v>
@@ -5661,13 +5670,16 @@
         <v>55</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H136" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I136" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J136" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K136" s="4" t="s">
         <v>132</v>
@@ -5675,19 +5687,19 @@
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="C137" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>25</v>
@@ -5695,8 +5707,8 @@
       <c r="H137" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J137" s="5">
-        <v>80</v>
+      <c r="J137" s="4">
+        <v>60</v>
       </c>
       <c r="K137" s="4" t="s">
         <v>132</v>
@@ -5704,10 +5716,10 @@
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="C138" s="15" t="s">
         <v>189</v>
@@ -5733,10 +5745,10 @@
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>189</v>
@@ -5745,12 +5757,15 @@
         <v>17</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H139" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J139" s="4">
+      <c r="J139" s="5">
         <v>80</v>
       </c>
       <c r="K139" s="4" t="s">
@@ -5759,42 +5774,36 @@
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>29</v>
+        <v>219</v>
       </c>
       <c r="C140" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F140" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G140" s="4" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="H140" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J140" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K140" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="141" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C141" s="15" t="s">
         <v>189</v>
@@ -5803,7 +5812,7 @@
         <v>18</v>
       </c>
       <c r="E141" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F141" s="4" t="s">
         <v>6</v>
@@ -5820,16 +5829,13 @@
       <c r="K141" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L141" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C142" s="15" t="s">
         <v>189</v>
@@ -5838,13 +5844,13 @@
         <v>18</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G142" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
@@ -5855,13 +5861,16 @@
       <c r="K142" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L142" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C143" s="15" t="s">
         <v>189</v>
@@ -5870,13 +5879,13 @@
         <v>18</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G143" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H143" s="13" t="s">
         <v>132</v>
@@ -5888,24 +5897,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="144" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C144" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>86</v>
+        <v>251</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G144" s="4" t="s">
         <v>24</v>
@@ -5922,10 +5931,10 @@
     </row>
     <row r="145" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C145" s="15" t="s">
         <v>189</v>
@@ -5952,27 +5961,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C146" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G146" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H146" s="13" t="s">
         <v>132</v>
@@ -5984,27 +5993,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="147" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
-        <v>139</v>
+        <v>88</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>311</v>
+        <v>154</v>
       </c>
       <c r="C147" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D147" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>310</v>
+        <v>131</v>
       </c>
       <c r="F147" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G147" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H147" s="13" t="s">
         <v>132</v>
@@ -6015,31 +6024,28 @@
       <c r="K147" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L147" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="148" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="C148" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="F148" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G148" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H148" s="13" t="s">
         <v>132</v>
@@ -6051,27 +6057,74 @@
         <v>132</v>
       </c>
       <c r="L148" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="149" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A149" s="4">
+        <v>142</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C149" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D149" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E149" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G149" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H149" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J149" s="4">
+        <v>99</v>
+      </c>
+      <c r="K149" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L149" s="4" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H149" s="13"/>
-    </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H150" s="13"/>
+    <row r="150" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A150" s="4">
+        <v>143</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="C150" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D150" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E150" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G150" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H150" s="13" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H151" s="13"/>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A152" s="9">
-        <f>MAX(A1:A151)</f>
-        <v>145</v>
-      </c>
-      <c r="B152" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C152" s="16"/>
       <c r="H152" s="13"/>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
@@ -6098,52 +6151,60 @@
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H160" s="13"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H161" s="13"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H162" s="13"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H163" s="13"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" s="9">
+        <f>MAX(A1:A163)</f>
+        <v>146</v>
+      </c>
+      <c r="B164" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C164" s="16"/>
       <c r="H164" s="13"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H165" s="13"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H166" s="13"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H167" s="13"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H168" s="13"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H169" s="13"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H170" s="13"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H171" s="13"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H172" s="13"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H173" s="13"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H174" s="13"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H175" s="13"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H176" s="13"/>
     </row>
     <row r="177" spans="8:8" x14ac:dyDescent="0.25">
@@ -8759,11 +8820,46 @@
     <row r="1047" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H1047" s="13"/>
     </row>
+    <row r="1048" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1048" s="13"/>
+    </row>
+    <row r="1049" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1049" s="13"/>
+    </row>
+    <row r="1050" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1050" s="13"/>
+    </row>
+    <row r="1051" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1051" s="13"/>
+    </row>
+    <row r="1052" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1052" s="13"/>
+    </row>
+    <row r="1053" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1053" s="13"/>
+    </row>
+    <row r="1054" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1054" s="13"/>
+    </row>
+    <row r="1055" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1055" s="13"/>
+    </row>
+    <row r="1056" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1056" s="13"/>
+    </row>
+    <row r="1057" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1057" s="13"/>
+    </row>
+    <row r="1058" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1058" s="13"/>
+    </row>
+    <row r="1059" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H1059" s="13"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B1:L148" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L149" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
-        <filter val="1.3.1"/>
         <filter val="1.4.0"/>
         <filter val="1.4.1"/>
         <filter val="Roadmap"/>
@@ -8773,10 +8869,10 @@
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L148">
-    <sortCondition ref="H2:H148"/>
-    <sortCondition ref="J2:J148"/>
-    <sortCondition ref="A2:A148"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L149">
+    <sortCondition ref="H2:H149"/>
+    <sortCondition ref="J2:J149"/>
+    <sortCondition ref="A2:A149"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Enable JSON Backup restoration
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE08882-DF59-4B9C-9CCD-2DDB1021949B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D04ED6-82F7-482B-8C40-2DE4AA6BCFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="333">
   <si>
     <t>Item</t>
   </si>
@@ -1047,13 +1047,13 @@
     <t>Support delete of table for unattached tables</t>
   </si>
   <si>
-    <t>In process</t>
-  </si>
-  <si>
-    <t>Create new table leaves it in New status and the Save button is gray</t>
-  </si>
-  <si>
     <t>1.4.2</t>
+  </si>
+  <si>
+    <t>Clone/Duplicate table from Maintenance Page</t>
+  </si>
+  <si>
+    <t>Coerce date and number formats from General format</t>
   </si>
 </sst>
 </file>
@@ -4607,7 +4607,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>65</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>119</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>138</v>
       </c>
@@ -4689,7 +4689,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>144</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>145</v>
       </c>
@@ -4738,79 +4738,64 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>253</v>
+        <v>230</v>
       </c>
       <c r="C106" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>254</v>
+        <v>55</v>
       </c>
       <c r="F106" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G106" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="H106" s="13" t="s">
         <v>328</v>
       </c>
-      <c r="J106" s="4">
-        <v>1</v>
-      </c>
       <c r="K106" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L106" s="4" t="s">
-        <v>324</v>
+        <v>26</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>239</v>
+        <v>329</v>
       </c>
       <c r="C107" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G107" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H107" s="13" t="s">
         <v>328</v>
       </c>
-      <c r="J107" s="4">
-        <v>2</v>
-      </c>
       <c r="K107" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>329</v>
+        <v>228</v>
       </c>
       <c r="C108" s="15" t="s">
         <v>190</v>
@@ -4825,21 +4810,21 @@
         <v>6</v>
       </c>
       <c r="H108" s="13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="J108" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>26</v>
+        <v>256</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>118</v>
+        <v>73</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="C109" s="15" t="s">
         <v>190</v>
@@ -4848,85 +4833,97 @@
         <v>17</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
+      </c>
+      <c r="G109" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H109" s="13" t="s">
-        <v>328</v>
-      </c>
-      <c r="J109" s="4">
-        <v>4</v>
+        <v>330</v>
+      </c>
+      <c r="J109" s="5">
+        <v>2</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>228</v>
+        <v>253</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>55</v>
+        <v>254</v>
       </c>
       <c r="F110" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G110" s="4" t="s">
+        <v>168</v>
+      </c>
       <c r="H110" s="13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="J110" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K110" s="4" t="s">
         <v>256</v>
       </c>
+      <c r="L110" s="4" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>214</v>
+        <v>239</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F111" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G111" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J111" s="5">
-        <v>10</v>
+        <v>330</v>
+      </c>
+      <c r="J111" s="4">
+        <v>4</v>
       </c>
       <c r="K111" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C112" s="15" t="s">
         <v>190</v>
@@ -4935,12 +4932,9 @@
         <v>17</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G112" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H112" s="13" t="s">
@@ -6095,7 +6089,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="150" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>143</v>
       </c>
@@ -6106,23 +6100,58 @@
         <v>189</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G150" s="4" t="s">
-        <v>168</v>
+        <v>11</v>
       </c>
       <c r="H150" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J150" s="4">
+        <v>10</v>
+      </c>
+      <c r="K150" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A151" s="4">
+        <v>144</v>
+      </c>
+      <c r="B151" s="4" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H151" s="13"/>
+      <c r="C151" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="D151" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E151" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G151" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H151" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J151" s="4">
+        <v>10</v>
+      </c>
+      <c r="K151" s="4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H152" s="13"/>
@@ -8860,8 +8889,8 @@
   <autoFilter ref="B1:L149" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
-        <filter val="1.4.0"/>
         <filter val="1.4.1"/>
+        <filter val="1.4.2"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>

</xml_diff>

<commit_message>
Initial configuration for checkbox column type
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D04ED6-82F7-482B-8C40-2DE4AA6BCFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3C98F1-94F6-442F-97B7-D916794EE455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
-    <sheet name="Data Types" sheetId="3" r:id="rId2"/>
-    <sheet name="date-time Data Shape" sheetId="5" r:id="rId3"/>
-    <sheet name="Number Data Shape" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
+    <sheet name="Features" sheetId="6" r:id="rId2"/>
+    <sheet name="Data Types" sheetId="3" r:id="rId3"/>
+    <sheet name="date-time Data Shape" sheetId="5" r:id="rId4"/>
+    <sheet name="Number Data Shape" sheetId="4" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$149</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1455" uniqueCount="380">
   <si>
     <t>Item</t>
   </si>
@@ -1054,6 +1055,147 @@
   </si>
   <si>
     <t>Coerce date and number formats from General format</t>
+  </si>
+  <si>
+    <t>1.4.3</t>
+  </si>
+  <si>
+    <t>Navigation &amp; Layout</t>
+  </si>
+  <si>
+    <t>Premium?</t>
+  </si>
+  <si>
+    <t>Insert Column</t>
+  </si>
+  <si>
+    <t>Move Column Left/Right</t>
+  </si>
+  <si>
+    <t>Insert Row</t>
+  </si>
+  <si>
+    <t>Delete Row</t>
+  </si>
+  <si>
+    <t>Move Row Up/Down</t>
+  </si>
+  <si>
+    <t>Delete Column</t>
+  </si>
+  <si>
+    <t>Set Column Width Dynamically</t>
+  </si>
+  <si>
+    <t>Banded Rows</t>
+  </si>
+  <si>
+    <t>Header Row</t>
+  </si>
+  <si>
+    <t>Sticky Header with vertical scrolling</t>
+  </si>
+  <si>
+    <t>Optional horizontal scroll</t>
+  </si>
+  <si>
+    <t>Paste limited to values within a column</t>
+  </si>
+  <si>
+    <t>Support paste from external sources</t>
+  </si>
+  <si>
+    <t>Multi-cell copy/paste</t>
+  </si>
+  <si>
+    <t>Enhanced copy/paste One Cell</t>
+  </si>
+  <si>
+    <t>Basic copy/paste one cell</t>
+  </si>
+  <si>
+    <t>Automatic data type conversion</t>
+  </si>
+  <si>
+    <t>Allow attempt to paste or conversion of existing data to a differents date type (e.g., general date to a data column type where interpretation is possible)</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>Formatting</t>
+  </si>
+  <si>
+    <t>Column Content Types (Basic)</t>
+  </si>
+  <si>
+    <t>Free-form data with formatting</t>
+  </si>
+  <si>
+    <t>Date, Time, or Date/Time</t>
+  </si>
+  <si>
+    <t>Decimal, Integer, Percent, Currency</t>
+  </si>
+  <si>
+    <t>Button</t>
+  </si>
+  <si>
+    <t>Table Types &amp; Creation Methods</t>
+  </si>
+  <si>
+    <t>New empty</t>
+  </si>
+  <si>
+    <t>Load from unattached table</t>
+  </si>
+  <si>
+    <t>Clone</t>
+  </si>
+  <si>
+    <t>Wordpress Patterns</t>
+  </si>
+  <si>
+    <t>Import CSV</t>
+  </si>
+  <si>
+    <t>Import/Restore Backup</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>Export Backup (JSON)</t>
+  </si>
+  <si>
+    <t>Export CVS</t>
+  </si>
+  <si>
+    <t>Creates unattached table available for loading to a block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optionally restores table or creates fully </t>
+  </si>
+  <si>
+    <t>Prompt/Lookup</t>
+  </si>
+  <si>
+    <t>Based on another table</t>
+  </si>
+  <si>
+    <t>Undo/Redo</t>
+  </si>
+  <si>
+    <t>External Data Source/API</t>
+  </si>
+  <si>
+    <t>Wordpress native content</t>
+  </si>
+  <si>
+    <t>Filtered list of posts, pages, custom post types, etc.</t>
+  </si>
+  <si>
+    <t>External Data Source/CSV File</t>
   </si>
 </sst>
 </file>
@@ -4812,11 +4954,8 @@
       <c r="H108" s="13" t="s">
         <v>330</v>
       </c>
-      <c r="J108" s="4">
-        <v>1</v>
-      </c>
       <c r="K108" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
@@ -4838,17 +4977,12 @@
       <c r="F109" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G109" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H109" s="13" t="s">
         <v>330</v>
       </c>
-      <c r="J109" s="5">
-        <v>2</v>
-      </c>
+      <c r="J109" s="5"/>
       <c r="K109" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="110" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -4874,10 +5008,10 @@
         <v>168</v>
       </c>
       <c r="H110" s="13" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="J110" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K110" s="4" t="s">
         <v>256</v>
@@ -4909,10 +5043,10 @@
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="J111" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K111" s="4" t="s">
         <v>256</v>
@@ -8909,6 +9043,370 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3791CA3F-8414-445D-AA49-2A38C1554C18}">
+  <dimension ref="B2:F52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="5.28515625" customWidth="1"/>
+    <col min="3" max="3" width="36.85546875" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="52.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D5" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>363</v>
+      </c>
+      <c r="D6" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D7" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>365</v>
+      </c>
+      <c r="D8" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>366</v>
+      </c>
+      <c r="D9" t="s">
+        <v>354</v>
+      </c>
+      <c r="F9" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>367</v>
+      </c>
+      <c r="D10" t="s">
+        <v>354</v>
+      </c>
+      <c r="F10" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>377</v>
+      </c>
+      <c r="F11" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>342</v>
+      </c>
+      <c r="D16" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>336</v>
+      </c>
+      <c r="D17" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>341</v>
+      </c>
+      <c r="D18" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>337</v>
+      </c>
+      <c r="D19" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>338</v>
+      </c>
+      <c r="D20" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>339</v>
+      </c>
+      <c r="D21" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>340</v>
+      </c>
+      <c r="D22" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>351</v>
+      </c>
+      <c r="D23" t="s">
+        <v>354</v>
+      </c>
+      <c r="F23" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>350</v>
+      </c>
+      <c r="D24" t="s">
+        <v>354</v>
+      </c>
+      <c r="F24" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>349</v>
+      </c>
+      <c r="D25" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D26" t="s">
+        <v>132</v>
+      </c>
+      <c r="F26" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>375</v>
+      </c>
+      <c r="D27" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>344</v>
+      </c>
+      <c r="D30" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>345</v>
+      </c>
+      <c r="D31" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>346</v>
+      </c>
+      <c r="D32" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>343</v>
+      </c>
+      <c r="D33" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>172</v>
+      </c>
+      <c r="D37" t="s">
+        <v>354</v>
+      </c>
+      <c r="F37" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" t="s">
+        <v>354</v>
+      </c>
+      <c r="F38" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>203</v>
+      </c>
+      <c r="D39" t="s">
+        <v>354</v>
+      </c>
+      <c r="F39" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>206</v>
+      </c>
+      <c r="D40" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>360</v>
+      </c>
+      <c r="D41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>202</v>
+      </c>
+      <c r="D42" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>201</v>
+      </c>
+      <c r="D43" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C44" t="s">
+        <v>200</v>
+      </c>
+      <c r="D44" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C47" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" t="s">
+        <v>132</v>
+      </c>
+      <c r="F47" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C51" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C52" t="s">
+        <v>370</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB00E3E-E598-4161-81A6-6FB0B476339E}">
   <dimension ref="A1:AS134"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13821,7 +14319,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C07A045-EDB0-4506-A2E7-225FA060F54C}">
   <dimension ref="B2:J13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13956,7 +14454,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F4CAB31-52FD-431F-AA77-05BD26AC0272}">
   <dimension ref="B2:I16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14140,7 +14638,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
   <dimension ref="B9:T43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add subscription for undo/redo
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6DEB44-02B9-4414-983C-59FAEE073F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C125EBE-741B-498C-9FCB-AFFE5C6EE3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -18,7 +18,8 @@
     <sheet name="Data Types" sheetId="3" r:id="rId3"/>
     <sheet name="date-time Data Shape" sheetId="5" r:id="rId4"/>
     <sheet name="Number Data Shape" sheetId="4" r:id="rId5"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId6"/>
+    <sheet name="Checkbox Data Shape" sheetId="7" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$152</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="387">
   <si>
     <t>Item</t>
   </si>
@@ -5042,47 +5043,38 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>253</v>
+        <v>216</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>254</v>
+        <v>86</v>
       </c>
       <c r="F111" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G111" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="H111" s="13" t="s">
         <v>386</v>
       </c>
-      <c r="J111" s="4">
-        <v>1</v>
-      </c>
       <c r="K111" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L111" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="C112" s="15" t="s">
         <v>189</v>
@@ -5091,59 +5083,65 @@
         <v>39</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>86</v>
+        <v>254</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G112" s="4" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="H112" s="13" t="s">
         <v>386</v>
       </c>
       <c r="J112" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>256</v>
       </c>
+      <c r="L112" s="4" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>214</v>
+        <v>239</v>
       </c>
       <c r="C113" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F113" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G113" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H113" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J113" s="5">
-        <v>10</v>
+        <v>386</v>
+      </c>
+      <c r="J113" s="4">
+        <v>2</v>
       </c>
       <c r="K113" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>141</v>
+        <v>214</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>190</v>
@@ -5152,30 +5150,27 @@
         <v>17</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H114" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I114" s="5">
-        <v>80</v>
+        <v>386</v>
       </c>
       <c r="J114" s="5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="K114" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>216</v>
+        <v>141</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>190</v>
@@ -5184,15 +5179,18 @@
         <v>17</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H115" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J115" s="4">
+      <c r="I115" s="5">
+        <v>80</v>
+      </c>
+      <c r="J115" s="5">
         <v>10</v>
       </c>
       <c r="K115" s="4" t="s">
@@ -9398,7 +9396,7 @@
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
-        <v>360</v>
+        <v>202</v>
       </c>
       <c r="D41" t="s">
         <v>132</v>
@@ -9406,7 +9404,7 @@
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D42" t="s">
         <v>132</v>
@@ -9414,7 +9412,7 @@
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C43" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D43" t="s">
         <v>132</v>
@@ -9422,7 +9420,7 @@
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C44" t="s">
-        <v>200</v>
+        <v>360</v>
       </c>
       <c r="D44" t="s">
         <v>132</v>
@@ -14717,6 +14715,193 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEDE6FBF-4912-4434-846B-E4148C1A58A6}">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="B2:I16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
+    <col min="2" max="5" width="3.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" customWidth="1"/>
+    <col min="9" max="9" width="68.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="29" t="s">
+        <v>276</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>264</v>
+      </c>
+      <c r="G3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G4" t="s">
+        <v>266</v>
+      </c>
+      <c r="H4" t="s">
+        <v>283</v>
+      </c>
+      <c r="I4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H6" t="s">
+        <v>283</v>
+      </c>
+      <c r="I6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>272</v>
+      </c>
+      <c r="G8" t="s">
+        <v>270</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>284</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>273</v>
+      </c>
+      <c r="G9" t="s">
+        <v>278</v>
+      </c>
+      <c r="H9" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="I9" s="22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>274</v>
+      </c>
+      <c r="G10" t="s">
+        <v>271</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="I10" s="22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>292</v>
+      </c>
+      <c r="G11" t="s">
+        <v>293</v>
+      </c>
+      <c r="H11" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="I11" s="22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>294</v>
+      </c>
+      <c r="G12" t="s">
+        <v>271</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="I12" s="22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>295</v>
+      </c>
+      <c r="G13" t="s">
+        <v>296</v>
+      </c>
+      <c r="H13" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="I13" s="22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>275</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
   <dimension ref="B9:T43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Fix checkbox config bug and prepare to publish 1.4.4
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C125EBE-741B-498C-9FCB-AFFE5C6EE3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61BEA4E-BD71-4401-BF2A-D18F0D3AAC95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1530" uniqueCount="390">
   <si>
     <t>Item</t>
   </si>
@@ -1224,6 +1224,15 @@
   </si>
   <si>
     <t>1.4.4</t>
+  </si>
+  <si>
+    <t>Fix bug preventing selection of hiding checkbox when no data is present</t>
+  </si>
+  <si>
+    <t>1.4.5</t>
+  </si>
+  <si>
+    <t>Hook into undo/redo subscription</t>
   </si>
 </sst>
 </file>
@@ -5092,7 +5101,7 @@
         <v>168</v>
       </c>
       <c r="H112" s="13" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="J112" s="4">
         <v>1</v>
@@ -5130,10 +5139,10 @@
         <v>386</v>
       </c>
       <c r="J113" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K113" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
@@ -5141,7 +5150,7 @@
         <v>56</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>214</v>
+        <v>389</v>
       </c>
       <c r="C114" s="15" t="s">
         <v>190</v>
@@ -5162,7 +5171,7 @@
         <v>3</v>
       </c>
       <c r="K114" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
@@ -6343,10 +6352,53 @@
       </c>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H153" s="13"/>
-    </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H154" s="13"/>
+      <c r="A153" s="4">
+        <v>146</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C153" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="D153" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E153" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F153" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H153" s="13" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A154" s="4">
+        <v>147</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="C154" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D154" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E154" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G154" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H154" s="13" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H155" s="13"/>
@@ -6378,7 +6430,7 @@
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <f>MAX(A1:A163)</f>
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B164" s="9" t="s">
         <v>95</v>

</xml_diff>

<commit_message>
Undo/redo batch caching and ignore capability
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FB4959-0C48-4AB2-8D00-9E3BDBA18FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8BF368-C62E-4CF3-AF3F-1E01915EFA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$155</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1532" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="393">
   <si>
     <t>Item</t>
   </si>
@@ -1233,6 +1233,15 @@
   </si>
   <si>
     <t>Hook into undo/redo subscription</t>
+  </si>
+  <si>
+    <t>Evaluate support for RTC syncConfig and determine if support can be safely added based on updates to WordPress.</t>
+  </si>
+  <si>
+    <t>1.4.6</t>
+  </si>
+  <si>
+    <t>Monitor ticket #80722</t>
   </si>
 </sst>
 </file>
@@ -5022,7 +5031,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>145</v>
       </c>
@@ -5134,47 +5143,41 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>253</v>
+        <v>214</v>
       </c>
       <c r="C114" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>254</v>
+        <v>55</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G114" s="4" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="H114" s="13" t="s">
         <v>388</v>
       </c>
       <c r="J114" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K114" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="L114" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>189</v>
@@ -5183,83 +5186,92 @@
         <v>39</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>86</v>
+        <v>254</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G115" s="4" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="H115" s="13" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="J115" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L115" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>214</v>
+        <v>390</v>
       </c>
       <c r="C116" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="E116" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F116" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G116" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H116" s="13" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="J116" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K116" s="4" t="s">
         <v>256</v>
       </c>
+      <c r="L116" s="4" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>77</v>
+        <v>124</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G117" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H117" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I117" s="5">
-        <v>80</v>
-      </c>
-      <c r="J117" s="5">
-        <v>10</v>
+        <v>391</v>
+      </c>
+      <c r="J117" s="4">
+        <v>3</v>
       </c>
       <c r="K117" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
@@ -5290,13 +5302,13 @@
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>17</v>
@@ -5308,7 +5320,7 @@
         <v>25</v>
       </c>
       <c r="G119" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H119" s="13" t="s">
         <v>132</v>
@@ -5322,10 +5334,10 @@
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>144</v>
+        <v>77</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>332</v>
+        <v>141</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>190</v>
@@ -5339,14 +5351,14 @@
       <c r="F120" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G120" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="H120" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J120" s="4">
-        <v>10</v>
+      <c r="I120" s="5">
+        <v>80</v>
+      </c>
+      <c r="J120" s="5">
+        <v>20</v>
       </c>
       <c r="K120" s="4" t="s">
         <v>132</v>
@@ -5447,10 +5459,10 @@
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>149</v>
+        <v>331</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>189</v>
@@ -5459,19 +5471,19 @@
         <v>17</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F124" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H124" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J124" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K124" s="4" t="s">
         <v>132</v>
@@ -5479,13 +5491,13 @@
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>17</v>
@@ -5494,7 +5506,10 @@
         <v>55</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G125" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H125" s="13" t="s">
         <v>132</v>
@@ -5508,24 +5523,21 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G126" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H126" s="13" t="s">
@@ -5540,21 +5552,24 @@
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E127" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F127" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G127" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H127" s="13" t="s">
@@ -5567,12 +5582,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C128" s="15" t="s">
         <v>190</v>
@@ -5596,12 +5611,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>190</v>
@@ -5627,10 +5642,10 @@
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>190</v>
@@ -5639,19 +5654,16 @@
         <v>17</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H130" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I130" s="5">
-        <v>139</v>
-      </c>
-      <c r="J130" s="5">
-        <v>40</v>
+      <c r="J130" s="4">
+        <v>30</v>
       </c>
       <c r="K130" s="4" t="s">
         <v>132</v>
@@ -5659,10 +5671,10 @@
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>190</v>
@@ -5671,18 +5683,18 @@
         <v>17</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I131" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J131" s="4">
+      <c r="I131" s="5">
+        <v>139</v>
+      </c>
+      <c r="J131" s="5">
         <v>40</v>
       </c>
       <c r="K131" s="4" t="s">
@@ -5691,29 +5703,29 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C132" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F132" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G132" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I132" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J132" s="4">
         <v>40</v>
       </c>
@@ -5723,10 +5735,10 @@
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C133" s="15" t="s">
         <v>189</v>
@@ -5753,12 +5765,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="134" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>189</v>
@@ -5767,10 +5779,10 @@
         <v>17</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G134" s="4" t="s">
         <v>11</v>
@@ -5779,7 +5791,7 @@
         <v>132</v>
       </c>
       <c r="J134" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K134" s="4" t="s">
         <v>132</v>
@@ -5787,39 +5799,42 @@
     </row>
     <row r="135" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C135" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G135" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J135" s="5">
+      <c r="J135" s="4">
         <v>50</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C136" s="15" t="s">
         <v>190</v>
@@ -5845,10 +5860,10 @@
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C137" s="15" t="s">
         <v>190</v>
@@ -5857,15 +5872,15 @@
         <v>17</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H137" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J137" s="4">
+      <c r="J137" s="5">
         <v>50</v>
       </c>
       <c r="K137" s="4" t="s">
@@ -5874,10 +5889,10 @@
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C138" s="15" t="s">
         <v>190</v>
@@ -5889,7 +5904,7 @@
         <v>55</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H138" s="13" t="s">
         <v>132</v>
@@ -5903,22 +5918,22 @@
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="C139" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E139" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H139" s="13" t="s">
         <v>132</v>
@@ -5932,13 +5947,13 @@
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="C140" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>18</v>
@@ -5947,10 +5962,7 @@
         <v>55</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G140" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H140" s="13" t="s">
         <v>132</v>
@@ -5961,48 +5973,48 @@
       <c r="K140" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L140" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="141" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>322</v>
+        <v>247</v>
       </c>
       <c r="C141" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D141" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E141" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F141" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G141" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H141" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I141" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="J141" s="4">
         <v>50</v>
       </c>
       <c r="K141" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L141" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>218</v>
+        <v>322</v>
       </c>
       <c r="C142" s="15" t="s">
         <v>190</v>
@@ -6014,13 +6026,16 @@
         <v>55</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I142" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J142" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K142" s="4" t="s">
         <v>132</v>
@@ -6028,19 +6043,19 @@
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="C143" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D143" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F143" s="4" t="s">
         <v>25</v>
@@ -6048,8 +6063,8 @@
       <c r="H143" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J143" s="5">
-        <v>80</v>
+      <c r="J143" s="4">
+        <v>60</v>
       </c>
       <c r="K143" s="4" t="s">
         <v>132</v>
@@ -6057,10 +6072,10 @@
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="C144" s="15" t="s">
         <v>189</v>
@@ -6086,10 +6101,10 @@
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="C145" s="15" t="s">
         <v>189</v>
@@ -6098,12 +6113,15 @@
         <v>17</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F145" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H145" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J145" s="4">
+      <c r="J145" s="5">
         <v>80</v>
       </c>
       <c r="K145" s="4" t="s">
@@ -6112,42 +6130,36 @@
     </row>
     <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>29</v>
+        <v>219</v>
       </c>
       <c r="C146" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F146" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G146" s="4" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="H146" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J146" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K146" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="147" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C147" s="15" t="s">
         <v>189</v>
@@ -6156,7 +6168,7 @@
         <v>18</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F147" s="4" t="s">
         <v>6</v>
@@ -6173,16 +6185,13 @@
       <c r="K147" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L147" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C148" s="15" t="s">
         <v>189</v>
@@ -6191,13 +6200,13 @@
         <v>18</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F148" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G148" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H148" s="13" t="s">
         <v>132</v>
@@ -6208,13 +6217,16 @@
       <c r="K148" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L148" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C149" s="15" t="s">
         <v>189</v>
@@ -6223,13 +6235,13 @@
         <v>18</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F149" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G149" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H149" s="13" t="s">
         <v>132</v>
@@ -6241,24 +6253,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="150" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C150" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>86</v>
+        <v>251</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G150" s="4" t="s">
         <v>24</v>
@@ -6275,10 +6287,10 @@
     </row>
     <row r="151" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C151" s="15" t="s">
         <v>189</v>
@@ -6305,27 +6317,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C152" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F152" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G152" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H152" s="13" t="s">
         <v>132</v>
@@ -6337,27 +6349,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="153" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" s="4">
-        <v>139</v>
+        <v>88</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>311</v>
+        <v>154</v>
       </c>
       <c r="C153" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>310</v>
+        <v>131</v>
       </c>
       <c r="F153" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G153" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H153" s="13" t="s">
         <v>132</v>
@@ -6368,31 +6380,28 @@
       <c r="K153" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L153" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="154" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="154" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A154" s="4">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="C154" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G154" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H154" s="13" t="s">
         <v>132</v>
@@ -6404,11 +6413,43 @@
         <v>132</v>
       </c>
       <c r="L154" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A155" s="4">
+        <v>142</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C155" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D155" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E155" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F155" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H155" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J155" s="4">
+        <v>99</v>
+      </c>
+      <c r="K155" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L155" s="4" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H155" s="13"/>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H156" s="13"/>
@@ -6437,7 +6478,7 @@
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <f>MAX(A1:A163)</f>
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B164" s="9" t="s">
         <v>95</v>
@@ -9131,12 +9172,12 @@
       <c r="H1059" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L154" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L155" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
-        <filter val="1.4.3"/>
         <filter val="1.4.4"/>
         <filter val="1.4.5"/>
+        <filter val="1.4.6"/>
         <filter val="Roadmap"/>
       </filters>
     </filterColumn>
@@ -9144,10 +9185,10 @@
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L154">
-    <sortCondition ref="H2:H154"/>
-    <sortCondition ref="J2:J154"/>
-    <sortCondition ref="A2:A154"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L155">
+    <sortCondition ref="H2:H155"/>
+    <sortCondition ref="J2:J155"/>
+    <sortCondition ref="A2:A155"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Initial Foundation for Advanced Edit and link data type
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8BF368-C62E-4CF3-AF3F-1E01915EFA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CAF086-0D8B-443F-9AF3-27064C715C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$156</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="394">
   <si>
     <t>Item</t>
   </si>
@@ -1242,6 +1242,9 @@
   </si>
   <si>
     <t>Monitor ticket #80722</t>
+  </si>
+  <si>
+    <t>Prevent new tables (attached) from going into the undo queue</t>
   </si>
 </sst>
 </file>
@@ -5165,11 +5168,8 @@
       <c r="H114" s="13" t="s">
         <v>388</v>
       </c>
-      <c r="J114" s="4">
-        <v>3</v>
-      </c>
       <c r="K114" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="115" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -5207,21 +5207,21 @@
         <v>324</v>
       </c>
     </row>
-    <row r="116" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>55</v>
+        <v>254</v>
       </c>
       <c r="F116" s="4" t="s">
         <v>6</v>
@@ -5238,25 +5238,22 @@
       <c r="K116" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="L116" s="4" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>239</v>
+        <v>390</v>
       </c>
       <c r="C117" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>6</v>
@@ -5273,54 +5270,57 @@
       <c r="K117" s="4" t="s">
         <v>256</v>
       </c>
+      <c r="L117" s="4" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G118" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H118" s="13" t="s">
-        <v>132</v>
+        <v>391</v>
       </c>
       <c r="J118" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K118" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>332</v>
+        <v>217</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F119" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G119" s="4" t="s">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="H119" s="13" t="s">
         <v>132</v>
@@ -5334,10 +5334,10 @@
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>77</v>
+        <v>144</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>141</v>
+        <v>332</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>190</v>
@@ -5351,14 +5351,14 @@
       <c r="F120" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="G120" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="H120" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I120" s="5">
-        <v>80</v>
-      </c>
-      <c r="J120" s="5">
-        <v>20</v>
+      <c r="J120" s="4">
+        <v>10</v>
       </c>
       <c r="K120" s="4" t="s">
         <v>132</v>
@@ -5366,19 +5366,19 @@
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="C121" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>25</v>
@@ -5386,6 +5386,9 @@
       <c r="H121" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I121" s="5">
+        <v>80</v>
+      </c>
       <c r="J121" s="5">
         <v>20</v>
       </c>
@@ -5395,27 +5398,27 @@
     </row>
     <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E122" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H122" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J122" s="4">
+      <c r="J122" s="5">
         <v>20</v>
       </c>
       <c r="K122" s="4" t="s">
@@ -5424,13 +5427,13 @@
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C123" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>18</v>
@@ -5439,10 +5442,7 @@
         <v>55</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G123" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H123" s="13" t="s">
         <v>132</v>
@@ -5453,31 +5453,28 @@
       <c r="K123" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L123" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>331</v>
+        <v>244</v>
       </c>
       <c r="C124" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H124" s="13" t="s">
         <v>132</v>
@@ -5488,13 +5485,16 @@
       <c r="K124" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L124" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>149</v>
+        <v>331</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>189</v>
@@ -5503,19 +5503,19 @@
         <v>17</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G125" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H125" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J125" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K125" s="4" t="s">
         <v>132</v>
@@ -5523,13 +5523,13 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>17</v>
@@ -5538,7 +5538,10 @@
         <v>55</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G126" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H126" s="13" t="s">
         <v>132</v>
@@ -5552,24 +5555,21 @@
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G127" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H127" s="13" t="s">
@@ -5584,21 +5584,24 @@
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E128" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F128" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G128" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H128" s="13" t="s">
@@ -5611,12 +5614,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="129" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>190</v>
@@ -5640,12 +5643,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>190</v>
@@ -5671,10 +5674,10 @@
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>190</v>
@@ -5683,19 +5686,16 @@
         <v>17</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I131" s="5">
-        <v>139</v>
-      </c>
-      <c r="J131" s="5">
-        <v>40</v>
+      <c r="J131" s="4">
+        <v>30</v>
       </c>
       <c r="K131" s="4" t="s">
         <v>132</v>
@@ -5703,10 +5703,10 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>229</v>
+        <v>142</v>
       </c>
       <c r="C132" s="15" t="s">
         <v>190</v>
@@ -5715,18 +5715,18 @@
         <v>17</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I132" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J132" s="4">
+      <c r="I132" s="5">
+        <v>139</v>
+      </c>
+      <c r="J132" s="5">
         <v>40</v>
       </c>
       <c r="K132" s="4" t="s">
@@ -5735,29 +5735,29 @@
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C133" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D133" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F133" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G133" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I133" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J133" s="4">
         <v>40</v>
       </c>
@@ -5767,10 +5767,10 @@
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>189</v>
@@ -5797,12 +5797,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="135" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C135" s="15" t="s">
         <v>189</v>
@@ -5811,10 +5811,10 @@
         <v>17</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G135" s="4" t="s">
         <v>11</v>
@@ -5823,7 +5823,7 @@
         <v>132</v>
       </c>
       <c r="J135" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>132</v>
@@ -5831,39 +5831,42 @@
     </row>
     <row r="136" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C136" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D136" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G136" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H136" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J136" s="5">
+      <c r="J136" s="4">
         <v>50</v>
       </c>
       <c r="K136" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C137" s="15" t="s">
         <v>190</v>
@@ -5889,10 +5892,10 @@
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
       <c r="C138" s="15" t="s">
         <v>190</v>
@@ -5901,15 +5904,15 @@
         <v>17</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H138" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J138" s="4">
+      <c r="J138" s="5">
         <v>50</v>
       </c>
       <c r="K138" s="4" t="s">
@@ -5918,10 +5921,10 @@
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>190</v>
@@ -5933,7 +5936,7 @@
         <v>55</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H139" s="13" t="s">
         <v>132</v>
@@ -5947,22 +5950,22 @@
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="C140" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E140" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H140" s="13" t="s">
         <v>132</v>
@@ -5976,13 +5979,13 @@
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="C141" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>18</v>
@@ -5991,10 +5994,7 @@
         <v>55</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G141" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H141" s="13" t="s">
         <v>132</v>
@@ -6005,48 +6005,48 @@
       <c r="K141" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L141" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="142" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>322</v>
+        <v>247</v>
       </c>
       <c r="C142" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E142" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F142" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G142" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I142" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="J142" s="4">
         <v>50</v>
       </c>
       <c r="K142" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L142" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>218</v>
+        <v>322</v>
       </c>
       <c r="C143" s="15" t="s">
         <v>190</v>
@@ -6058,13 +6058,16 @@
         <v>55</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H143" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I143" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J143" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K143" s="4" t="s">
         <v>132</v>
@@ -6072,19 +6075,19 @@
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="C144" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D144" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F144" s="4" t="s">
         <v>25</v>
@@ -6092,8 +6095,8 @@
       <c r="H144" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J144" s="5">
-        <v>80</v>
+      <c r="J144" s="4">
+        <v>60</v>
       </c>
       <c r="K144" s="4" t="s">
         <v>132</v>
@@ -6101,10 +6104,10 @@
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="C145" s="15" t="s">
         <v>189</v>
@@ -6130,10 +6133,10 @@
     </row>
     <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="C146" s="15" t="s">
         <v>189</v>
@@ -6142,12 +6145,15 @@
         <v>17</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H146" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J146" s="4">
+      <c r="J146" s="5">
         <v>80</v>
       </c>
       <c r="K146" s="4" t="s">
@@ -6156,42 +6162,36 @@
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>29</v>
+        <v>219</v>
       </c>
       <c r="C147" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D147" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F147" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G147" s="4" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="H147" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J147" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K147" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="148" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C148" s="15" t="s">
         <v>189</v>
@@ -6200,7 +6200,7 @@
         <v>18</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F148" s="4" t="s">
         <v>6</v>
@@ -6217,16 +6217,13 @@
       <c r="K148" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L148" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C149" s="15" t="s">
         <v>189</v>
@@ -6235,13 +6232,13 @@
         <v>18</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F149" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G149" s="4" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="H149" s="13" t="s">
         <v>132</v>
@@ -6252,13 +6249,16 @@
       <c r="K149" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L149" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C150" s="15" t="s">
         <v>189</v>
@@ -6267,13 +6267,13 @@
         <v>18</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G150" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H150" s="13" t="s">
         <v>132</v>
@@ -6285,24 +6285,24 @@
         <v>132</v>
       </c>
     </row>
-    <row r="151" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C151" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E151" s="4" t="s">
-        <v>86</v>
+        <v>251</v>
       </c>
       <c r="F151" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G151" s="4" t="s">
         <v>24</v>
@@ -6319,10 +6319,10 @@
     </row>
     <row r="152" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C152" s="15" t="s">
         <v>189</v>
@@ -6349,27 +6349,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A153" s="4">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C153" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F153" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G153" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H153" s="13" t="s">
         <v>132</v>
@@ -6381,27 +6381,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="154" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" s="4">
-        <v>139</v>
+        <v>88</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>311</v>
+        <v>154</v>
       </c>
       <c r="C154" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>310</v>
+        <v>131</v>
       </c>
       <c r="F154" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G154" s="4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H154" s="13" t="s">
         <v>132</v>
@@ -6412,31 +6412,28 @@
       <c r="K154" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L154" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="155" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A155" s="4">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="C155" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D155" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E155" s="4" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="F155" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G155" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H155" s="13" t="s">
         <v>132</v>
@@ -6448,11 +6445,43 @@
         <v>132</v>
       </c>
       <c r="L155" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A156" s="4">
+        <v>142</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C156" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D156" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E156" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G156" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H156" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J156" s="4">
+        <v>99</v>
+      </c>
+      <c r="K156" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L156" s="4" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H156" s="13"/>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H157" s="13"/>
@@ -6478,7 +6507,7 @@
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <f>MAX(A1:A163)</f>
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B164" s="9" t="s">
         <v>95</v>
@@ -9172,7 +9201,7 @@
       <c r="H1059" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L155" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L156" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <filterColumn colId="6">
       <filters>
         <filter val="1.4.4"/>
@@ -9185,10 +9214,10 @@
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L155">
-    <sortCondition ref="H2:H155"/>
-    <sortCondition ref="J2:J155"/>
-    <sortCondition ref="A2:A155"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L156">
+    <sortCondition ref="H2:H156"/>
+    <sortCondition ref="J2:J156"/>
+    <sortCondition ref="A2:A156"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Initial editor config for link content type
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CAF086-0D8B-443F-9AF3-27064C715C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B51BDC-1FF8-4C88-9619-6AFCAD55EFB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="1" activeTab="6" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="date-time Data Shape" sheetId="5" r:id="rId4"/>
     <sheet name="Number Data Shape" sheetId="4" r:id="rId5"/>
     <sheet name="Checkbox Data Shape" sheetId="7" r:id="rId6"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId7"/>
+    <sheet name="Link Data Shape" sheetId="8" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$156</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1619" uniqueCount="422">
   <si>
     <t>Item</t>
   </si>
@@ -1245,6 +1246,90 @@
   </si>
   <si>
     <t>Prevent new tables (attached) from going into the undo queue</t>
+  </si>
+  <si>
+    <t>Column Type Definition:</t>
+  </si>
+  <si>
+    <t>Cell Content Definition:</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>attributes.value {</t>
+  </si>
+  <si>
+    <t>canonical {</t>
+  </si>
+  <si>
+    <t>refs {</t>
+  </si>
+  <si>
+    <t>indexText</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>any well formed url</t>
+  </si>
+  <si>
+    <t>icon</t>
+  </si>
+  <si>
+    <t>iconLabel</t>
+  </si>
+  <si>
+    <t>iconApped {</t>
+  </si>
+  <si>
+    <t>position</t>
+  </si>
+  <si>
+    <t>ChatGPT Proposed Value Shapes</t>
+  </si>
+  <si>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>attributes.value</t>
+  </si>
+  <si>
+    <t>{ "type": "richtext", "raw": "&lt;p&gt;Hello &lt;strong&gt;world&lt;/strong&gt;&lt;/p&gt;" }</t>
+  </si>
+  <si>
+    <t>attributes.indexText</t>
+  </si>
+  <si>
+    <t>{ "type": "url", "href": "https://example.com", "label": "Docs" }</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>{ "type": "media", "id": 123, "mime": "image/jpeg", "size": "medium" }</t>
+  </si>
+  <si>
+    <t>{ "type": "post", "id": 456, "postType": "page" }</t>
+  </si>
+  <si>
+    <t>{ "type": "attachment", "id": 123 }</t>
+  </si>
+  <si>
+    <t>{ "type": "post", "id": 456 }</t>
+  </si>
+  <si>
+    <t>attributes.refs</t>
+  </si>
+  <si>
+    <t>type</t>
   </si>
 </sst>
 </file>
@@ -1355,7 +1440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1434,6 +1519,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9420,21 +9509,21 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
-        <v>352</v>
+        <v>375</v>
       </c>
       <c r="D26" t="s">
-        <v>132</v>
-      </c>
-      <c r="F26" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
-        <v>375</v>
+        <v>352</v>
       </c>
       <c r="D27" t="s">
         <v>132</v>
+      </c>
+      <c r="F27" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -9571,19 +9660,25 @@
         <v>374</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C51" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D51" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C52" t="s">
         <v>370</v>
+      </c>
+      <c r="D52" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -10525,16 +10620,21 @@
       <c r="AS17" s="11"/>
     </row>
     <row r="18" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
+      <c r="A18" s="31" t="s">
+        <v>409</v>
+      </c>
       <c r="B18" s="4"/>
       <c r="C18" s="15"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="14"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
+      <c r="G18" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>410</v>
+      </c>
       <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
@@ -10574,14 +10674,17 @@
     <row r="19" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
-      <c r="C19" s="15"/>
+      <c r="C19" s="4"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="14"/>
       <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
+      <c r="H19" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="I19" t="s">
+        <v>412</v>
+      </c>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -10626,7 +10729,9 @@
       <c r="E20" s="13"/>
       <c r="F20" s="14"/>
       <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="H20" s="11" t="s">
+        <v>420</v>
+      </c>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
@@ -10673,7 +10778,9 @@
       <c r="E21" s="13"/>
       <c r="F21" s="14"/>
       <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
+      <c r="H21" s="11" t="s">
+        <v>413</v>
+      </c>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
@@ -10766,10 +10873,12 @@
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="14"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
+      <c r="G23" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>410</v>
+      </c>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -10814,9 +10923,12 @@
       <c r="E24" s="13"/>
       <c r="F24" s="14"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
+      <c r="H24" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="I24" t="s">
+        <v>414</v>
+      </c>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -10861,7 +10973,9 @@
       <c r="E25" s="13"/>
       <c r="F25" s="14"/>
       <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
+      <c r="H25" s="11" t="s">
+        <v>420</v>
+      </c>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
@@ -10908,7 +11022,9 @@
       <c r="E26" s="15"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+      <c r="H26" s="11" t="s">
+        <v>413</v>
+      </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
@@ -11001,8 +11117,12 @@
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
       <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
+      <c r="G28" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>410</v>
+      </c>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
@@ -11049,9 +11169,12 @@
       <c r="E29" s="15"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
+      <c r="H29" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="I29" t="s">
+        <v>416</v>
+      </c>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
@@ -11096,8 +11219,12 @@
       <c r="E30" s="15"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
+      <c r="H30" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="I30" t="s">
+        <v>418</v>
+      </c>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
@@ -11143,7 +11270,9 @@
       <c r="E31" s="15"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
+      <c r="H31" s="11" t="s">
+        <v>413</v>
+      </c>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
@@ -11236,8 +11365,12 @@
       <c r="D33" s="15"/>
       <c r="E33" s="15"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
+      <c r="G33" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>410</v>
+      </c>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
@@ -11284,9 +11417,12 @@
       <c r="E34" s="15"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
+      <c r="H34" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="I34" t="s">
+        <v>417</v>
+      </c>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -11331,8 +11467,12 @@
       <c r="E35" s="15"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
+      <c r="H35" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="I35" t="s">
+        <v>419</v>
+      </c>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
@@ -11378,7 +11518,9 @@
       <c r="E36" s="15"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
+      <c r="H36" s="11" t="s">
+        <v>413</v>
+      </c>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
@@ -14526,7 +14668,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C07A045-EDB0-4506-A2E7-225FA060F54C}">
-  <dimension ref="B2:J13"/>
+  <dimension ref="B2:J15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
@@ -14556,100 +14698,110 @@
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="B3" s="30" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>264</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G4" t="s">
         <v>263</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>265</v>
-      </c>
-      <c r="G4" t="s">
-        <v>266</v>
-      </c>
-      <c r="H4" t="s">
-        <v>280</v>
-      </c>
-      <c r="I4" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G5" t="s">
+        <v>266</v>
+      </c>
+      <c r="H5" t="s">
+        <v>280</v>
+      </c>
+      <c r="I5" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
         <v>267</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>268</v>
-      </c>
-      <c r="G6" t="s">
-        <v>277</v>
-      </c>
-      <c r="H6" t="s">
-        <v>281</v>
-      </c>
-      <c r="I6" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>287</v>
+        <v>268</v>
       </c>
       <c r="G7" t="s">
-        <v>288</v>
-      </c>
-      <c r="H7" s="22" t="s">
-        <v>285</v>
+        <v>277</v>
+      </c>
+      <c r="H7" t="s">
+        <v>281</v>
+      </c>
+      <c r="I7" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
+        <v>287</v>
+      </c>
+      <c r="G8" t="s">
+        <v>288</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
         <v>269</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I9" s="22" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
         <v>295</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G10" t="s">
         <v>296</v>
       </c>
-      <c r="H9" s="22" t="s">
+      <c r="H10" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="I9" s="22" t="s">
+      <c r="I10" s="22" t="s">
         <v>291</v>
       </c>
-      <c r="J9" s="22"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
+      <c r="J10" s="22"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
         <v>275</v>
       </c>
-      <c r="I10" s="22"/>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C11" t="s">
+      <c r="I11" s="22"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
         <v>275</v>
       </c>
-      <c r="I11" s="22"/>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="I12" s="22"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
         <v>275</v>
       </c>
-      <c r="I12" s="22"/>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I13" s="22"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="I14" s="22"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="30" t="s">
+        <v>395</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -15031,6 +15183,203 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EB2FAD8-07BE-4066-8361-86590C51D015}">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="B2:I28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
+    <col min="2" max="5" width="3.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" customWidth="1"/>
+    <col min="9" max="9" width="68.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="29" t="s">
+        <v>276</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="30" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>264</v>
+      </c>
+      <c r="G4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G5" t="s">
+        <v>266</v>
+      </c>
+      <c r="H5" t="s">
+        <v>396</v>
+      </c>
+      <c r="I5" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>268</v>
+      </c>
+      <c r="G7" t="s">
+        <v>277</v>
+      </c>
+      <c r="H7" t="s">
+        <v>397</v>
+      </c>
+      <c r="I7" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="30" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>421</v>
+      </c>
+      <c r="I16" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>402</v>
+      </c>
+      <c r="I17" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>403</v>
+      </c>
+      <c r="I18" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>275</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
   <dimension ref="B9:T43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Cleanup and support for WP 7.1
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B55E544-F533-4AD2-B0AC-4B0CD54DB05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0045F5C-9D97-49B2-B91B-D2058F667651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
@@ -24,10 +24,9 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$165</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1761" uniqueCount="469">
   <si>
     <t>Item</t>
   </si>
@@ -1519,9 +1518,6 @@
     <t>Add link content type</t>
   </si>
   <si>
-    <t>In process</t>
-  </si>
-  <si>
     <t>- Open in new tab</t>
   </si>
   <si>
@@ -1532,6 +1528,33 @@
   </si>
   <si>
     <t>{</t>
+  </si>
+  <si>
+    <t>Add formatting options to Table Name display or make it RichText</t>
+  </si>
+  <si>
+    <t>Add column option to make input required and optionally show a "required" indicator.</t>
+  </si>
+  <si>
+    <t>Allow a single column with a bullet (choose bullet or numbered list)</t>
+  </si>
+  <si>
+    <t>Support conversion of a typed fractions to a single fraction character where one exists (e.g., 1/2 goes to a single character rather than 3 characters).</t>
+  </si>
+  <si>
+    <t>Allow the enter key during edit to close edit mode</t>
+  </si>
+  <si>
+    <t>Support column specific formatting so that all values are say bold, italics, a different font size or color,etc.)</t>
+  </si>
+  <si>
+    <t>Allow fields to be concatenated for display purposes to form a single text string from the values in the columns.  Optionally make it a bulleted or numbered list.</t>
+  </si>
+  <si>
+    <t>1.4.7</t>
+  </si>
+  <si>
+    <t>Elected to make it apply to all columns, concatinated. Essentially #154 will support both.</t>
   </si>
 </sst>
 </file>
@@ -1718,22 +1741,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1756,6 +1763,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2075,8 +2098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:O1059"/>
+  <dimension ref="A1:O1078"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.42578125" style="4" customWidth="1"/>
@@ -2133,7 +2155,7 @@
       <c r="N1" s="7"/>
       <c r="O1" s="8"/>
     </row>
-    <row r="2" spans="1:15" hidden="1">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2162,7 +2184,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="75" hidden="1">
+    <row r="3" spans="1:15" ht="75">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2194,7 +2216,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:15" hidden="1">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2226,7 +2248,7 @@
       </c>
       <c r="L4"/>
     </row>
-    <row r="5" spans="1:15" hidden="1">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2258,7 +2280,7 @@
       </c>
       <c r="L5"/>
     </row>
-    <row r="6" spans="1:15" hidden="1">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2290,7 +2312,7 @@
       </c>
       <c r="L6"/>
     </row>
-    <row r="7" spans="1:15" hidden="1">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2322,7 +2344,7 @@
       </c>
       <c r="L7"/>
     </row>
-    <row r="8" spans="1:15" hidden="1">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2354,7 +2376,7 @@
       </c>
       <c r="L8"/>
     </row>
-    <row r="9" spans="1:15" hidden="1">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2386,7 +2408,7 @@
       </c>
       <c r="L9"/>
     </row>
-    <row r="10" spans="1:15" hidden="1">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2418,7 +2440,7 @@
       </c>
       <c r="L10"/>
     </row>
-    <row r="11" spans="1:15" hidden="1">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2450,7 +2472,7 @@
       </c>
       <c r="L11"/>
     </row>
-    <row r="12" spans="1:15" hidden="1">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2482,7 +2504,7 @@
       </c>
       <c r="L12"/>
     </row>
-    <row r="13" spans="1:15" hidden="1">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2514,7 +2536,7 @@
       </c>
       <c r="L13"/>
     </row>
-    <row r="14" spans="1:15" hidden="1">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2546,7 +2568,7 @@
       </c>
       <c r="L14"/>
     </row>
-    <row r="15" spans="1:15" hidden="1">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2578,7 +2600,7 @@
       </c>
       <c r="L15"/>
     </row>
-    <row r="16" spans="1:15" hidden="1">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2610,7 +2632,7 @@
       </c>
       <c r="L16"/>
     </row>
-    <row r="17" spans="1:12" hidden="1">
+    <row r="17" spans="1:12">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2642,7 +2664,7 @@
       </c>
       <c r="L17"/>
     </row>
-    <row r="18" spans="1:12" hidden="1">
+    <row r="18" spans="1:12">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2674,7 +2696,7 @@
       </c>
       <c r="L18"/>
     </row>
-    <row r="19" spans="1:12" hidden="1">
+    <row r="19" spans="1:12">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2706,7 +2728,7 @@
       </c>
       <c r="L19"/>
     </row>
-    <row r="20" spans="1:12" hidden="1">
+    <row r="20" spans="1:12">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2738,7 +2760,7 @@
       </c>
       <c r="L20"/>
     </row>
-    <row r="21" spans="1:12" hidden="1">
+    <row r="21" spans="1:12">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2770,7 +2792,7 @@
       </c>
       <c r="L21"/>
     </row>
-    <row r="22" spans="1:12" hidden="1">
+    <row r="22" spans="1:12">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2802,7 +2824,7 @@
       </c>
       <c r="L22"/>
     </row>
-    <row r="23" spans="1:12" hidden="1">
+    <row r="23" spans="1:12">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2834,7 +2856,7 @@
       </c>
       <c r="L23"/>
     </row>
-    <row r="24" spans="1:12" hidden="1">
+    <row r="24" spans="1:12">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2866,7 +2888,7 @@
       </c>
       <c r="L24"/>
     </row>
-    <row r="25" spans="1:12" hidden="1">
+    <row r="25" spans="1:12">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2898,7 +2920,7 @@
       </c>
       <c r="L25"/>
     </row>
-    <row r="26" spans="1:12" hidden="1">
+    <row r="26" spans="1:12">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2930,7 +2952,7 @@
       </c>
       <c r="L26"/>
     </row>
-    <row r="27" spans="1:12" hidden="1">
+    <row r="27" spans="1:12">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2959,7 +2981,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1">
+    <row r="28" spans="1:12">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2991,7 +3013,7 @@
       </c>
       <c r="L28"/>
     </row>
-    <row r="29" spans="1:12" hidden="1">
+    <row r="29" spans="1:12">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3023,7 +3045,7 @@
       </c>
       <c r="L29"/>
     </row>
-    <row r="30" spans="1:12" hidden="1">
+    <row r="30" spans="1:12">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -3052,7 +3074,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:12" hidden="1">
+    <row r="31" spans="1:12">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3084,7 +3106,7 @@
       </c>
       <c r="L31"/>
     </row>
-    <row r="32" spans="1:12" hidden="1">
+    <row r="32" spans="1:12">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -3113,7 +3135,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="45" hidden="1">
+    <row r="33" spans="1:12" ht="45">
       <c r="A33" s="4">
         <v>33</v>
       </c>
@@ -3145,7 +3167,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:12" hidden="1">
+    <row r="34" spans="1:12">
       <c r="A34" s="4">
         <v>34</v>
       </c>
@@ -3174,7 +3196,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1">
+    <row r="35" spans="1:12">
       <c r="A35">
         <v>37</v>
       </c>
@@ -3206,7 +3228,7 @@
       </c>
       <c r="L35"/>
     </row>
-    <row r="36" spans="1:12" hidden="1">
+    <row r="36" spans="1:12">
       <c r="A36" s="4">
         <v>38</v>
       </c>
@@ -3235,7 +3257,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:12" hidden="1">
+    <row r="37" spans="1:12">
       <c r="A37" s="4">
         <v>40</v>
       </c>
@@ -3264,7 +3286,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:12" hidden="1">
+    <row r="38" spans="1:12">
       <c r="A38">
         <v>41</v>
       </c>
@@ -3294,7 +3316,7 @@
       </c>
       <c r="L38"/>
     </row>
-    <row r="39" spans="1:12" hidden="1">
+    <row r="39" spans="1:12">
       <c r="A39">
         <v>42</v>
       </c>
@@ -3326,7 +3348,7 @@
       </c>
       <c r="L39"/>
     </row>
-    <row r="40" spans="1:12" hidden="1">
+    <row r="40" spans="1:12">
       <c r="A40" s="4">
         <v>44</v>
       </c>
@@ -3358,7 +3380,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:12" hidden="1">
+    <row r="41" spans="1:12">
       <c r="A41" s="4">
         <v>45</v>
       </c>
@@ -3387,7 +3409,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:12" hidden="1">
+    <row r="42" spans="1:12">
       <c r="A42" s="4">
         <v>46</v>
       </c>
@@ -3416,7 +3438,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="120" hidden="1">
+    <row r="43" spans="1:12" ht="120">
       <c r="A43" s="4">
         <v>47</v>
       </c>
@@ -3448,7 +3470,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:12" hidden="1">
+    <row r="44" spans="1:12">
       <c r="A44">
         <v>48</v>
       </c>
@@ -3480,7 +3502,7 @@
       </c>
       <c r="L44"/>
     </row>
-    <row r="45" spans="1:12" hidden="1">
+    <row r="45" spans="1:12">
       <c r="A45" s="4">
         <v>49</v>
       </c>
@@ -3509,7 +3531,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1">
+    <row r="46" spans="1:12">
       <c r="A46" s="4">
         <v>50</v>
       </c>
@@ -3538,7 +3560,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1">
+    <row r="47" spans="1:12">
       <c r="A47">
         <v>51</v>
       </c>
@@ -3570,7 +3592,7 @@
       </c>
       <c r="L47"/>
     </row>
-    <row r="48" spans="1:12" hidden="1">
+    <row r="48" spans="1:12">
       <c r="A48" s="4">
         <v>57</v>
       </c>
@@ -3602,7 +3624,7 @@
       </c>
       <c r="L48"/>
     </row>
-    <row r="49" spans="1:12" hidden="1">
+    <row r="49" spans="1:12">
       <c r="A49" s="4">
         <v>58</v>
       </c>
@@ -3631,7 +3653,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:12" hidden="1">
+    <row r="50" spans="1:12">
       <c r="A50">
         <v>59</v>
       </c>
@@ -3663,7 +3685,7 @@
       </c>
       <c r="L50"/>
     </row>
-    <row r="51" spans="1:12" hidden="1">
+    <row r="51" spans="1:12">
       <c r="A51" s="4">
         <v>60</v>
       </c>
@@ -3692,7 +3714,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:12" hidden="1">
+    <row r="52" spans="1:12">
       <c r="A52" s="4">
         <v>62</v>
       </c>
@@ -3721,7 +3743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:12" hidden="1">
+    <row r="53" spans="1:12">
       <c r="A53" s="4">
         <v>63</v>
       </c>
@@ -3751,7 +3773,7 @@
       </c>
       <c r="L53" s="6"/>
     </row>
-    <row r="54" spans="1:12" hidden="1">
+    <row r="54" spans="1:12">
       <c r="A54" s="4">
         <v>66</v>
       </c>
@@ -3783,7 +3805,7 @@
       </c>
       <c r="L54"/>
     </row>
-    <row r="55" spans="1:12" hidden="1">
+    <row r="55" spans="1:12">
       <c r="A55" s="4">
         <v>67</v>
       </c>
@@ -3812,7 +3834,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:12" hidden="1">
+    <row r="56" spans="1:12">
       <c r="A56" s="4">
         <v>69</v>
       </c>
@@ -3841,7 +3863,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:12" hidden="1">
+    <row r="57" spans="1:12">
       <c r="A57" s="4">
         <v>76</v>
       </c>
@@ -3870,7 +3892,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:12" hidden="1">
+    <row r="58" spans="1:12">
       <c r="A58" s="4">
         <v>76</v>
       </c>
@@ -3899,7 +3921,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="30" hidden="1">
+    <row r="59" spans="1:12" ht="30">
       <c r="A59" s="4">
         <v>82</v>
       </c>
@@ -3929,7 +3951,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:12" hidden="1">
+    <row r="60" spans="1:12">
       <c r="A60" s="4">
         <v>83</v>
       </c>
@@ -3962,7 +3984,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="61" spans="1:12" hidden="1">
+    <row r="61" spans="1:12">
       <c r="A61" s="4">
         <v>85</v>
       </c>
@@ -3992,7 +4014,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:12" hidden="1">
+    <row r="62" spans="1:12">
       <c r="A62" s="4">
         <v>32</v>
       </c>
@@ -4021,7 +4043,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:12" hidden="1">
+    <row r="63" spans="1:12">
       <c r="A63" s="4">
         <v>54</v>
       </c>
@@ -4047,7 +4069,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:12" hidden="1">
+    <row r="64" spans="1:12">
       <c r="A64" s="4">
         <v>61</v>
       </c>
@@ -4074,7 +4096,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:12" hidden="1">
+    <row r="65" spans="1:12">
       <c r="A65" s="4">
         <v>87</v>
       </c>
@@ -4101,7 +4123,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:12" hidden="1">
+    <row r="66" spans="1:12">
       <c r="A66" s="4">
         <v>89</v>
       </c>
@@ -4130,7 +4152,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:12" hidden="1">
+    <row r="67" spans="1:12">
       <c r="A67" s="4">
         <v>74</v>
       </c>
@@ -4157,7 +4179,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:12" hidden="1">
+    <row r="68" spans="1:12">
       <c r="A68" s="4">
         <v>91</v>
       </c>
@@ -4183,7 +4205,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:12" hidden="1">
+    <row r="69" spans="1:12">
       <c r="A69" s="4">
         <v>92</v>
       </c>
@@ -4210,7 +4232,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="30" hidden="1">
+    <row r="70" spans="1:12" ht="30">
       <c r="A70" s="4">
         <v>68</v>
       </c>
@@ -4239,7 +4261,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="30" hidden="1">
+    <row r="71" spans="1:12" ht="30">
       <c r="A71" s="4">
         <v>78</v>
       </c>
@@ -4269,7 +4291,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:12" hidden="1">
+    <row r="72" spans="1:12">
       <c r="A72" s="4">
         <v>93</v>
       </c>
@@ -4299,7 +4321,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1">
+    <row r="73" spans="1:12">
       <c r="A73" s="4">
         <v>94</v>
       </c>
@@ -4329,7 +4351,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1">
+    <row r="74" spans="1:12">
       <c r="A74" s="4">
         <v>98</v>
       </c>
@@ -4356,7 +4378,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1">
+    <row r="75" spans="1:12">
       <c r="A75" s="4">
         <v>99</v>
       </c>
@@ -4388,7 +4410,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="76" spans="1:12" hidden="1">
+    <row r="76" spans="1:12">
       <c r="A76" s="4">
         <v>90</v>
       </c>
@@ -4418,7 +4440,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="30" hidden="1">
+    <row r="77" spans="1:12" ht="30">
       <c r="A77" s="4">
         <v>95</v>
       </c>
@@ -4448,7 +4470,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="30" hidden="1">
+    <row r="78" spans="1:12" ht="30">
       <c r="A78" s="4">
         <v>96</v>
       </c>
@@ -4478,7 +4500,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="30" hidden="1">
+    <row r="79" spans="1:12" ht="30">
       <c r="A79" s="4">
         <v>97</v>
       </c>
@@ -4511,7 +4533,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1">
+    <row r="80" spans="1:12">
       <c r="A80" s="4">
         <v>109</v>
       </c>
@@ -4540,7 +4562,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1">
+    <row r="81" spans="1:12">
       <c r="A81" s="4">
         <v>110</v>
       </c>
@@ -4569,7 +4591,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="30" hidden="1">
+    <row r="82" spans="1:12" ht="30">
       <c r="A82" s="4">
         <v>111</v>
       </c>
@@ -4598,7 +4620,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="30" hidden="1">
+    <row r="83" spans="1:12" ht="30">
       <c r="A83" s="4">
         <v>125</v>
       </c>
@@ -4627,7 +4649,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1">
+    <row r="84" spans="1:12">
       <c r="A84" s="4">
         <v>128</v>
       </c>
@@ -4656,7 +4678,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1">
+    <row r="85" spans="1:12">
       <c r="A85" s="4">
         <v>129</v>
       </c>
@@ -4685,7 +4707,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:12" hidden="1">
+    <row r="86" spans="1:12">
       <c r="A86" s="4">
         <v>135</v>
       </c>
@@ -4714,7 +4736,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:12" hidden="1">
+    <row r="87" spans="1:12">
       <c r="A87" s="4">
         <v>133</v>
       </c>
@@ -4740,7 +4762,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:12" hidden="1">
+    <row r="88" spans="1:12">
       <c r="A88" s="4">
         <v>136</v>
       </c>
@@ -4769,7 +4791,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1">
+    <row r="89" spans="1:12">
       <c r="A89" s="4">
         <v>134</v>
       </c>
@@ -4798,7 +4820,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1">
+    <row r="90" spans="1:12">
       <c r="A90" s="4">
         <v>137</v>
       </c>
@@ -4827,7 +4849,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="30" hidden="1">
+    <row r="91" spans="1:12" ht="30">
       <c r="A91" s="4">
         <v>140</v>
       </c>
@@ -4856,7 +4878,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:12" hidden="1">
+    <row r="92" spans="1:12">
       <c r="A92" s="4">
         <v>141</v>
       </c>
@@ -4888,7 +4910,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1">
+    <row r="93" spans="1:12">
       <c r="A93" s="4">
         <v>35</v>
       </c>
@@ -4920,7 +4942,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="94" spans="1:12" hidden="1">
+    <row r="94" spans="1:12">
       <c r="A94" s="4">
         <v>39</v>
       </c>
@@ -4949,7 +4971,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:12" hidden="1">
+    <row r="95" spans="1:12">
       <c r="A95" s="4">
         <v>43</v>
       </c>
@@ -4978,7 +5000,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:12" hidden="1">
+    <row r="96" spans="1:12">
       <c r="A96" s="4">
         <v>81</v>
       </c>
@@ -5010,7 +5032,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="97" spans="1:11" hidden="1">
+    <row r="97" spans="1:11">
       <c r="A97" s="4">
         <v>120</v>
       </c>
@@ -5036,7 +5058,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:11" hidden="1">
+    <row r="98" spans="1:11">
       <c r="A98" s="4">
         <v>101</v>
       </c>
@@ -5062,7 +5084,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:11" hidden="1">
+    <row r="99" spans="1:11">
       <c r="A99" s="4">
         <v>126</v>
       </c>
@@ -5091,7 +5113,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:11" hidden="1">
+    <row r="100" spans="1:11">
       <c r="A100" s="4">
         <v>131</v>
       </c>
@@ -5120,7 +5142,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:11" hidden="1">
+    <row r="101" spans="1:11">
       <c r="A101" s="4">
         <v>65</v>
       </c>
@@ -5147,7 +5169,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:11" hidden="1">
+    <row r="102" spans="1:11">
       <c r="A102" s="4">
         <v>119</v>
       </c>
@@ -5173,7 +5195,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:11" hidden="1">
+    <row r="103" spans="1:11">
       <c r="A103" s="4">
         <v>138</v>
       </c>
@@ -5202,7 +5224,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:11" hidden="1">
+    <row r="104" spans="1:11">
       <c r="A104" s="4">
         <v>144</v>
       </c>
@@ -5228,7 +5250,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:11" hidden="1">
+    <row r="105" spans="1:11">
       <c r="A105" s="4">
         <v>145</v>
       </c>
@@ -5251,7 +5273,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:11" hidden="1">
+    <row r="106" spans="1:11">
       <c r="A106" s="4">
         <v>118</v>
       </c>
@@ -5277,7 +5299,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:11" hidden="1">
+    <row r="107" spans="1:11">
       <c r="A107" s="4">
         <v>146</v>
       </c>
@@ -5303,7 +5325,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:11" hidden="1">
+    <row r="108" spans="1:11">
       <c r="A108" s="4">
         <v>73</v>
       </c>
@@ -5330,7 +5352,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:11" hidden="1">
+    <row r="109" spans="1:11">
       <c r="A109" s="4">
         <v>116</v>
       </c>
@@ -5356,7 +5378,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:11" hidden="1">
+    <row r="110" spans="1:11">
       <c r="A110" s="4">
         <v>145</v>
       </c>
@@ -5386,7 +5408,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:11" hidden="1">
+    <row r="111" spans="1:11">
       <c r="A111" s="4">
         <v>56</v>
       </c>
@@ -5413,7 +5435,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="112" spans="1:11" hidden="1">
+    <row r="112" spans="1:11">
       <c r="A112" s="4">
         <v>104</v>
       </c>
@@ -5439,7 +5461,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:12" ht="30" hidden="1">
+    <row r="113" spans="1:12" ht="30">
       <c r="A113" s="4">
         <v>147</v>
       </c>
@@ -5494,152 +5516,137 @@
         <v>26</v>
       </c>
     </row>
-    <row r="115" spans="1:12" ht="45">
+    <row r="115" spans="1:12">
       <c r="A115" s="4">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>253</v>
+        <v>454</v>
       </c>
       <c r="C115" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>254</v>
+        <v>86</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G115" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="H115" s="13" t="s">
         <v>391</v>
       </c>
-      <c r="J115" s="4">
-        <v>1</v>
-      </c>
       <c r="K115" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L115" s="4" t="s">
-        <v>324</v>
+        <v>26</v>
       </c>
     </row>
     <row r="116" spans="1:12">
       <c r="A116" s="4">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>393</v>
+        <v>455</v>
       </c>
       <c r="C116" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>254</v>
+        <v>86</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G116" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H116" s="13" t="s">
         <v>391</v>
       </c>
-      <c r="J116" s="4">
-        <v>2</v>
-      </c>
       <c r="K116" s="4" t="s">
-        <v>256</v>
+        <v>26</v>
       </c>
     </row>
     <row r="117" spans="1:12" ht="30">
       <c r="A117" s="4">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>390</v>
+        <v>462</v>
       </c>
       <c r="C117" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E117" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E117" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G117" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H117" s="13" t="s">
-        <v>391</v>
+        <v>467</v>
       </c>
       <c r="J117" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K117" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L117" s="4" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="118" spans="1:12">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" ht="45">
       <c r="A118" s="4">
-        <v>124</v>
+        <v>158</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>239</v>
+        <v>466</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F118" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G118" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H118" s="13" t="s">
-        <v>391</v>
+        <v>467</v>
       </c>
       <c r="J118" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K118" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="119" spans="1:12">
+        <v>155</v>
+      </c>
+      <c r="L118" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" ht="30">
       <c r="A119" s="4">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E119" s="4" t="s">
         <v>86</v>
@@ -5647,237 +5654,249 @@
       <c r="F119" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="G119" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="H119" s="13" t="s">
-        <v>391</v>
+        <v>467</v>
       </c>
       <c r="J119" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K119" s="4" t="s">
-        <v>456</v>
+        <v>256</v>
       </c>
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="4">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F120" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G120" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H120" s="13" t="s">
-        <v>391</v>
+        <v>467</v>
       </c>
       <c r="J120" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K120" s="4" t="s">
-        <v>456</v>
+        <v>256</v>
       </c>
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="4">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G121" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H121" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J121" s="4">
-        <v>10</v>
+        <v>467</v>
+      </c>
+      <c r="J121" s="5">
+        <v>5</v>
       </c>
       <c r="K121" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="4">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>332</v>
+        <v>393</v>
       </c>
       <c r="C122" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>131</v>
+        <v>254</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G122" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H122" s="13" t="s">
+        <v>467</v>
+      </c>
+      <c r="J122" s="5">
+        <v>6</v>
+      </c>
+      <c r="K122" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" ht="45">
+      <c r="A123" s="4">
         <v>132</v>
       </c>
-      <c r="J122" s="4">
-        <v>10</v>
-      </c>
-      <c r="K122" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12">
-      <c r="A123" s="4">
-        <v>77</v>
-      </c>
       <c r="B123" s="4" t="s">
-        <v>141</v>
+        <v>253</v>
       </c>
       <c r="C123" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>131</v>
+        <v>254</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G123" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="H123" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I123" s="5">
-        <v>80</v>
+        <v>467</v>
       </c>
       <c r="J123" s="5">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="K123" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="124" spans="1:12">
+        <v>256</v>
+      </c>
+      <c r="L123" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" ht="30">
       <c r="A124" s="4">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>211</v>
+        <v>390</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="E124" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G124" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H124" s="13" t="s">
-        <v>132</v>
+        <v>467</v>
       </c>
       <c r="J124" s="5">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="K124" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12">
+        <v>256</v>
+      </c>
+      <c r="L124" s="4" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" ht="30">
       <c r="A125" s="4">
-        <v>100</v>
+        <v>152</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>246</v>
+        <v>460</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="G125" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H125" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J125" s="4">
-        <v>20</v>
+        <v>467</v>
       </c>
       <c r="K125" s="4" t="s">
-        <v>132</v>
+        <v>26</v>
       </c>
     </row>
     <row r="126" spans="1:12">
       <c r="A126" s="4">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>244</v>
+        <v>217</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E126" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F126" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G126" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="H126" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J126" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K126" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L126" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="127" spans="1:12">
       <c r="A127" s="4">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>17</v>
@@ -5889,13 +5908,13 @@
         <v>25</v>
       </c>
       <c r="G127" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H127" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J127" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K127" s="4" t="s">
         <v>132</v>
@@ -5903,31 +5922,31 @@
     </row>
     <row r="128" spans="1:12">
       <c r="A128" s="4">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G128" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="H128" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J128" s="4">
-        <v>30</v>
+      <c r="I128" s="5">
+        <v>80</v>
+      </c>
+      <c r="J128" s="5">
+        <v>20</v>
       </c>
       <c r="K128" s="4" t="s">
         <v>132</v>
@@ -5935,13 +5954,13 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" s="4">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>171</v>
+        <v>211</v>
       </c>
       <c r="C129" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>17</v>
@@ -5950,13 +5969,13 @@
         <v>55</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H129" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J129" s="4">
-        <v>30</v>
+      <c r="J129" s="5">
+        <v>20</v>
       </c>
       <c r="K129" s="4" t="s">
         <v>132</v>
@@ -5964,31 +5983,28 @@
     </row>
     <row r="130" spans="1:12">
       <c r="A130" s="4">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>223</v>
+        <v>246</v>
       </c>
       <c r="C130" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G130" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H130" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J130" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K130" s="4" t="s">
         <v>132</v>
@@ -5996,57 +6012,66 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" s="4">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="G131" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J131" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K131" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="132" spans="1:12" ht="30">
+      <c r="L131" s="4" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12">
       <c r="A132" s="4">
-        <v>114</v>
+        <v>143</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>226</v>
+        <v>331</v>
       </c>
       <c r="C132" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G132" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J132" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K132" s="4" t="s">
         <v>132</v>
@@ -6054,22 +6079,25 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" s="4">
-        <v>115</v>
+        <v>83</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>225</v>
+        <v>149</v>
       </c>
       <c r="C133" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D133" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G133" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
@@ -6083,10 +6111,10 @@
     </row>
     <row r="134" spans="1:12">
       <c r="A134" s="4">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>142</v>
+        <v>171</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>190</v>
@@ -6095,19 +6123,16 @@
         <v>17</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H134" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I134" s="5">
-        <v>139</v>
-      </c>
-      <c r="J134" s="5">
-        <v>40</v>
+      <c r="J134" s="4">
+        <v>30</v>
       </c>
       <c r="K134" s="4" t="s">
         <v>132</v>
@@ -6115,31 +6140,31 @@
     </row>
     <row r="135" spans="1:12">
       <c r="A135" s="4">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C135" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F135" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G135" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I135" s="5" t="s">
-        <v>232</v>
-      </c>
       <c r="J135" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>132</v>
@@ -6147,13 +6172,13 @@
     </row>
     <row r="136" spans="1:12">
       <c r="A136" s="4">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="C136" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D136" s="4" t="s">
         <v>17</v>
@@ -6164,28 +6189,25 @@
       <c r="F136" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G136" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H136" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J136" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K136" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="137" spans="1:12">
+    <row r="137" spans="1:12" ht="30">
       <c r="A137" s="4">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="C137" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>17</v>
@@ -6196,57 +6218,51 @@
       <c r="F137" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G137" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H137" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J137" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K137" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="138" spans="1:12" ht="30">
+    <row r="138" spans="1:12">
       <c r="A138" s="4">
-        <v>26</v>
+        <v>115</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="C138" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D138" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G138" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H138" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J138" s="4">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K138" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="139" spans="1:12" ht="30">
+    <row r="139" spans="1:12">
       <c r="A139" s="4">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>190</v>
@@ -6263,8 +6279,11 @@
       <c r="H139" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I139" s="5">
+        <v>139</v>
+      </c>
       <c r="J139" s="5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K139" s="4" t="s">
         <v>132</v>
@@ -6272,10 +6291,10 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" s="4">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>143</v>
+        <v>229</v>
       </c>
       <c r="C140" s="15" t="s">
         <v>190</v>
@@ -6284,16 +6303,19 @@
         <v>17</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H140" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J140" s="5">
-        <v>50</v>
+      <c r="I140" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="J140" s="4">
+        <v>40</v>
       </c>
       <c r="K140" s="4" t="s">
         <v>132</v>
@@ -6301,28 +6323,31 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" s="4">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="C141" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E141" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F141" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="G141" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="H141" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J141" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K141" s="4" t="s">
         <v>132</v>
@@ -6330,51 +6355,57 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" s="4">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
       <c r="C142" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D142" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
+      </c>
+      <c r="G142" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J142" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K142" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="143" spans="1:12">
+    <row r="143" spans="1:12" ht="30">
       <c r="A143" s="4">
-        <v>121</v>
+        <v>26</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C143" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E143" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="G143" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H143" s="13" t="s">
         <v>132</v>
@@ -6386,47 +6417,41 @@
         <v>132</v>
       </c>
     </row>
-    <row r="144" spans="1:12">
+    <row r="144" spans="1:12" ht="30">
       <c r="A144" s="4">
+        <v>72</v>
+      </c>
+      <c r="B144" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>247</v>
       </c>
       <c r="C144" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G144" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H144" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J144" s="4">
+      <c r="J144" s="5">
         <v>50</v>
       </c>
       <c r="K144" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L144" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="145" spans="1:12" ht="30">
+    </row>
+    <row r="145" spans="1:12">
       <c r="A145" s="4">
+        <v>80</v>
+      </c>
+      <c r="B145" s="4" t="s">
         <v>143</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>322</v>
       </c>
       <c r="C145" s="15" t="s">
         <v>190</v>
@@ -6435,18 +6460,15 @@
         <v>17</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H145" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I145" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="J145" s="4">
+      <c r="J145" s="5">
         <v>50</v>
       </c>
       <c r="K145" s="4" t="s">
@@ -6455,10 +6477,10 @@
     </row>
     <row r="146" spans="1:12">
       <c r="A146" s="4">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C146" s="15" t="s">
         <v>190</v>
@@ -6470,13 +6492,13 @@
         <v>55</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H146" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J146" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K146" s="4" t="s">
         <v>132</v>
@@ -6484,19 +6506,19 @@
     </row>
     <row r="147" spans="1:12">
       <c r="A147" s="4">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>133</v>
+        <v>220</v>
       </c>
       <c r="C147" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F147" s="4" t="s">
         <v>25</v>
@@ -6504,8 +6526,8 @@
       <c r="H147" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J147" s="5">
-        <v>80</v>
+      <c r="J147" s="4">
+        <v>50</v>
       </c>
       <c r="K147" s="4" t="s">
         <v>132</v>
@@ -6513,28 +6535,28 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="4">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>150</v>
+        <v>234</v>
       </c>
       <c r="C148" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F148" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H148" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J148" s="5">
-        <v>80</v>
+      <c r="J148" s="4">
+        <v>50</v>
       </c>
       <c r="K148" s="4" t="s">
         <v>132</v>
@@ -6542,124 +6564,124 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="4">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="C149" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D149" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>146</v>
+        <v>55</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G149" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H149" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J149" s="4">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="K149" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="150" spans="1:12">
+      <c r="L149" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12" ht="30">
       <c r="A150" s="4">
-        <v>36</v>
+        <v>143</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>29</v>
+        <v>322</v>
       </c>
       <c r="C150" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G150" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H150" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I150" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="J150" s="4">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="K150" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="151" spans="1:12" ht="30">
+    <row r="151" spans="1:12">
       <c r="A151" s="4">
-        <v>52</v>
+        <v>106</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>28</v>
+        <v>218</v>
       </c>
       <c r="C151" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E151" s="4" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="F151" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G151" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H151" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J151" s="4">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="K151" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L151" s="4" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="152" spans="1:12">
       <c r="A152" s="4">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>40</v>
+        <v>133</v>
       </c>
       <c r="C152" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>30</v>
+        <v>131</v>
       </c>
       <c r="F152" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G152" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H152" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J152" s="4">
-        <v>99</v>
+      <c r="J152" s="5">
+        <v>80</v>
       </c>
       <c r="K152" s="4" t="s">
         <v>132</v>
@@ -6667,83 +6689,74 @@
     </row>
     <row r="153" spans="1:12">
       <c r="A153" s="4">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>79</v>
+        <v>150</v>
       </c>
       <c r="C153" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>251</v>
+        <v>131</v>
       </c>
       <c r="F153" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G153" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="H153" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J153" s="4">
-        <v>99</v>
+      <c r="J153" s="5">
+        <v>80</v>
       </c>
       <c r="K153" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="154" spans="1:12" ht="30">
+    <row r="154" spans="1:12">
       <c r="A154" s="4">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>125</v>
+        <v>219</v>
       </c>
       <c r="C154" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F154" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G154" s="4" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="H154" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J154" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K154" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="155" spans="1:12" ht="30">
+    <row r="155" spans="1:12">
       <c r="A155" s="4">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>128</v>
+        <v>29</v>
       </c>
       <c r="C155" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D155" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E155" s="4" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="F155" s="4" t="s">
         <v>6</v>
@@ -6761,27 +6774,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="156" spans="1:12">
+    <row r="156" spans="1:12" ht="30">
       <c r="A156" s="4">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>154</v>
+        <v>28</v>
       </c>
       <c r="C156" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D156" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E156" s="4" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="F156" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G156" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H156" s="13" t="s">
         <v>132</v>
@@ -6792,28 +6805,31 @@
       <c r="K156" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="157" spans="1:12" ht="30">
+      <c r="L156" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="157" spans="1:12">
       <c r="A157" s="4">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>311</v>
+        <v>40</v>
       </c>
       <c r="C157" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D157" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E157" s="4" t="s">
-        <v>310</v>
+        <v>30</v>
       </c>
       <c r="F157" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G157" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H157" s="13" t="s">
         <v>132</v>
@@ -6824,16 +6840,13 @@
       <c r="K157" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L157" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="158" spans="1:12" ht="45">
+    </row>
+    <row r="158" spans="1:12">
       <c r="A158" s="4">
-        <v>142</v>
+        <v>55</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>319</v>
+        <v>79</v>
       </c>
       <c r="C158" s="15" t="s">
         <v>189</v>
@@ -6842,13 +6855,13 @@
         <v>18</v>
       </c>
       <c r="E158" s="4" t="s">
-        <v>320</v>
+        <v>251</v>
       </c>
       <c r="F158" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G158" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H158" s="13" t="s">
         <v>132</v>
@@ -6859,118 +6872,324 @@
       <c r="K158" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L158" s="4" t="s">
+    </row>
+    <row r="159" spans="1:12" ht="30">
+      <c r="A159" s="4">
+        <v>70</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C159" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D159" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E159" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F159" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G159" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H159" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J159" s="4">
+        <v>99</v>
+      </c>
+      <c r="K159" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" ht="30">
+      <c r="A160" s="4">
+        <v>71</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C160" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D160" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E160" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G160" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H160" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J160" s="4">
+        <v>99</v>
+      </c>
+      <c r="K160" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12">
+      <c r="A161" s="4">
+        <v>88</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C161" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D161" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E161" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F161" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G161" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H161" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J161" s="4">
+        <v>99</v>
+      </c>
+      <c r="K161" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12" ht="30">
+      <c r="A162" s="4">
+        <v>139</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C162" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D162" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E162" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G162" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H162" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J162" s="4">
+        <v>99</v>
+      </c>
+      <c r="K162" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L162" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12" ht="45">
+      <c r="A163" s="4">
+        <v>142</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C163" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D163" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E163" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G163" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H163" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J163" s="4">
+        <v>99</v>
+      </c>
+      <c r="K163" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L163" s="4" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="159" spans="1:12">
-      <c r="H159" s="13"/>
-    </row>
-    <row r="160" spans="1:12">
-      <c r="H160" s="13"/>
-    </row>
-    <row r="161" spans="1:8">
-      <c r="H161" s="13"/>
-    </row>
-    <row r="162" spans="1:8">
-      <c r="H162" s="13"/>
-    </row>
-    <row r="163" spans="1:8">
-      <c r="H163" s="13"/>
-    </row>
-    <row r="164" spans="1:8">
-      <c r="A164" s="9">
-        <f>MAX(A1:A163)</f>
-        <v>151</v>
-      </c>
-      <c r="B164" s="9" t="s">
+    <row r="164" spans="1:12" ht="45">
+      <c r="A164" s="4">
+        <v>155</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="C164" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D164" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E164" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G164" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H164" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J164" s="4">
+        <v>99</v>
+      </c>
+      <c r="K164" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="165" spans="1:12" ht="30">
+      <c r="A165" s="4">
+        <v>157</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="C165" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D165" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E165" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F165" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G165" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H165" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J165" s="4">
+        <v>99</v>
+      </c>
+      <c r="K165" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12">
+      <c r="H166" s="13"/>
+    </row>
+    <row r="167" spans="1:12">
+      <c r="H167" s="13"/>
+    </row>
+    <row r="168" spans="1:12">
+      <c r="H168" s="13"/>
+    </row>
+    <row r="169" spans="1:12">
+      <c r="H169" s="13"/>
+    </row>
+    <row r="170" spans="1:12">
+      <c r="H170" s="13"/>
+    </row>
+    <row r="171" spans="1:12">
+      <c r="H171" s="13"/>
+    </row>
+    <row r="172" spans="1:12">
+      <c r="H172" s="13"/>
+    </row>
+    <row r="173" spans="1:12">
+      <c r="H173" s="13"/>
+    </row>
+    <row r="174" spans="1:12">
+      <c r="H174" s="13"/>
+    </row>
+    <row r="175" spans="1:12">
+      <c r="H175" s="13"/>
+    </row>
+    <row r="176" spans="1:12">
+      <c r="H176" s="13"/>
+    </row>
+    <row r="177" spans="1:8">
+      <c r="H177" s="13"/>
+    </row>
+    <row r="178" spans="1:8">
+      <c r="H178" s="13"/>
+    </row>
+    <row r="179" spans="1:8">
+      <c r="H179" s="13"/>
+    </row>
+    <row r="180" spans="1:8">
+      <c r="H180" s="13"/>
+    </row>
+    <row r="181" spans="1:8">
+      <c r="H181" s="13"/>
+    </row>
+    <row r="182" spans="1:8">
+      <c r="H182" s="13"/>
+    </row>
+    <row r="183" spans="1:8">
+      <c r="A183" s="9">
+        <f>MAX(A1:A182)</f>
+        <v>158</v>
+      </c>
+      <c r="B183" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C164" s="16"/>
-      <c r="H164" s="13"/>
-    </row>
-    <row r="165" spans="1:8">
-      <c r="H165" s="13"/>
-    </row>
-    <row r="166" spans="1:8">
-      <c r="H166" s="13"/>
-    </row>
-    <row r="167" spans="1:8">
-      <c r="H167" s="13"/>
-    </row>
-    <row r="168" spans="1:8">
-      <c r="H168" s="13"/>
-    </row>
-    <row r="169" spans="1:8">
-      <c r="H169" s="13"/>
-    </row>
-    <row r="170" spans="1:8">
-      <c r="H170" s="13"/>
-    </row>
-    <row r="171" spans="1:8">
-      <c r="H171" s="13"/>
-    </row>
-    <row r="172" spans="1:8">
-      <c r="H172" s="13"/>
-    </row>
-    <row r="173" spans="1:8">
-      <c r="H173" s="13"/>
-    </row>
-    <row r="174" spans="1:8">
-      <c r="H174" s="13"/>
-    </row>
-    <row r="175" spans="1:8">
-      <c r="H175" s="13"/>
-    </row>
-    <row r="176" spans="1:8">
-      <c r="H176" s="13"/>
-    </row>
-    <row r="177" spans="8:8">
-      <c r="H177" s="13"/>
-    </row>
-    <row r="178" spans="8:8">
-      <c r="H178" s="13"/>
-    </row>
-    <row r="179" spans="8:8">
-      <c r="H179" s="13"/>
-    </row>
-    <row r="180" spans="8:8">
-      <c r="H180" s="13"/>
-    </row>
-    <row r="181" spans="8:8">
-      <c r="H181" s="13"/>
-    </row>
-    <row r="182" spans="8:8">
-      <c r="H182" s="13"/>
-    </row>
-    <row r="183" spans="8:8">
+      <c r="C183" s="16"/>
       <c r="H183" s="13"/>
     </row>
-    <row r="184" spans="8:8">
+    <row r="184" spans="1:8">
       <c r="H184" s="13"/>
     </row>
-    <row r="185" spans="8:8">
+    <row r="185" spans="1:8">
       <c r="H185" s="13"/>
     </row>
-    <row r="186" spans="8:8">
+    <row r="186" spans="1:8">
       <c r="H186" s="13"/>
     </row>
-    <row r="187" spans="8:8">
+    <row r="187" spans="1:8">
       <c r="H187" s="13"/>
     </row>
-    <row r="188" spans="8:8">
+    <row r="188" spans="1:8">
       <c r="H188" s="13"/>
     </row>
-    <row r="189" spans="8:8">
+    <row r="189" spans="1:8">
       <c r="H189" s="13"/>
     </row>
-    <row r="190" spans="8:8">
+    <row r="190" spans="1:8">
       <c r="H190" s="13"/>
     </row>
-    <row r="191" spans="8:8">
+    <row r="191" spans="1:8">
       <c r="H191" s="13"/>
     </row>
-    <row r="192" spans="8:8">
+    <row r="192" spans="1:8">
       <c r="H192" s="13"/>
     </row>
     <row r="193" spans="8:8">
@@ -9574,23 +9793,73 @@
     <row r="1059" spans="8:8">
       <c r="H1059" s="13"/>
     </row>
+    <row r="1060" spans="8:8">
+      <c r="H1060" s="13"/>
+    </row>
+    <row r="1061" spans="8:8">
+      <c r="H1061" s="13"/>
+    </row>
+    <row r="1062" spans="8:8">
+      <c r="H1062" s="13"/>
+    </row>
+    <row r="1063" spans="8:8">
+      <c r="H1063" s="13"/>
+    </row>
+    <row r="1064" spans="8:8">
+      <c r="H1064" s="13"/>
+    </row>
+    <row r="1065" spans="8:8">
+      <c r="H1065" s="13"/>
+    </row>
+    <row r="1066" spans="8:8">
+      <c r="H1066" s="13"/>
+    </row>
+    <row r="1067" spans="8:8">
+      <c r="H1067" s="13"/>
+    </row>
+    <row r="1068" spans="8:8">
+      <c r="H1068" s="13"/>
+    </row>
+    <row r="1069" spans="8:8">
+      <c r="H1069" s="13"/>
+    </row>
+    <row r="1070" spans="8:8">
+      <c r="H1070" s="13"/>
+    </row>
+    <row r="1071" spans="8:8">
+      <c r="H1071" s="13"/>
+    </row>
+    <row r="1072" spans="8:8">
+      <c r="H1072" s="13"/>
+    </row>
+    <row r="1073" spans="8:8">
+      <c r="H1073" s="13"/>
+    </row>
+    <row r="1074" spans="8:8">
+      <c r="H1074" s="13"/>
+    </row>
+    <row r="1075" spans="8:8">
+      <c r="H1075" s="13"/>
+    </row>
+    <row r="1076" spans="8:8">
+      <c r="H1076" s="13"/>
+    </row>
+    <row r="1077" spans="8:8">
+      <c r="H1077" s="13"/>
+    </row>
+    <row r="1078" spans="8:8">
+      <c r="H1078" s="13"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B1:L158" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="1.4.5"/>
-        <filter val="1.4.6"/>
-        <filter val="Roadmap"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="B1:L165" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L77">
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L158">
-    <sortCondition ref="H2:H158"/>
-    <sortCondition ref="J2:J158"/>
-    <sortCondition ref="A2:A158"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L165">
+    <sortCondition ref="H2:H165"/>
+    <sortCondition ref="J2:J165"/>
+    <sortCondition ref="A2:A165"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9989,43 +10258,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="35" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="19"/>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="34" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="26"/>
-      <c r="F1" s="24" t="s">
+      <c r="E1" s="34"/>
+      <c r="F1" s="32" t="s">
         <v>197</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="32" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="32" t="s">
         <v>175</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="32" t="s">
         <v>177</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="K1" s="26"/>
-      <c r="L1" s="24" t="s">
+      <c r="K1" s="34"/>
+      <c r="L1" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="32" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:45" ht="30.75" customHeight="1">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
+      <c r="A2" s="36"/>
+      <c r="B2" s="36"/>
       <c r="C2" s="20" t="s">
         <v>16</v>
       </c>
@@ -10035,18 +10304,18 @@
       <c r="E2" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
       <c r="J2" s="18" t="s">
         <v>185</v>
       </c>
       <c r="K2" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -10415,7 +10684,7 @@
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>189</v>
@@ -10424,7 +10693,7 @@
         <v>189</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
@@ -10914,7 +11183,7 @@
       <c r="AS17" s="11"/>
     </row>
     <row r="18" spans="1:45">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="25" t="s">
         <v>407</v>
       </c>
       <c r="B18" s="4"/>
@@ -14976,13 +15245,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="37" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
         <v>448</v>
       </c>
@@ -15000,7 +15269,7 @@
       </c>
     </row>
     <row r="3" spans="2:11">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="24" t="s">
         <v>394</v>
       </c>
     </row>
@@ -15101,7 +15370,7 @@
       <c r="J14" s="22"/>
     </row>
     <row r="15" spans="2:11">
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="24" t="s">
         <v>395</v>
       </c>
     </row>
@@ -15129,13 +15398,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="37" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
         <v>448</v>
       </c>
@@ -15324,13 +15593,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="37" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
         <v>448</v>
       </c>
@@ -15519,13 +15788,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="37" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
         <v>448</v>
       </c>
@@ -15543,7 +15812,7 @@
       </c>
     </row>
     <row r="3" spans="2:11">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="24" t="s">
         <v>394</v>
       </c>
     </row>
@@ -15609,7 +15878,7 @@
       </c>
     </row>
     <row r="13" spans="2:11">
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="24" t="s">
         <v>395</v>
       </c>
     </row>
@@ -15694,7 +15963,7 @@
     </row>
     <row r="23" spans="3:11">
       <c r="D23" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K23" t="s">
         <v>452</v>
@@ -15702,7 +15971,7 @@
     </row>
     <row r="24" spans="3:11">
       <c r="E24" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="25" spans="3:11">
@@ -15812,105 +16081,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="23.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="26" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="45">
-      <c r="A3" s="33" t="s">
+    <row r="3" spans="1:4">
+      <c r="A3" s="27" t="s">
         <v>427</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="27" t="s">
         <v>428</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="27" t="s">
         <v>429</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="27" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="60">
-      <c r="A4" s="35" t="s">
+    <row r="4" spans="1:4" ht="30">
+      <c r="A4" s="29" t="s">
         <v>399</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="28" t="s">
         <v>431</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="28" t="s">
         <v>190</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="28" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="75">
-      <c r="A5" s="35" t="s">
+    <row r="5" spans="1:4" ht="30">
+      <c r="A5" s="29" t="s">
         <v>432</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="28" t="s">
         <v>434</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="28" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="75">
-      <c r="A6" s="35" t="s">
+    <row r="6" spans="1:4" ht="30">
+      <c r="A6" s="29" t="s">
         <v>435</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="28" t="s">
         <v>436</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="28" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="90">
-      <c r="A7" s="35" t="s">
+    <row r="7" spans="1:4" ht="45">
+      <c r="A7" s="29" t="s">
         <v>437</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="28" t="s">
         <v>438</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="28" t="s">
         <v>190</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="28" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="45">
-      <c r="A8" s="35" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8" s="29" t="s">
         <v>401</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="28" t="s">
         <v>439</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="28" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="60">
-      <c r="A9" s="35" t="s">
+    <row r="9" spans="1:4" ht="30">
+      <c r="A9" s="29" t="s">
         <v>440</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="28" t="s">
         <v>441</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="28" t="s">
         <v>190</v>
       </c>
     </row>
@@ -15925,15 +16194,15 @@
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="36"/>
+      <c r="A14" s="30"/>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="31" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="31" t="s">
         <v>445</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Support data type coersion in paste specify column names during table creation
</commit_message>
<xml_diff>
--- a/Development Docs/ToDo.xlsx
+++ b/Development Docs/ToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greg\Local Sites\schaub-labs\app\public\wp-content\plugins\dynamic-table-blocks\Development Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFE1948-4F3E-40F5-B009-EAAE78192012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EC5534-59DD-42D5-B5CC-C208970652BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A3DBE3D2-0DAF-4481-8DC4-68682F930EC6}"/>
   </bookViews>
@@ -16,15 +16,16 @@
     <sheet name="Prioritized List" sheetId="1" r:id="rId1"/>
     <sheet name="Features" sheetId="6" r:id="rId2"/>
     <sheet name="Data Types" sheetId="3" r:id="rId3"/>
-    <sheet name="date-time Data Shape" sheetId="5" r:id="rId4"/>
-    <sheet name="Number Data Shape" sheetId="4" r:id="rId5"/>
-    <sheet name="Checkbox Data Shape" sheetId="7" r:id="rId6"/>
-    <sheet name="Link Data Shape" sheetId="8" r:id="rId7"/>
-    <sheet name="Sheet3" sheetId="9" r:id="rId8"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId9"/>
+    <sheet name="Data Type Conversion" sheetId="10" r:id="rId4"/>
+    <sheet name="date-time Data Shape" sheetId="5" r:id="rId5"/>
+    <sheet name="Number Data Shape" sheetId="4" r:id="rId6"/>
+    <sheet name="Checkbox Data Shape" sheetId="7" r:id="rId7"/>
+    <sheet name="Link Data Shape" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet3" sheetId="9" r:id="rId9"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritized List'!$B$1:$L$167</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1825" uniqueCount="484">
   <si>
     <t>Item</t>
   </si>
@@ -1054,9 +1055,6 @@
   </si>
   <si>
     <t>Clone/Duplicate table from Maintenance Page</t>
-  </si>
-  <si>
-    <t>Coerce date and number formats from General format</t>
   </si>
   <si>
     <t>1.4.3</t>
@@ -1558,6 +1556,114 @@
   </si>
   <si>
     <t>HIgh</t>
+  </si>
+  <si>
+    <t>1.4.8</t>
+  </si>
+  <si>
+    <t>Fix bug that causes tables to be deleted when they should not be.</t>
+  </si>
+  <si>
+    <t>1.4.9</t>
+  </si>
+  <si>
+    <t>Done except for styling</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TO:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Data Type</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">FROM: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Type =&gt;</t>
+    </r>
+  </si>
+  <si>
+    <t>Cooerce</t>
+  </si>
+  <si>
+    <t>Conversion Method</t>
+  </si>
+  <si>
+    <t>- Cooerce: Attemp Conversion and deliver an compatibility error if data cannot be coerced</t>
+  </si>
+  <si>
+    <t>- Incompatible: Data Types cannot be coerced. Deliver a compatibility error when coercing</t>
+  </si>
+  <si>
+    <t>Incompatible</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">See </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Type Conversion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tab</t>
+    </r>
+  </si>
+  <si>
+    <t>Coerce content types for paste</t>
+  </si>
+  <si>
+    <t>Coerce content types for column content type updates</t>
+  </si>
+  <si>
+    <t>Make green cell border that shows the current cell go away when the block loses focus</t>
   </si>
 </sst>
 </file>
@@ -1602,7 +1708,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1627,8 +1733,29 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="lightGrid"/>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1677,11 +1804,215 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1782,6 +2113,71 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5386,7 +5782,7 @@
         <v>145</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C110" s="15" t="s">
         <v>190</v>
@@ -5404,7 +5800,7 @@
         <v>11</v>
       </c>
       <c r="H110" s="13" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J110" s="5"/>
       <c r="K110" s="4" t="s">
@@ -5416,7 +5812,7 @@
         <v>56</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C111" s="15" t="s">
         <v>190</v>
@@ -5431,7 +5827,7 @@
         <v>7</v>
       </c>
       <c r="H111" s="13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="J111" s="5"/>
       <c r="K111" s="4" t="s">
@@ -5458,7 +5854,7 @@
         <v>6</v>
       </c>
       <c r="H112" s="13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>26</v>
@@ -5469,7 +5865,7 @@
         <v>147</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C113" s="15" t="s">
         <v>189</v>
@@ -5487,7 +5883,7 @@
         <v>7</v>
       </c>
       <c r="H113" s="13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="K113" s="4" t="s">
         <v>26</v>
@@ -5516,7 +5912,7 @@
         <v>7</v>
       </c>
       <c r="H114" s="13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="K114" s="4" t="s">
         <v>26</v>
@@ -5527,7 +5923,7 @@
         <v>150</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C115" s="15" t="s">
         <v>190</v>
@@ -5542,10 +5938,10 @@
         <v>6</v>
       </c>
       <c r="G115" s="4" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="H115" s="13" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>26</v>
@@ -5556,7 +5952,7 @@
         <v>151</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C116" s="15" t="s">
         <v>190</v>
@@ -5574,56 +5970,57 @@
         <v>7</v>
       </c>
       <c r="H116" s="13" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K116" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="117" spans="1:12" ht="30">
+    <row r="117" spans="1:12">
       <c r="A117" s="4">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>462</v>
+        <v>392</v>
       </c>
       <c r="C117" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>86</v>
+        <v>254</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G117" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H117" s="13" t="s">
-        <v>467</v>
-      </c>
+        <v>466</v>
+      </c>
+      <c r="J117" s="5"/>
       <c r="K117" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="118" spans="1:12" ht="45">
+    <row r="118" spans="1:12" ht="30">
       <c r="A118" s="4">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="C118" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F118" s="4" t="s">
         <v>6</v>
@@ -5632,18 +6029,15 @@
         <v>11</v>
       </c>
       <c r="H118" s="13" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K118" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L118" s="4" t="s">
-        <v>468</v>
-      </c>
     </row>
     <row r="119" spans="1:12" ht="30">
       <c r="A119" s="4">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B119" s="4" t="s">
         <v>461</v>
@@ -5652,7 +6046,7 @@
         <v>189</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E119" s="4" t="s">
         <v>86</v>
@@ -5664,27 +6058,24 @@
         <v>11</v>
       </c>
       <c r="H119" s="13" t="s">
-        <v>467</v>
-      </c>
-      <c r="J119" s="4">
-        <v>3</v>
+        <v>466</v>
       </c>
       <c r="K119" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="120" spans="1:12">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" ht="45">
       <c r="A120" s="4">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E120" s="4" t="s">
         <v>55</v>
@@ -5696,21 +6087,21 @@
         <v>11</v>
       </c>
       <c r="H120" s="13" t="s">
+        <v>466</v>
+      </c>
+      <c r="K120" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L120" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="J120" s="4">
-        <v>4</v>
-      </c>
-      <c r="K120" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="121" spans="1:12">
+    </row>
+    <row r="121" spans="1:12" ht="30">
       <c r="A121" s="4">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>239</v>
+        <v>470</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>189</v>
@@ -5719,132 +6110,120 @@
         <v>39</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G121" s="4" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="H121" s="13" t="s">
-        <v>467</v>
-      </c>
-      <c r="J121" s="5">
-        <v>5</v>
+        <v>469</v>
       </c>
       <c r="K121" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="122" spans="1:12">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" ht="30">
       <c r="A122" s="4">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>393</v>
+        <v>483</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>39</v>
+        <v>307</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>254</v>
+        <v>86</v>
       </c>
       <c r="F122" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G122" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H122" s="13" t="s">
-        <v>467</v>
-      </c>
-      <c r="J122" s="5">
-        <v>6</v>
+        <v>469</v>
       </c>
       <c r="K122" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12" ht="45">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12">
       <c r="A123" s="4">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>253</v>
+        <v>217</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="F123" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G123" s="4" t="s">
-        <v>168</v>
+        <v>55</v>
       </c>
       <c r="H123" s="13" t="s">
-        <v>467</v>
-      </c>
-      <c r="J123" s="5">
-        <v>7</v>
+        <v>471</v>
+      </c>
+      <c r="J123" s="38">
+        <v>1</v>
       </c>
       <c r="K123" s="4" t="s">
-        <v>256</v>
+        <v>155</v>
       </c>
       <c r="L123" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="124" spans="1:12" ht="30">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12">
       <c r="A124" s="4">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>390</v>
+        <v>481</v>
       </c>
       <c r="C124" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G124" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H124" s="13" t="s">
-        <v>467</v>
-      </c>
-      <c r="J124" s="5">
-        <v>8</v>
+        <v>471</v>
+      </c>
+      <c r="J124" s="38">
+        <v>2</v>
       </c>
       <c r="K124" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="L124" s="4" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12" ht="30">
+        <v>155</v>
+      </c>
+      <c r="L124" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12">
       <c r="A125" s="4">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="C125" s="15" t="s">
         <v>189</v>
@@ -5853,7 +6232,7 @@
         <v>307</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>6</v>
@@ -5862,155 +6241,179 @@
         <v>11</v>
       </c>
       <c r="H125" s="13" t="s">
-        <v>467</v>
+        <v>471</v>
+      </c>
+      <c r="J125" s="38">
+        <v>3</v>
       </c>
       <c r="K125" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="126" spans="1:12">
+    <row r="126" spans="1:12" ht="30">
       <c r="A126" s="4">
-        <v>105</v>
+        <v>153</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>217</v>
+        <v>460</v>
       </c>
       <c r="C126" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G126" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H126" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J126" s="4">
-        <v>10</v>
+        <v>471</v>
+      </c>
+      <c r="J126" s="38">
+        <v>4</v>
       </c>
       <c r="K126" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
       </c>
     </row>
     <row r="127" spans="1:12">
       <c r="A127" s="4">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>332</v>
+        <v>239</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G127" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H127" s="13" t="s">
+        <v>471</v>
+      </c>
+      <c r="J127" s="38">
+        <v>5</v>
+      </c>
+      <c r="K127" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" ht="45">
+      <c r="A128" s="4">
         <v>132</v>
       </c>
-      <c r="J127" s="4">
-        <v>10</v>
-      </c>
-      <c r="K127" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="128" spans="1:12">
-      <c r="A128" s="4">
-        <v>77</v>
-      </c>
       <c r="B128" s="4" t="s">
-        <v>141</v>
+        <v>253</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>131</v>
+        <v>254</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G128" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="H128" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I128" s="5">
-        <v>80</v>
-      </c>
-      <c r="J128" s="5">
-        <v>20</v>
+        <v>471</v>
+      </c>
+      <c r="J128" s="39">
+        <v>6</v>
       </c>
       <c r="K128" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="129" spans="1:12">
+        <v>256</v>
+      </c>
+      <c r="L128" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" ht="30">
       <c r="A129" s="4">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>211</v>
+        <v>389</v>
       </c>
       <c r="C129" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="E129" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G129" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H129" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="J129" s="5">
-        <v>20</v>
+        <v>471</v>
+      </c>
+      <c r="J129" s="39">
+        <v>7</v>
       </c>
       <c r="K129" s="4" t="s">
-        <v>132</v>
+        <v>256</v>
+      </c>
+      <c r="L129" s="4" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="130" spans="1:12">
       <c r="A130" s="4">
-        <v>100</v>
+        <v>159</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>246</v>
+        <v>482</v>
       </c>
       <c r="C130" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F130" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G130" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H130" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I130" s="5">
+        <v>144</v>
+      </c>
       <c r="J130" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K130" s="4" t="s">
         <v>132</v>
@@ -6018,45 +6421,42 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" s="4">
-        <v>127</v>
+        <v>77</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>244</v>
+        <v>141</v>
       </c>
       <c r="C131" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G131" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H131" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J131" s="4">
+      <c r="I131" s="5">
+        <v>80</v>
+      </c>
+      <c r="J131" s="5">
         <v>20</v>
       </c>
       <c r="K131" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L131" s="4" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="132" spans="1:12">
       <c r="A132" s="4">
-        <v>143</v>
+        <v>86</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>331</v>
+        <v>211</v>
       </c>
       <c r="C132" s="15" t="s">
         <v>189</v>
@@ -6065,18 +6465,15 @@
         <v>17</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F132" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G132" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H132" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J132" s="4">
+      <c r="J132" s="5">
         <v>20</v>
       </c>
       <c r="K132" s="4" t="s">
@@ -6085,31 +6482,28 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" s="4">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>149</v>
+        <v>246</v>
       </c>
       <c r="C133" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G133" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H133" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J133" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K133" s="4" t="s">
         <v>132</v>
@@ -6117,60 +6511,66 @@
     </row>
     <row r="134" spans="1:12">
       <c r="A134" s="4">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>171</v>
+        <v>244</v>
       </c>
       <c r="C134" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E134" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="G134" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H134" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J134" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K134" s="4" t="s">
         <v>132</v>
       </c>
+      <c r="L134" s="4" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="135" spans="1:12">
       <c r="A135" s="4">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>223</v>
+        <v>331</v>
       </c>
       <c r="C135" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G135" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H135" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J135" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>132</v>
@@ -6178,22 +6578,25 @@
     </row>
     <row r="136" spans="1:12">
       <c r="A136" s="4">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>224</v>
+        <v>149</v>
       </c>
       <c r="C136" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D136" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="G136" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H136" s="13" t="s">
         <v>132</v>
@@ -6205,12 +6608,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="137" spans="1:12" ht="30">
+    <row r="137" spans="1:12">
       <c r="A137" s="4">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>226</v>
+        <v>171</v>
       </c>
       <c r="C137" s="15" t="s">
         <v>190</v>
@@ -6219,7 +6622,7 @@
         <v>17</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>7</v>
@@ -6236,21 +6639,24 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" s="4">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C138" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E138" s="4" t="s">
         <v>86</v>
       </c>
       <c r="F138" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G138" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H138" s="13" t="s">
@@ -6265,10 +6671,10 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" s="4">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>142</v>
+        <v>224</v>
       </c>
       <c r="C139" s="15" t="s">
         <v>190</v>
@@ -6277,30 +6683,27 @@
         <v>17</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H139" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I139" s="5">
-        <v>139</v>
-      </c>
-      <c r="J139" s="5">
-        <v>40</v>
+      <c r="J139" s="4">
+        <v>30</v>
       </c>
       <c r="K139" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="140" spans="1:12">
+    <row r="140" spans="1:12" ht="30">
       <c r="A140" s="4">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C140" s="15" t="s">
         <v>190</v>
@@ -6309,7 +6712,7 @@
         <v>17</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="F140" s="4" t="s">
         <v>7</v>
@@ -6317,11 +6720,8 @@
       <c r="H140" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I140" s="5" t="s">
-        <v>232</v>
-      </c>
       <c r="J140" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K140" s="4" t="s">
         <v>132</v>
@@ -6329,13 +6729,13 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" s="4">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="C141" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>17</v>
@@ -6346,14 +6746,11 @@
       <c r="F141" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G141" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="H141" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J141" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K141" s="4" t="s">
         <v>132</v>
@@ -6361,45 +6758,45 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" s="4">
-        <v>123</v>
+        <v>79</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>237</v>
+        <v>142</v>
       </c>
       <c r="C142" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D142" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G142" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H142" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J142" s="4">
+      <c r="I142" s="5">
+        <v>139</v>
+      </c>
+      <c r="J142" s="5">
         <v>40</v>
       </c>
       <c r="K142" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="143" spans="1:12" ht="30">
+    <row r="143" spans="1:12">
       <c r="A143" s="4">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="C143" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D143" s="4" t="s">
         <v>17</v>
@@ -6408,45 +6805,48 @@
         <v>55</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G143" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H143" s="13" t="s">
         <v>132</v>
       </c>
+      <c r="I143" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="J143" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K143" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="144" spans="1:12" ht="30">
+    <row r="144" spans="1:12">
       <c r="A144" s="4">
-        <v>72</v>
+        <v>122</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>130</v>
+        <v>236</v>
       </c>
       <c r="C144" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D144" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
+      </c>
+      <c r="G144" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H144" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J144" s="5">
-        <v>50</v>
+      <c r="J144" s="4">
+        <v>40</v>
       </c>
       <c r="K144" s="4" t="s">
         <v>132</v>
@@ -6454,42 +6854,45 @@
     </row>
     <row r="145" spans="1:12">
       <c r="A145" s="4">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>143</v>
+        <v>237</v>
       </c>
       <c r="C145" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D145" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
+      </c>
+      <c r="G145" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H145" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J145" s="5">
-        <v>50</v>
+      <c r="J145" s="4">
+        <v>40</v>
       </c>
       <c r="K145" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="146" spans="1:12">
+    <row r="146" spans="1:12" ht="30">
       <c r="A146" s="4">
-        <v>103</v>
+        <v>26</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>215</v>
+        <v>241</v>
       </c>
       <c r="C146" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D146" s="4" t="s">
         <v>17</v>
@@ -6498,7 +6901,10 @@
         <v>55</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
+      </c>
+      <c r="G146" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H146" s="13" t="s">
         <v>132</v>
@@ -6510,12 +6916,12 @@
         <v>132</v>
       </c>
     </row>
-    <row r="147" spans="1:12">
+    <row r="147" spans="1:12" ht="30">
       <c r="A147" s="4">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="C147" s="15" t="s">
         <v>190</v>
@@ -6524,7 +6930,7 @@
         <v>17</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F147" s="4" t="s">
         <v>25</v>
@@ -6532,7 +6938,7 @@
       <c r="H147" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J147" s="4">
+      <c r="J147" s="5">
         <v>50</v>
       </c>
       <c r="K147" s="4" t="s">
@@ -6541,27 +6947,27 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="4">
-        <v>121</v>
+        <v>80</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>234</v>
+        <v>143</v>
       </c>
       <c r="C148" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>55</v>
+        <v>131</v>
       </c>
       <c r="F148" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H148" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J148" s="4">
+      <c r="J148" s="5">
         <v>50</v>
       </c>
       <c r="K148" s="4" t="s">
@@ -6570,24 +6976,21 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="4">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>247</v>
+        <v>215</v>
       </c>
       <c r="C149" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D149" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E149" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F149" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G149" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H149" s="13" t="s">
@@ -6599,16 +7002,13 @@
       <c r="K149" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L149" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="150" spans="1:12" ht="30">
+    </row>
+    <row r="150" spans="1:12">
       <c r="A150" s="4">
-        <v>143</v>
+        <v>108</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>322</v>
+        <v>220</v>
       </c>
       <c r="C150" s="15" t="s">
         <v>190</v>
@@ -6620,14 +7020,11 @@
         <v>55</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H150" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="I150" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="J150" s="4">
         <v>50</v>
       </c>
@@ -6637,28 +7034,28 @@
     </row>
     <row r="151" spans="1:12">
       <c r="A151" s="4">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="C151" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E151" s="4" t="s">
         <v>55</v>
       </c>
       <c r="F151" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H151" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J151" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K151" s="4" t="s">
         <v>132</v>
@@ -6666,57 +7063,66 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" s="4">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>133</v>
+        <v>247</v>
       </c>
       <c r="C152" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F152" s="4" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G152" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H152" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J152" s="5">
-        <v>80</v>
+      <c r="J152" s="4">
+        <v>50</v>
       </c>
       <c r="K152" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="153" spans="1:12">
+      <c r="L152" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12" ht="30">
       <c r="A153" s="4">
-        <v>84</v>
+        <v>143</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>150</v>
+        <v>322</v>
       </c>
       <c r="C153" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="F153" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H153" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J153" s="5">
-        <v>80</v>
+      <c r="I153" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="J153" s="4">
+        <v>50</v>
       </c>
       <c r="K153" s="4" t="s">
         <v>132</v>
@@ -6724,25 +7130,28 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" s="4">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C154" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D154" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>146</v>
+        <v>55</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H154" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J154" s="4">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K154" s="4" t="s">
         <v>132</v>
@@ -6750,98 +7159,83 @@
     </row>
     <row r="155" spans="1:12">
       <c r="A155" s="4">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>29</v>
+        <v>133</v>
       </c>
       <c r="C155" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D155" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E155" s="4" t="s">
-        <v>30</v>
+        <v>131</v>
       </c>
       <c r="F155" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G155" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H155" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J155" s="4">
-        <v>99</v>
+      <c r="J155" s="5">
+        <v>80</v>
       </c>
       <c r="K155" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="156" spans="1:12" ht="30">
+    <row r="156" spans="1:12">
       <c r="A156" s="4">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>28</v>
+        <v>150</v>
       </c>
       <c r="C156" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D156" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E156" s="4" t="s">
-        <v>21</v>
+        <v>131</v>
       </c>
       <c r="F156" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G156" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H156" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J156" s="4">
-        <v>99</v>
+      <c r="J156" s="5">
+        <v>80</v>
       </c>
       <c r="K156" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L156" s="4" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="157" spans="1:12">
       <c r="A157" s="4">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>40</v>
+        <v>219</v>
       </c>
       <c r="C157" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D157" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E157" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F157" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G157" s="4" t="s">
-        <v>7</v>
+        <v>146</v>
       </c>
       <c r="H157" s="13" t="s">
         <v>132</v>
       </c>
       <c r="J157" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="K157" s="4" t="s">
         <v>132</v>
@@ -6849,10 +7243,10 @@
     </row>
     <row r="158" spans="1:12">
       <c r="A158" s="4">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="C158" s="15" t="s">
         <v>189</v>
@@ -6861,10 +7255,10 @@
         <v>18</v>
       </c>
       <c r="E158" s="4" t="s">
-        <v>251</v>
+        <v>30</v>
       </c>
       <c r="F158" s="4" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G158" s="4" t="s">
         <v>24</v>
@@ -6881,19 +7275,19 @@
     </row>
     <row r="159" spans="1:12" ht="30">
       <c r="A159" s="4">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>125</v>
+        <v>28</v>
       </c>
       <c r="C159" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D159" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E159" s="4" t="s">
-        <v>86</v>
+        <v>21</v>
       </c>
       <c r="F159" s="4" t="s">
         <v>6</v>
@@ -6910,28 +7304,31 @@
       <c r="K159" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="160" spans="1:12" ht="30">
+      <c r="L159" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12">
       <c r="A160" s="4">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>128</v>
+        <v>40</v>
       </c>
       <c r="C160" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D160" s="4" t="s">
-        <v>307</v>
+        <v>18</v>
       </c>
       <c r="E160" s="4" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="F160" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G160" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H160" s="13" t="s">
         <v>132</v>
@@ -6945,25 +7342,25 @@
     </row>
     <row r="161" spans="1:12">
       <c r="A161" s="4">
-        <v>88</v>
+        <v>55</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>154</v>
+        <v>79</v>
       </c>
       <c r="C161" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D161" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E161" s="4" t="s">
-        <v>131</v>
+        <v>251</v>
       </c>
       <c r="F161" s="4" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G161" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H161" s="13" t="s">
         <v>132</v>
@@ -6977,10 +7374,10 @@
     </row>
     <row r="162" spans="1:12" ht="30">
       <c r="A162" s="4">
-        <v>139</v>
+        <v>70</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>311</v>
+        <v>125</v>
       </c>
       <c r="C162" s="15" t="s">
         <v>189</v>
@@ -6989,10 +7386,10 @@
         <v>307</v>
       </c>
       <c r="E162" s="4" t="s">
-        <v>310</v>
+        <v>86</v>
       </c>
       <c r="F162" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G162" s="4" t="s">
         <v>24</v>
@@ -7006,31 +7403,28 @@
       <c r="K162" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L162" s="4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="163" spans="1:12" ht="45">
+    </row>
+    <row r="163" spans="1:12" ht="30">
       <c r="A163" s="4">
-        <v>142</v>
+        <v>71</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>319</v>
+        <v>128</v>
       </c>
       <c r="C163" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="E163" s="4" t="s">
-        <v>320</v>
+        <v>86</v>
       </c>
       <c r="F163" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G163" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H163" s="13" t="s">
         <v>132</v>
@@ -7041,28 +7435,25 @@
       <c r="K163" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="L163" s="4" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="164" spans="1:12" ht="45">
+    </row>
+    <row r="164" spans="1:12">
       <c r="A164" s="4">
-        <v>155</v>
+        <v>88</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>463</v>
+        <v>154</v>
       </c>
       <c r="C164" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D164" s="4" t="s">
-        <v>307</v>
+        <v>17</v>
       </c>
       <c r="E164" s="4" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="F164" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G164" s="4" t="s">
         <v>11</v>
@@ -7079,25 +7470,25 @@
     </row>
     <row r="165" spans="1:12" ht="30">
       <c r="A165" s="4">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>465</v>
+        <v>311</v>
       </c>
       <c r="C165" s="15" t="s">
         <v>189</v>
       </c>
       <c r="D165" s="4" t="s">
-        <v>17</v>
+        <v>307</v>
       </c>
       <c r="E165" s="4" t="s">
-        <v>55</v>
+        <v>310</v>
       </c>
       <c r="F165" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G165" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H165" s="13" t="s">
         <v>132</v>
@@ -7108,15 +7499,108 @@
       <c r="K165" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="166" spans="1:12">
-      <c r="H166" s="13"/>
-    </row>
-    <row r="167" spans="1:12">
-      <c r="H167" s="13"/>
-    </row>
-    <row r="168" spans="1:12">
-      <c r="H168" s="13"/>
+      <c r="L165" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12" ht="45">
+      <c r="A166" s="4">
+        <v>142</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C166" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G166" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H166" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J166" s="4">
+        <v>99</v>
+      </c>
+      <c r="K166" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L166" s="4" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="167" spans="1:12" ht="45">
+      <c r="A167" s="4">
+        <v>155</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="C167" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G167" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H167" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J167" s="4">
+        <v>99</v>
+      </c>
+      <c r="K167" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" ht="30">
+      <c r="A168" s="4">
+        <v>157</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="C168" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D168" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E168" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G168" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H168" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J168" s="4">
+        <v>99</v>
+      </c>
+      <c r="K168" s="4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="169" spans="1:12">
       <c r="H169" s="13"/>
@@ -7163,7 +7647,7 @@
     <row r="183" spans="1:8">
       <c r="A183" s="9">
         <f>MAX(A1:A182)</f>
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B183" s="9" t="s">
         <v>95</v>
@@ -9857,18 +10341,179 @@
       <c r="H1078" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:L165" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
+  <autoFilter ref="B1:L167" xr:uid="{C9A95F50-2338-43A7-B2D8-210D78A54828}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L77">
       <sortCondition ref="J1:J77"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L165">
-    <sortCondition ref="H2:H165"/>
-    <sortCondition ref="J2:J165"/>
-    <sortCondition ref="A2:A165"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L168">
+    <sortCondition ref="H2:H168"/>
+    <sortCondition ref="J2:J168"/>
+    <sortCondition ref="A2:A168"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
+  <dimension ref="B9:T43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="9" spans="2:20">
+      <c r="B9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20">
+      <c r="T16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7">
+      <c r="B19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" t="s">
+        <v>98</v>
+      </c>
+      <c r="D19" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" t="s">
+        <v>100</v>
+      </c>
+      <c r="G19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7">
+      <c r="G20" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7">
+      <c r="G21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7">
+      <c r="B24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" t="s">
+        <v>100</v>
+      </c>
+      <c r="G24" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7">
+      <c r="G25" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7">
+      <c r="B29" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" t="s">
+        <v>98</v>
+      </c>
+      <c r="D29" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" t="s">
+        <v>100</v>
+      </c>
+      <c r="G29" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7">
+      <c r="G30" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="5:7">
+      <c r="E33" t="s">
+        <v>104</v>
+      </c>
+      <c r="G33" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34" spans="5:7">
+      <c r="G34" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="5:7">
+      <c r="E36" t="s">
+        <v>107</v>
+      </c>
+      <c r="G36" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="5:7">
+      <c r="G37" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="38" spans="5:7">
+      <c r="G38" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="39" spans="5:7">
+      <c r="G39" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="5:7" ht="15.75">
+      <c r="G40" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="5:7">
+      <c r="G41" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="5:7">
+      <c r="G42" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="43" spans="5:7">
+      <c r="G43" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -9895,236 +10540,236 @@
         <v>16</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" spans="2:6">
       <c r="C5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="C6" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D6" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="C7" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8" spans="2:6">
       <c r="C8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" spans="2:6">
       <c r="C9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D9" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F9" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="10" spans="2:6">
       <c r="C10" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D10" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="C11" t="s">
+        <v>376</v>
+      </c>
+      <c r="F11" t="s">
         <v>377</v>
-      </c>
-      <c r="F11" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="12" spans="2:6">
       <c r="C12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="13" spans="2:6">
       <c r="C13" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="15" spans="2:6">
       <c r="B15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" spans="2:6">
       <c r="C16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" spans="2:6">
       <c r="C17" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D17" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="18" spans="2:6">
       <c r="C18" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D18" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="19" spans="2:6">
       <c r="C19" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D19" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20" spans="2:6">
       <c r="C20" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D20" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="C21" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D21" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="22" spans="2:6">
       <c r="C22" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D22" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="23" spans="2:6">
       <c r="C23" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D23" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F23" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="24" spans="2:6">
       <c r="C24" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D24" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F24" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="25" spans="2:6">
       <c r="C25" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D25" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="26" spans="2:6">
       <c r="C26" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D26" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="27" spans="2:6">
       <c r="C27" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D27" t="s">
         <v>132</v>
       </c>
       <c r="F27" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="30" spans="2:6">
       <c r="C30" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D30" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="31" spans="2:6">
       <c r="C31" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D31" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="32" spans="2:6">
       <c r="C32" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D32" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="33" spans="2:6">
       <c r="C33" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="36" spans="2:6">
       <c r="B36" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="37" spans="2:6">
@@ -10132,10 +10777,10 @@
         <v>172</v>
       </c>
       <c r="D37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="38" spans="2:6">
@@ -10143,10 +10788,10 @@
         <v>174</v>
       </c>
       <c r="D38" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F38" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="39" spans="2:6">
@@ -10154,10 +10799,10 @@
         <v>203</v>
       </c>
       <c r="D39" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F39" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="40" spans="2:6">
@@ -10165,10 +10810,10 @@
         <v>206</v>
       </c>
       <c r="D40" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F40" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="41" spans="2:6">
@@ -10197,7 +10842,7 @@
     </row>
     <row r="44" spans="2:6">
       <c r="C44" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D44" t="s">
         <v>132</v>
@@ -10205,39 +10850,39 @@
     </row>
     <row r="46" spans="2:6">
       <c r="B46" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="47" spans="2:6">
       <c r="C47" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D47" t="s">
         <v>132</v>
       </c>
       <c r="F47" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="50" spans="2:4">
       <c r="B50" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="51" spans="2:4">
       <c r="C51" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D51" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="52" spans="2:4">
       <c r="C52" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D52" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -10610,10 +11255,10 @@
         <v>258</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>185</v>
@@ -10622,10 +11267,10 @@
         <v>206</v>
       </c>
       <c r="H7" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>381</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>382</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>190</v>
@@ -10634,10 +11279,10 @@
         <v>189</v>
       </c>
       <c r="L7" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="M7" s="4" t="s">
         <v>383</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>384</v>
       </c>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
@@ -10681,7 +11326,7 @@
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="13" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="14"/>
@@ -10690,7 +11335,7 @@
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>189</v>
@@ -10699,7 +11344,7 @@
         <v>189</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
@@ -11190,7 +11835,7 @@
     </row>
     <row r="18" spans="1:45">
       <c r="A18" s="25" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="15"/>
@@ -11201,7 +11846,7 @@
         <v>172</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="I18" s="4"/>
       <c r="K18" s="4"/>
@@ -11249,10 +11894,10 @@
       <c r="F19" s="14"/>
       <c r="G19" s="4"/>
       <c r="H19" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="I19" t="s">
         <v>409</v>
-      </c>
-      <c r="I19" t="s">
-        <v>410</v>
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
@@ -11299,7 +11944,7 @@
       <c r="F20" s="14"/>
       <c r="G20" s="4"/>
       <c r="H20" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
@@ -11348,7 +11993,7 @@
       <c r="F21" s="14"/>
       <c r="G21" s="4"/>
       <c r="H21" s="11" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
@@ -11446,7 +12091,7 @@
         <v>202</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
@@ -11493,10 +12138,10 @@
       <c r="F24" s="14"/>
       <c r="G24" s="4"/>
       <c r="H24" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I24" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
@@ -11543,7 +12188,7 @@
       <c r="F25" s="14"/>
       <c r="G25" s="4"/>
       <c r="H25" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
@@ -11592,7 +12237,7 @@
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="11" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -11687,10 +12332,10 @@
       <c r="E28" s="15"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
@@ -11739,10 +12384,10 @@
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I29" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
@@ -11789,10 +12434,10 @@
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I30" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
@@ -11840,7 +12485,7 @@
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="11" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
@@ -11938,7 +12583,7 @@
         <v>204</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
@@ -11987,10 +12632,10 @@
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I34" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
@@ -12037,10 +12682,10 @@
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I35" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
@@ -12088,7 +12733,7 @@
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="11" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
@@ -15236,6 +15881,170 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E50596-9C0B-4729-BABF-DA694A59DEC6}">
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="7" width="15.5703125" customWidth="1"/>
+    <col min="9" max="9" width="65.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="57" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="58" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="58" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" thickBot="1"/>
+    <row r="6" spans="1:6" ht="15.75" thickBot="1">
+      <c r="A6" s="45" t="s">
+        <v>474</v>
+      </c>
+      <c r="B6" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>174</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="F6" s="41" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" thickBot="1">
+      <c r="A7" s="46" t="s">
+        <v>473</v>
+      </c>
+      <c r="B7" s="42"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="44"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="47" t="s">
+        <v>172</v>
+      </c>
+      <c r="B8" s="49"/>
+      <c r="C8" s="60" t="s">
+        <v>475</v>
+      </c>
+      <c r="D8" s="60" t="s">
+        <v>475</v>
+      </c>
+      <c r="E8" s="60" t="s">
+        <v>475</v>
+      </c>
+      <c r="F8" s="50" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="B9" s="61" t="s">
+        <v>256</v>
+      </c>
+      <c r="C9" s="51"/>
+      <c r="D9" s="52" t="s">
+        <v>479</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>479</v>
+      </c>
+      <c r="F9" s="53" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="62" t="s">
+        <v>256</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>479</v>
+      </c>
+      <c r="D10" s="51"/>
+      <c r="E10" s="52" t="s">
+        <v>479</v>
+      </c>
+      <c r="F10" s="53" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="47" t="s">
+        <v>206</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>475</v>
+      </c>
+      <c r="C11" s="52" t="s">
+        <v>479</v>
+      </c>
+      <c r="D11" s="52" t="s">
+        <v>479</v>
+      </c>
+      <c r="E11" s="51"/>
+      <c r="F11" s="53" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" thickBot="1">
+      <c r="A12" s="48" t="s">
+        <v>202</v>
+      </c>
+      <c r="B12" s="54" t="s">
+        <v>479</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>479</v>
+      </c>
+      <c r="D12" s="55" t="s">
+        <v>479</v>
+      </c>
+      <c r="E12" s="55" t="s">
+        <v>479</v>
+      </c>
+      <c r="F12" s="56"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="57"/>
+    </row>
+    <row r="24" spans="9:9">
+      <c r="I24" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C07A045-EDB0-4506-A2E7-225FA060F54C}">
   <dimension ref="B2:K15"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15259,7 +16068,7 @@
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H2" s="21" t="s">
         <v>279</v>
@@ -15271,12 +16080,12 @@
         <v>289</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" spans="2:11">
       <c r="B3" s="24" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="2:11">
@@ -15377,7 +16186,7 @@
     </row>
     <row r="15" spans="2:11">
       <c r="B15" s="24" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -15388,7 +16197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F4CAB31-52FD-431F-AA77-05BD26AC0272}">
   <dimension ref="B2:K16"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15412,7 +16221,7 @@
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H2" s="21" t="s">
         <v>279</v>
@@ -15424,7 +16233,7 @@
         <v>289</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" spans="2:11">
@@ -15580,7 +16389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEDE6FBF-4912-4434-846B-E4148C1A58A6}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -15607,7 +16416,7 @@
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H2" s="21" t="s">
         <v>279</v>
@@ -15619,7 +16428,7 @@
         <v>289</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" spans="2:11">
@@ -15775,7 +16584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EB2FAD8-07BE-4066-8361-86590C51D015}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -15802,7 +16611,7 @@
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
       <c r="G2" s="21" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H2" s="21" t="s">
         <v>279</v>
@@ -15814,12 +16623,12 @@
         <v>289</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" spans="2:11">
       <c r="B3" s="24" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="2:11">
@@ -15838,10 +16647,10 @@
         <v>266</v>
       </c>
       <c r="I5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="2:11">
@@ -15857,10 +16666,10 @@
         <v>277</v>
       </c>
       <c r="I7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="J7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="2:11">
@@ -15885,47 +16694,47 @@
     </row>
     <row r="13" spans="2:11">
       <c r="B13" s="24" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="14" spans="2:11">
       <c r="B14" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="15" spans="2:11">
       <c r="C15" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" spans="2:11">
       <c r="D16" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G16" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J16" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="17" spans="3:11">
       <c r="D17" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="G17" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="J17" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="18" spans="3:11">
       <c r="D18" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G18" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H18" s="22"/>
       <c r="I18" s="22" t="s">
@@ -15935,31 +16744,31 @@
         <v>291</v>
       </c>
       <c r="K18" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="19" spans="3:11">
       <c r="D19" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="K19" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="20" spans="3:11">
       <c r="E20" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K20" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="21" spans="3:11">
       <c r="E21" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="K21" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="22" spans="3:11">
@@ -15969,31 +16778,31 @@
     </row>
     <row r="23" spans="3:11">
       <c r="D23" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="K23" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="24" spans="3:11">
       <c r="E24" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="25" spans="3:11">
       <c r="F25" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="K25" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="26" spans="3:11">
       <c r="F26" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="K26" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="27" spans="3:11">
@@ -16003,7 +16812,7 @@
     </row>
     <row r="28" spans="3:11">
       <c r="D28" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="29" spans="3:11">
@@ -16013,7 +16822,7 @@
     </row>
     <row r="30" spans="3:11">
       <c r="C30" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="K30" t="s">
         <v>178</v>
@@ -16021,17 +16830,17 @@
     </row>
     <row r="31" spans="3:11">
       <c r="D31" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="32" spans="3:11">
       <c r="C32" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="33" spans="2:11">
       <c r="C33" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="K33" t="s">
         <v>178</v>
@@ -16044,7 +16853,7 @@
     </row>
     <row r="35" spans="2:11">
       <c r="C35" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="K35" t="s">
         <v>178</v>
@@ -16057,10 +16866,10 @@
     </row>
     <row r="37" spans="2:11">
       <c r="C37" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I37" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="38" spans="2:11">
@@ -16076,7 +16885,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9AB0EEF-943E-4A80-BEA9-7E9C713A7508}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16088,29 +16897,29 @@
   <sheetData>
     <row r="1" spans="1:4" ht="23.25">
       <c r="A1" s="26" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="27" t="s">
+        <v>426</v>
+      </c>
+      <c r="B3" s="27" t="s">
         <v>427</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="C3" s="27" t="s">
         <v>428</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="D3" s="27" t="s">
         <v>429</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30">
       <c r="A4" s="29" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C4" s="28" t="s">
         <v>190</v>
@@ -16121,13 +16930,13 @@
     </row>
     <row r="5" spans="1:4" ht="30">
       <c r="A5" s="29" t="s">
+        <v>431</v>
+      </c>
+      <c r="B5" s="28" t="s">
         <v>432</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="C5" s="28" t="s">
         <v>433</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>434</v>
       </c>
       <c r="D5" s="28" t="s">
         <v>190</v>
@@ -16135,10 +16944,10 @@
     </row>
     <row r="6" spans="1:4" ht="30">
       <c r="A6" s="29" t="s">
+        <v>434</v>
+      </c>
+      <c r="B6" s="28" t="s">
         <v>435</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>436</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>189</v>
@@ -16149,10 +16958,10 @@
     </row>
     <row r="7" spans="1:4" ht="45">
       <c r="A7" s="29" t="s">
+        <v>436</v>
+      </c>
+      <c r="B7" s="28" t="s">
         <v>437</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>438</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>190</v>
@@ -16163,10 +16972,10 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C8" s="28" t="s">
         <v>189</v>
@@ -16177,10 +16986,10 @@
     </row>
     <row r="9" spans="1:4" ht="30">
       <c r="A9" s="29" t="s">
+        <v>439</v>
+      </c>
+      <c r="B9" s="28" t="s">
         <v>440</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>441</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>189</v>
@@ -16191,12 +17000,12 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -16204,173 +17013,12 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="31" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="31" t="s">
-        <v>445</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D206C0-E6E2-47CC-9389-62C309532CCD}">
-  <dimension ref="B9:T43"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="9" spans="2:20">
-      <c r="B9" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" t="s">
-        <v>98</v>
-      </c>
-      <c r="D9" t="s">
-        <v>97</v>
-      </c>
-      <c r="E9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="2:20">
-      <c r="T16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7">
-      <c r="B19" t="s">
-        <v>97</v>
-      </c>
-      <c r="C19" t="s">
-        <v>98</v>
-      </c>
-      <c r="D19" t="s">
-        <v>99</v>
-      </c>
-      <c r="E19" t="s">
-        <v>100</v>
-      </c>
-      <c r="G19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7">
-      <c r="G20" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7">
-      <c r="G21" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7">
-      <c r="B24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" t="s">
-        <v>98</v>
-      </c>
-      <c r="D24" t="s">
-        <v>117</v>
-      </c>
-      <c r="E24" t="s">
-        <v>100</v>
-      </c>
-      <c r="G24" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7">
-      <c r="G25" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7">
-      <c r="B29" t="s">
-        <v>97</v>
-      </c>
-      <c r="C29" t="s">
-        <v>98</v>
-      </c>
-      <c r="D29" t="s">
-        <v>102</v>
-      </c>
-      <c r="E29" t="s">
-        <v>100</v>
-      </c>
-      <c r="G29" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7">
-      <c r="G30" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="33" spans="5:7">
-      <c r="E33" t="s">
-        <v>104</v>
-      </c>
-      <c r="G33" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="34" spans="5:7">
-      <c r="G34" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="36" spans="5:7">
-      <c r="E36" t="s">
-        <v>107</v>
-      </c>
-      <c r="G36" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="37" spans="5:7">
-      <c r="G37" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="38" spans="5:7">
-      <c r="G38" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="39" spans="5:7">
-      <c r="G39" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="40" spans="5:7" ht="15.75">
-      <c r="G40" s="10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="41" spans="5:7">
-      <c r="G41" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="42" spans="5:7">
-      <c r="G42" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="43" spans="5:7">
-      <c r="G43" t="s">
-        <v>113</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>